<commit_message>
Updated from U43.4 to U45.3
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
+++ b/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\SourceFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE84C66A-2DE0-4088-AA5C-52B6006F12F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67688B74-9242-4EC4-AADD-44FCA595B3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13995" yWindow="30" windowWidth="14895" windowHeight="11550" tabRatio="869" firstSheet="6" activeTab="11" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="-21525" yWindow="2025" windowWidth="21600" windowHeight="11295" tabRatio="869" firstSheet="6" activeTab="10" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="378">
   <si>
     <t>TIER</t>
   </si>
@@ -1161,6 +1161,24 @@
   </si>
   <si>
     <t>Tales of the Ikorbân Valley</t>
+  </si>
+  <si>
+    <t>Renewer of Hamât</t>
+  </si>
+  <si>
+    <t>Dangers in Shagâna</t>
+  </si>
+  <si>
+    <t>Ekhamâti-bane of Shagâna (Advanced)</t>
+  </si>
+  <si>
+    <t>Ekhamâti-bane of Shagâna</t>
+  </si>
+  <si>
+    <t>Tales of the Crown of Hamât</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Shagâna</t>
   </si>
 </sst>
 </file>
@@ -1204,10 +1222,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2490,7 +2507,7 @@
       <c r="A20">
         <v>1879491622</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>322</v>
       </c>
       <c r="C20">
@@ -4597,7 +4614,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80148505-5553-4AE9-BBB8-D9A478F757ED}">
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -4703,35 +4720,35 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <f t="shared" ref="G3:G66" si="0">IF(AND(A3&gt;0,C3&gt;0),CONCATENATE("[",A3,"] = ",C3,", // ",B3),"")</f>
+        <f t="shared" ref="G3:G33" si="0">IF(AND(A3&gt;0,C3&gt;0),CONCATENATE("[",A3,"] = ",C3,", // ",B3),"")</f>
         <v>[1879491626] = 1, // Exploring Imhûlar</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H66" si="1">CONCATENATE(J3,K3,L3,N3," -- ",B3)</f>
+        <f t="shared" ref="H3:H33" si="1">CONCATENATE(J3,K3,L3,N3," -- ",B3)</f>
         <v xml:space="preserve"> [2] = {["ID"] = 1879491626; }; -- Exploring Imhûlar</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I66" si="2">ROW()-1</f>
+        <f t="shared" ref="I3:I33" si="2">ROW()-1</f>
         <v>2</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J3:J66" si="3">CONCATENATE(REPT(" ",2-LEN(I3)),"[",I3,"] = {")</f>
+        <f t="shared" ref="J3:J33" si="3">CONCATENATE(REPT(" ",2-LEN(I3)),"[",I3,"] = {")</f>
         <v xml:space="preserve"> [2] = {</v>
       </c>
       <c r="K3" t="str">
-        <f t="shared" ref="K3:K66" si="4">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
+        <f t="shared" ref="K3:K33" si="4">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879491626; </v>
       </c>
       <c r="L3" t="str">
-        <f t="shared" ref="L3:L66" si="5">IF(LEN(D3)&gt;0,CONCATENATE("[""CAT_ID""] = ",D3,"; "),"")</f>
+        <f t="shared" ref="L3:L33" si="5">IF(LEN(D3)&gt;0,CONCATENATE("[""CAT_ID""] = ",D3,"; "),"")</f>
         <v/>
       </c>
       <c r="M3" t="str">
-        <f t="shared" ref="M3:M66" si="6">CONCATENATE("[""TIER""] = ",TEXT(C3,"0"),"; ")</f>
+        <f t="shared" ref="M3:M33" si="6">CONCATENATE("[""TIER""] = ",TEXT(C3,"0"),"; ")</f>
         <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N3" t="str">
-        <f t="shared" ref="N3:N66" si="7">CONCATENATE("};")</f>
+        <f t="shared" ref="N3:N33" si="7">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
@@ -5427,7 +5444,7 @@
       <c r="A20">
         <v>1879491641</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>341</v>
       </c>
       <c r="C20">
@@ -5596,6 +5613,12 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>1879503580</v>
+      </c>
+      <c r="B24" t="s">
+        <v>372</v>
+      </c>
       <c r="C24" s="1"/>
       <c r="G24" t="str">
         <f t="shared" si="0"/>
@@ -5603,7 +5626,7 @@
       </c>
       <c r="H24" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[23] = {}; -- </v>
+        <v>[23] = {["ID"] = 1879503580; }; -- Renewer of Hamât</v>
       </c>
       <c r="I24">
         <f t="shared" si="2"/>
@@ -5615,7 +5638,7 @@
       </c>
       <c r="K24" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503580; </v>
       </c>
       <c r="L24" t="str">
         <f t="shared" si="5"/>
@@ -5631,14 +5654,22 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C25" s="1"/>
+      <c r="A25">
+        <v>1879503578</v>
+      </c>
+      <c r="B25" t="s">
+        <v>373</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1</v>
+      </c>
       <c r="G25" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>[1879503578] = 1, // Dangers in Shagâna</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[24] = {}; -- </v>
+        <v>[24] = {["ID"] = 1879503578; }; -- Dangers in Shagâna</v>
       </c>
       <c r="I25">
         <f t="shared" si="2"/>
@@ -5650,7 +5681,7 @@
       </c>
       <c r="K25" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503578; </v>
       </c>
       <c r="L25" t="str">
         <f t="shared" si="5"/>
@@ -5658,7 +5689,7 @@
       </c>
       <c r="M25" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N25" t="str">
         <f t="shared" si="7"/>
@@ -5666,14 +5697,22 @@
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C26" s="1"/>
+      <c r="A26">
+        <v>1879503579</v>
+      </c>
+      <c r="B26" t="s">
+        <v>374</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
       <c r="G26" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>[1879503579] = 1, // Ekhamâti-bane of Shagâna (Advanced)</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[25] = {}; -- </v>
+        <v>[25] = {["ID"] = 1879503579; }; -- Ekhamâti-bane of Shagâna (Advanced)</v>
       </c>
       <c r="I26">
         <f t="shared" si="2"/>
@@ -5685,7 +5724,7 @@
       </c>
       <c r="K26" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503579; </v>
       </c>
       <c r="L26" t="str">
         <f t="shared" si="5"/>
@@ -5693,7 +5732,7 @@
       </c>
       <c r="M26" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N26" t="str">
         <f t="shared" si="7"/>
@@ -5701,14 +5740,22 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C27" s="1"/>
+      <c r="A27">
+        <v>1879503581</v>
+      </c>
+      <c r="B27" t="s">
+        <v>375</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
       <c r="G27" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>[1879503581] = 2, // Ekhamâti-bane of Shagâna</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[26] = {}; -- </v>
+        <v>[26] = {["ID"] = 1879503581; }; -- Ekhamâti-bane of Shagâna</v>
       </c>
       <c r="I27">
         <f t="shared" si="2"/>
@@ -5720,7 +5767,7 @@
       </c>
       <c r="K27" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503581; </v>
       </c>
       <c r="L27" t="str">
         <f t="shared" si="5"/>
@@ -5728,7 +5775,7 @@
       </c>
       <c r="M27" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N27" t="str">
         <f t="shared" si="7"/>
@@ -5736,14 +5783,22 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C28" s="1"/>
+      <c r="A28">
+        <v>1879503582</v>
+      </c>
+      <c r="B28" t="s">
+        <v>376</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1</v>
+      </c>
       <c r="G28" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>[1879503582] = 1, // Tales of the Crown of Hamât</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[27] = {}; -- </v>
+        <v>[27] = {["ID"] = 1879503582; }; -- Tales of the Crown of Hamât</v>
       </c>
       <c r="I28">
         <f t="shared" si="2"/>
@@ -5755,7 +5810,7 @@
       </c>
       <c r="K28" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503582; </v>
       </c>
       <c r="L28" t="str">
         <f t="shared" si="5"/>
@@ -5763,7 +5818,7 @@
       </c>
       <c r="M28" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N28" t="str">
         <f t="shared" si="7"/>
@@ -5771,14 +5826,22 @@
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C29" s="1"/>
+      <c r="A29">
+        <v>1879503577</v>
+      </c>
+      <c r="B29" t="s">
+        <v>377</v>
+      </c>
+      <c r="C29" s="1">
+        <v>1</v>
+      </c>
       <c r="G29" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>[1879503577] = 1, // Treasure-seeker of Shagâna</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">[28] = {}; -- </v>
+        <v>[28] = {["ID"] = 1879503577; }; -- Treasure-seeker of Shagâna</v>
       </c>
       <c r="I29">
         <f t="shared" si="2"/>
@@ -5790,7 +5853,7 @@
       </c>
       <c r="K29" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879503577; </v>
       </c>
       <c r="L29" t="str">
         <f t="shared" si="5"/>
@@ -5798,7 +5861,7 @@
       </c>
       <c r="M29" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">["TIER"] = 0; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N29" t="str">
         <f t="shared" si="7"/>
@@ -5948,1611 +6011,1646 @@
     <row r="34" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C34" s="1"/>
       <c r="G34" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G3:G67" si="8">IF(AND(A34&gt;0,C34&gt;0),CONCATENATE("[",A34,"] = ",C34,", // ",B34),"")</f>
         <v/>
       </c>
       <c r="H34" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="H3:H67" si="9">CONCATENATE(J34,K34,L34,N34," -- ",B34)</f>
         <v xml:space="preserve">[33] = {}; -- </v>
       </c>
       <c r="I34">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I3:I67" si="10">ROW()-1</f>
         <v>33</v>
       </c>
       <c r="J34" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J3:J67" si="11">CONCATENATE(REPT(" ",2-LEN(I34)),"[",I34,"] = {")</f>
         <v>[33] = {</v>
       </c>
       <c r="K34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="K3:K67" si="12">IF(LEN(A34)&gt;0,CONCATENATE("[""ID""] = ",A34,"; "),"")</f>
         <v/>
       </c>
       <c r="L34" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="L3:L67" si="13">IF(LEN(D34)&gt;0,CONCATENATE("[""CAT_ID""] = ",D34,"; "),"")</f>
         <v/>
       </c>
       <c r="M34" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="M3:M67" si="14">CONCATENATE("[""TIER""] = ",TEXT(C34,"0"),"; ")</f>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N34" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="N3:N67" si="15">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
     <row r="35" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C35" s="1"/>
       <c r="G35" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H35" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[34] = {}; -- </v>
       </c>
       <c r="I35">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>34</v>
       </c>
       <c r="J35" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[34] = {</v>
       </c>
       <c r="K35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L35" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M35" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N35" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="36" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C36" s="1"/>
       <c r="G36" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H36" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[35] = {}; -- </v>
       </c>
       <c r="I36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>35</v>
       </c>
       <c r="J36" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[35] = {</v>
       </c>
       <c r="K36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L36" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M36" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N36" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="37" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C37" s="1"/>
       <c r="G37" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H37" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[36] = {}; -- </v>
       </c>
       <c r="I37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>36</v>
       </c>
       <c r="J37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[36] = {</v>
       </c>
       <c r="K37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L37" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M37" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N37" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="38" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C38" s="1"/>
       <c r="G38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H38" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[37] = {}; -- </v>
       </c>
       <c r="I38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>37</v>
       </c>
       <c r="J38" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[37] = {</v>
       </c>
       <c r="K38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L38" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M38" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N38" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="39" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C39" s="1"/>
       <c r="G39" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H39" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[38] = {}; -- </v>
       </c>
       <c r="I39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>38</v>
       </c>
       <c r="J39" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[38] = {</v>
       </c>
       <c r="K39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L39" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M39" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N39" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="40" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C40" s="1"/>
       <c r="G40" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H40" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[39] = {}; -- </v>
       </c>
       <c r="I40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>39</v>
       </c>
       <c r="J40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[39] = {</v>
       </c>
       <c r="K40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L40" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M40" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N40" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="41" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C41" s="1"/>
       <c r="G41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[40] = {}; -- </v>
       </c>
       <c r="I41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>40</v>
       </c>
       <c r="J41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[40] = {</v>
       </c>
       <c r="K41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L41" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M41" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N41" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="42" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C42" s="1"/>
       <c r="G42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H42" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[41] = {}; -- </v>
       </c>
       <c r="I42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>41</v>
       </c>
       <c r="J42" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[41] = {</v>
       </c>
       <c r="K42" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L42" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M42" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N42" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="43" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C43" s="1"/>
       <c r="G43" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H43" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[42] = {}; -- </v>
       </c>
       <c r="I43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>42</v>
       </c>
       <c r="J43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[42] = {</v>
       </c>
       <c r="K43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L43" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M43" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N43" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="44" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C44" s="1"/>
       <c r="G44" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H44" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[43] = {}; -- </v>
       </c>
       <c r="I44">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>43</v>
       </c>
       <c r="J44" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[43] = {</v>
       </c>
       <c r="K44" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L44" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M44" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N44" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="45" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C45" s="1"/>
       <c r="G45" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H45" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[44] = {}; -- </v>
       </c>
       <c r="I45">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>44</v>
       </c>
       <c r="J45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[44] = {</v>
       </c>
       <c r="K45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L45" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M45" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N45" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="46" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C46" s="1"/>
       <c r="G46" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H46" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[45] = {}; -- </v>
       </c>
       <c r="I46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>45</v>
       </c>
       <c r="J46" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[45] = {</v>
       </c>
       <c r="K46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L46" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="47" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C47" s="1"/>
       <c r="G47" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H47" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[46] = {}; -- </v>
       </c>
       <c r="I47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>46</v>
       </c>
       <c r="J47" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[46] = {</v>
       </c>
       <c r="K47" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L47" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M47" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N47" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="48" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C48" s="1"/>
       <c r="G48" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H48" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[47] = {}; -- </v>
       </c>
       <c r="I48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>47</v>
       </c>
       <c r="J48" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[47] = {</v>
       </c>
       <c r="K48" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L48" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M48" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N48" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="49" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C49" s="1"/>
       <c r="G49" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H49" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[48] = {}; -- </v>
       </c>
       <c r="I49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>48</v>
       </c>
       <c r="J49" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[48] = {</v>
       </c>
       <c r="K49" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L49" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M49" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N49" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="50" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C50" s="1"/>
       <c r="G50" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H50" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[49] = {}; -- </v>
       </c>
       <c r="I50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>49</v>
       </c>
       <c r="J50" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[49] = {</v>
       </c>
       <c r="K50" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L50" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M50" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N50" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="51" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C51" s="1"/>
       <c r="G51" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H51" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[50] = {}; -- </v>
       </c>
       <c r="I51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>50</v>
       </c>
       <c r="J51" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[50] = {</v>
       </c>
       <c r="K51" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L51" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M51" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N51" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="52" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C52" s="1"/>
       <c r="G52" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H52" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[51] = {}; -- </v>
       </c>
       <c r="I52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>51</v>
       </c>
       <c r="J52" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[51] = {</v>
       </c>
       <c r="K52" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L52" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M52" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N52" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="53" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C53" s="1"/>
       <c r="G53" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H53" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[52] = {}; -- </v>
       </c>
       <c r="I53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>52</v>
       </c>
       <c r="J53" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[52] = {</v>
       </c>
       <c r="K53" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L53" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M53" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N53" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="54" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C54" s="1"/>
       <c r="G54" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H54" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[53] = {}; -- </v>
       </c>
       <c r="I54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>53</v>
       </c>
       <c r="J54" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[53] = {</v>
       </c>
       <c r="K54" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L54" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M54" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N54" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="55" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C55" s="1"/>
       <c r="G55" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H55" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[54] = {}; -- </v>
       </c>
       <c r="I55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>54</v>
       </c>
       <c r="J55" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[54] = {</v>
       </c>
       <c r="K55" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L55" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M55" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N55" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="56" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C56" s="1"/>
       <c r="G56" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H56" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[55] = {}; -- </v>
       </c>
       <c r="I56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>55</v>
       </c>
       <c r="J56" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[55] = {</v>
       </c>
       <c r="K56" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L56" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M56" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N56" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="57" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C57" s="1"/>
       <c r="G57" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H57" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[56] = {}; -- </v>
       </c>
       <c r="I57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>56</v>
       </c>
       <c r="J57" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[56] = {</v>
       </c>
       <c r="K57" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L57" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M57" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N57" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="58" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C58" s="1"/>
       <c r="G58" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H58" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[57] = {}; -- </v>
       </c>
       <c r="I58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>57</v>
       </c>
       <c r="J58" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[57] = {</v>
       </c>
       <c r="K58" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L58" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M58" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N58" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="59" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C59" s="1"/>
       <c r="G59" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H59" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[58] = {}; -- </v>
       </c>
       <c r="I59">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>58</v>
       </c>
       <c r="J59" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[58] = {</v>
       </c>
       <c r="K59" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L59" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M59" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N59" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="60" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C60" s="1"/>
       <c r="G60" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H60" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[59] = {}; -- </v>
       </c>
       <c r="I60">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>59</v>
       </c>
       <c r="J60" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[59] = {</v>
       </c>
       <c r="K60" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L60" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M60" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N60" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="61" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C61" s="1"/>
       <c r="G61" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H61" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[60] = {}; -- </v>
       </c>
       <c r="I61">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>60</v>
       </c>
       <c r="J61" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[60] = {</v>
       </c>
       <c r="K61" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L61" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M61" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N61" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="62" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C62" s="1"/>
       <c r="G62" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H62" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[61] = {}; -- </v>
       </c>
       <c r="I62">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>61</v>
       </c>
       <c r="J62" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[61] = {</v>
       </c>
       <c r="K62" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L62" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M62" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N62" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="63" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C63" s="1"/>
       <c r="G63" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H63" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[62] = {}; -- </v>
       </c>
       <c r="I63">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>62</v>
       </c>
       <c r="J63" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[62] = {</v>
       </c>
       <c r="K63" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L63" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M63" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N63" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="64" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C64" s="1"/>
       <c r="G64" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H64" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[63] = {}; -- </v>
       </c>
       <c r="I64">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>63</v>
       </c>
       <c r="J64" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[63] = {</v>
       </c>
       <c r="K64" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L64" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M64" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N64" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="65" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C65" s="1"/>
       <c r="G65" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H65" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[64] = {}; -- </v>
       </c>
       <c r="I65">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>64</v>
       </c>
       <c r="J65" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[64] = {</v>
       </c>
       <c r="K65" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L65" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M65" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N65" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="66" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C66" s="1"/>
       <c r="G66" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H66" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[65] = {}; -- </v>
       </c>
       <c r="I66">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>65</v>
       </c>
       <c r="J66" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>[65] = {</v>
       </c>
       <c r="K66" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L66" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M66" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N66" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="67" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C67" s="1"/>
       <c r="G67" t="str">
-        <f t="shared" ref="G67:G78" si="8">IF(AND(A67&gt;0,C67&gt;0),CONCATENATE("[",A67,"] = ",C67,", // ",B67),"")</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="H67" t="str">
-        <f t="shared" ref="H67:H79" si="9">CONCATENATE(J67,K67,L67,N67," -- ",B67)</f>
+        <f t="shared" si="9"/>
         <v xml:space="preserve">[66] = {}; -- </v>
       </c>
       <c r="I67">
-        <f t="shared" ref="I67:I79" si="10">ROW()-1</f>
+        <f t="shared" si="10"/>
         <v>66</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" ref="J67:J79" si="11">CONCATENATE(REPT(" ",2-LEN(I67)),"[",I67,"] = {")</f>
+        <f t="shared" si="11"/>
         <v>[66] = {</v>
       </c>
       <c r="K67" t="str">
-        <f t="shared" ref="K67:K79" si="12">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="L67" t="str">
-        <f t="shared" ref="L67:L79" si="13">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M79" si="14">CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; ")</f>
+        <f t="shared" si="14"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N67" t="str">
-        <f t="shared" ref="N67:N79" si="15">CONCATENATE("};")</f>
+        <f t="shared" si="15"/>
         <v>};</v>
       </c>
     </row>
     <row r="68" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C68" s="1"/>
       <c r="G68" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="G68:G79" si="16">IF(AND(A68&gt;0,C68&gt;0),CONCATENATE("[",A68,"] = ",C68,", // ",B68),"")</f>
         <v/>
       </c>
       <c r="H68" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="H68:H80" si="17">CONCATENATE(J68,K68,L68,N68," -- ",B68)</f>
         <v xml:space="preserve">[67] = {}; -- </v>
       </c>
       <c r="I68">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I68:I80" si="18">ROW()-1</f>
         <v>67</v>
       </c>
       <c r="J68" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="J68:J80" si="19">CONCATENATE(REPT(" ",2-LEN(I68)),"[",I68,"] = {")</f>
         <v>[67] = {</v>
       </c>
       <c r="K68" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="K68:K80" si="20">IF(LEN(A68)&gt;0,CONCATENATE("[""ID""] = ",A68,"; "),"")</f>
         <v/>
       </c>
       <c r="L68" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="L68:L80" si="21">IF(LEN(D68)&gt;0,CONCATENATE("[""CAT_ID""] = ",D68,"; "),"")</f>
         <v/>
       </c>
       <c r="M68" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="M68:M80" si="22">CONCATENATE("[""TIER""] = ",TEXT(C68,"0"),"; ")</f>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N68" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="N68:N80" si="23">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
     <row r="69" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C69" s="1"/>
       <c r="G69" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H69" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[68] = {}; -- </v>
       </c>
       <c r="I69">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>68</v>
       </c>
       <c r="J69" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[68] = {</v>
       </c>
       <c r="K69" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L69" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M69" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N69" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="70" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C70" s="1"/>
       <c r="G70" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H70" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[69] = {}; -- </v>
       </c>
       <c r="I70">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>69</v>
       </c>
       <c r="J70" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[69] = {</v>
       </c>
       <c r="K70" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L70" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M70" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N70" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="71" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C71" s="1"/>
       <c r="G71" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H71" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[70] = {}; -- </v>
       </c>
       <c r="I71">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>70</v>
       </c>
       <c r="J71" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[70] = {</v>
       </c>
       <c r="K71" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L71" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M71" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N71" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="72" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C72" s="1"/>
       <c r="G72" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H72" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[71] = {}; -- </v>
       </c>
       <c r="I72">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>71</v>
       </c>
       <c r="J72" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[71] = {</v>
       </c>
       <c r="K72" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L72" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M72" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N72" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="73" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C73" s="1"/>
       <c r="G73" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H73" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[72] = {}; -- </v>
       </c>
       <c r="I73">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>72</v>
       </c>
       <c r="J73" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[72] = {</v>
       </c>
       <c r="K73" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L73" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M73" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N73" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="74" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C74" s="1"/>
       <c r="G74" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H74" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[73] = {}; -- </v>
       </c>
       <c r="I74">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>73</v>
       </c>
       <c r="J74" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[73] = {</v>
       </c>
       <c r="K74" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L74" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M74" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N74" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="75" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C75" s="1"/>
       <c r="G75" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H75" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[74] = {}; -- </v>
       </c>
       <c r="I75">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>74</v>
       </c>
       <c r="J75" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[74] = {</v>
       </c>
       <c r="K75" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L75" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M75" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N75" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="76" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C76" s="1"/>
       <c r="G76" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H76" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[75] = {}; -- </v>
       </c>
       <c r="I76">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>75</v>
       </c>
       <c r="J76" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[75] = {</v>
       </c>
       <c r="K76" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L76" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M76" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N76" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="77" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C77" s="1"/>
       <c r="G77" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H77" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[76] = {}; -- </v>
       </c>
       <c r="I77">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>76</v>
       </c>
       <c r="J77" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[76] = {</v>
       </c>
       <c r="K77" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L77" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M77" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N77" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="78" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C78" s="1"/>
       <c r="G78" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="H78" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[77] = {}; -- </v>
       </c>
       <c r="I78">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>77</v>
       </c>
       <c r="J78" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[77] = {</v>
       </c>
       <c r="K78" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L78" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M78" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N78" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
     <row r="79" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C79" s="1"/>
+      <c r="G79" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
       <c r="H79" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">[78] = {}; -- </v>
       </c>
       <c r="I79">
-        <f t="shared" si="10"/>
+        <f t="shared" si="18"/>
         <v>78</v>
       </c>
       <c r="J79" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="19"/>
         <v>[78] = {</v>
       </c>
       <c r="K79" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
       <c r="L79" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
       <c r="M79" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v xml:space="preserve">["TIER"] = 0; </v>
       </c>
       <c r="N79" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="23"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="80" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="H80" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">[79] = {}; -- </v>
+      </c>
+      <c r="I80">
+        <f t="shared" si="18"/>
+        <v>79</v>
+      </c>
+      <c r="J80" t="str">
+        <f t="shared" si="19"/>
+        <v>[79] = {</v>
+      </c>
+      <c r="K80" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="L80" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="M80" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="N80" t="str">
+        <f t="shared" si="23"/>
         <v>};</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8388,7 +8486,7 @@
       <c r="A20">
         <v>1879491692</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>363</v>
       </c>
       <c r="C20">
@@ -18064,7 +18162,7 @@
       <c r="A20">
         <v>1879491603</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>304</v>
       </c>
       <c r="C20">

</xml_diff>

<commit_message>
Updated with U46: Kingdoms of Harad deeds.
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
+++ b/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEFFCFE9-5967-4E7B-AC15-42BC430734AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F472B9-C877-4EBE-BBB3-9E792CFC15AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18555" yWindow="1905" windowWidth="18600" windowHeight="14025" tabRatio="869" activeTab="5" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="6540" yWindow="870" windowWidth="21285" windowHeight="14325" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="Khûd Zagin" sheetId="26" r:id="rId10"/>
     <sheet name="Imhûlar" sheetId="27" r:id="rId11"/>
     <sheet name="Urash Dâr" sheetId="29" r:id="rId12"/>
+    <sheet name="Mûr Ghala" sheetId="30" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="477">
   <si>
     <t>TIER</t>
   </si>
@@ -1179,6 +1180,303 @@
   </si>
   <si>
     <t>Treasure-seeker of Shagâna</t>
+  </si>
+  <si>
+    <t>Rejuvenator of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Renewing Adagím</t>
+  </si>
+  <si>
+    <t>Exploring Adagím</t>
+  </si>
+  <si>
+    <t>New Threats in Adagím</t>
+  </si>
+  <si>
+    <t>Scouting Adagím</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Adagím</t>
+  </si>
+  <si>
+    <t>Slayer of Adagím</t>
+  </si>
+  <si>
+    <t>Bog-slayer of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Bog-slayer of Adagím</t>
+  </si>
+  <si>
+    <t>Crocodile-slayer of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Crocodile-slayer of Adagím</t>
+  </si>
+  <si>
+    <t>Huorn-bane of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Huorn-bane of Adagím</t>
+  </si>
+  <si>
+    <t>Orc-bane of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Orc-bane of Adagím</t>
+  </si>
+  <si>
+    <t>Spider-slayer of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Spider-slayer of Adagím</t>
+  </si>
+  <si>
+    <t>Wood-troll Slayer of Adagím (Advanced)</t>
+  </si>
+  <si>
+    <t>Wood-troll Slayer of Adagím</t>
+  </si>
+  <si>
+    <t>Tales of Adagím</t>
+  </si>
+  <si>
+    <t>Rejuvenator of Kighân</t>
+  </si>
+  <si>
+    <t>Explorer of Kighân</t>
+  </si>
+  <si>
+    <t>Dangers in Kighân</t>
+  </si>
+  <si>
+    <t>Scouting Kighân</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Kighân</t>
+  </si>
+  <si>
+    <t>Slayer of Kighân</t>
+  </si>
+  <si>
+    <t>Tarsâri-bane of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Tarsâri-bane of Kighân</t>
+  </si>
+  <si>
+    <t>Bee-slayer of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Bee-slayer of Kighân</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Kighân</t>
+  </si>
+  <si>
+    <t>Goblin-bane of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Goblin-bane of Kighân</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Kighân</t>
+  </si>
+  <si>
+    <t>Spider-slayer of Kighân (Advanced)</t>
+  </si>
+  <si>
+    <t>Spider-slayer of Kighân</t>
+  </si>
+  <si>
+    <t>Tales of Kighân</t>
+  </si>
+  <si>
+    <t>Rejuvenator of An Shêru</t>
+  </si>
+  <si>
+    <t>Explorer of An Shêru</t>
+  </si>
+  <si>
+    <t>New Threats in An Shêru</t>
+  </si>
+  <si>
+    <t>Reclaiming An Shêru</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of An Shêru</t>
+  </si>
+  <si>
+    <t>Slayer of An Shêru</t>
+  </si>
+  <si>
+    <t>Brigand-bane of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Brigand-bane of An Shêru</t>
+  </si>
+  <si>
+    <t>Dead-slayer of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Dead-slayer of An Shêru</t>
+  </si>
+  <si>
+    <t>Utûgi-bane of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Utûgi-bane of An Shêru</t>
+  </si>
+  <si>
+    <t>Grodbog-slayer of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Grodbog-slayer of An Shêru</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of An Shêru</t>
+  </si>
+  <si>
+    <t>Worm-bane of An Shêru (Advanced)</t>
+  </si>
+  <si>
+    <t>Worm-bane of An Shêru</t>
+  </si>
+  <si>
+    <t>Tales of An Shêru</t>
+  </si>
+  <si>
+    <t>Renewer of Idagâl</t>
+  </si>
+  <si>
+    <t>Explorer of Idagâl</t>
+  </si>
+  <si>
+    <t>New Threats in Idagâl</t>
+  </si>
+  <si>
+    <t>Reclaiming Idagâl</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Idagâl</t>
+  </si>
+  <si>
+    <t>Slayer of Idagâl</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Idagâl</t>
+  </si>
+  <si>
+    <t>Cobra-slayer of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Cobra-slayer of Idagâl</t>
+  </si>
+  <si>
+    <t>Drake-slayer of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Drake-slayer of Idagâl</t>
+  </si>
+  <si>
+    <t>Utûgi-bane of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Utûgi-bane of Idagâl</t>
+  </si>
+  <si>
+    <t>Kergrim-slayer of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Kergrim-slayer of Idagâl</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Idagâl (Advanced)</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Idagâl</t>
+  </si>
+  <si>
+    <t>Tales of Idagâl</t>
+  </si>
+  <si>
+    <t>Adagím</t>
+  </si>
+  <si>
+    <t>Kighân</t>
+  </si>
+  <si>
+    <t>An Shêru</t>
+  </si>
+  <si>
+    <t>Idagâl</t>
+  </si>
+  <si>
+    <t>Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Hunter of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Adversaries of Adagím</t>
+  </si>
+  <si>
+    <t>Combatants of Kighân</t>
+  </si>
+  <si>
+    <t>Enemies of An Shêru</t>
+  </si>
+  <si>
+    <t>Invaders of Idagâl</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Nightmare of the Ordâkhai</t>
+  </si>
+  <si>
+    <t>Spider-slayer of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Slayer of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Orc-slayer of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Tales of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Explorer of Mûr Ghala</t>
+  </si>
+  <si>
+    <t>Defender of Adagím</t>
+  </si>
+  <si>
+    <t>Defender of Kighân</t>
+  </si>
+  <si>
+    <t>Defender of An Shêru</t>
+  </si>
+  <si>
+    <t>Defender of Idagâl</t>
   </si>
 </sst>
 </file>
@@ -5630,6 +5928,4124 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D727EC7-6195-47C5-8CEB-067AA7EF5F9D}">
+  <dimension ref="A1:N103"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="48.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="85.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G1" t="s">
+        <v>188</v>
+      </c>
+      <c r="H1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" t="s">
+        <v>123</v>
+      </c>
+      <c r="L1" t="s">
+        <v>122</v>
+      </c>
+      <c r="M1" t="s">
+        <v>126</v>
+      </c>
+      <c r="N1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1879513802</v>
+      </c>
+      <c r="B2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G2" t="str">
+        <f>IF(AND(A2&gt;0,C2&gt;0),CONCATENATE("[",A2,"] = ",C2,", // ",B2),"")</f>
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <f>CONCATENATE(J2,K2,L2,M2,N2," -- ",B2)</f>
+        <v xml:space="preserve"> [1] = {["ID"] = 1879513802; }; -- Rejuvenator of Mûr Ghala</v>
+      </c>
+      <c r="I2">
+        <f>ROW()-1</f>
+        <v>1</v>
+      </c>
+      <c r="J2" t="str">
+        <f>CONCATENATE(REPT(" ",2-LEN(I2)),"[",I2,"] = {")</f>
+        <v xml:space="preserve"> [1] = {</v>
+      </c>
+      <c r="K2" t="str">
+        <f>IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"")</f>
+        <v xml:space="preserve">["ID"] = 1879513802; </v>
+      </c>
+      <c r="L2" t="str">
+        <f>IF(LEN(D2)&gt;0,CONCATENATE("[""CAT_ID""] = ",D2,"; "),"")</f>
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <f>IF(C2&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C2,"0"),"; "),"")</f>
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <f>CONCATENATE("};")</f>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>337</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H66" si="0">CONCATENATE(J3,K3,L3,M3,N3," -- ",B3)</f>
+        <v xml:space="preserve"> [2] = {["CAT_ID"] = 337; ["TIER"] = 1; }; -- Adagím</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I66" si="1">ROW()-1</f>
+        <v>2</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J66" si="2">CONCATENATE(REPT(" ",2-LEN(I3)),"[",I3,"] = {")</f>
+        <v xml:space="preserve"> [2] = {</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K66" si="3">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L66" si="4">IF(LEN(D3)&gt;0,CONCATENATE("[""CAT_ID""] = ",D3,"; "),"")</f>
+        <v xml:space="preserve">["CAT_ID"] = 337; </v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M66" si="5">IF(C3&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C3,"0"),"; "),"")</f>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:N66" si="6">CONCATENATE("};")</f>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1879513774</v>
+      </c>
+      <c r="B4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" ref="G4:G41" si="7">IF(AND(A4&gt;0,C4&gt;0),CONCATENATE("[",A4,"] = ",C4,", // ",B4),"")</f>
+        <v>[1879513774] = 1, // Renewing Adagím</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [3] = {["ID"] = 1879513774; ["TIER"] = 1; }; -- Renewing Adagím</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [3] = {</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513774; </v>
+      </c>
+      <c r="L4" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1879513785</v>
+      </c>
+      <c r="B5" t="s">
+        <v>380</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513785] = 2, // Exploring Adagím</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [4] = {["ID"] = 1879513785; ["TIER"] = 2; }; -- Exploring Adagím</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [4] = {</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513785; </v>
+      </c>
+      <c r="L5" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1879513778</v>
+      </c>
+      <c r="B6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513778] = 3, // New Threats in Adagím</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [5] = {["ID"] = 1879513778; ["TIER"] = 3; }; -- New Threats in Adagím</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [5] = {</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513778; </v>
+      </c>
+      <c r="L6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1879513790</v>
+      </c>
+      <c r="B7" t="s">
+        <v>382</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513790] = 3, // Scouting Adagím</v>
+      </c>
+      <c r="H7" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [6] = {["ID"] = 1879513790; ["TIER"] = 3; }; -- Scouting Adagím</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [6] = {</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513790; </v>
+      </c>
+      <c r="L7" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N7" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1879513702</v>
+      </c>
+      <c r="B8" t="s">
+        <v>383</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513702] = 3, // Treasure-seeker of Adagím</v>
+      </c>
+      <c r="H8" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [7] = {["ID"] = 1879513702; ["TIER"] = 3; }; -- Treasure-seeker of Adagím</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [7] = {</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513702; </v>
+      </c>
+      <c r="L8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N8" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1879513704</v>
+      </c>
+      <c r="B9" t="s">
+        <v>384</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513704] = 2, // Slayer of Adagím</v>
+      </c>
+      <c r="H9" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [8] = {["ID"] = 1879513704; ["TIER"] = 2; }; -- Slayer of Adagím</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [8] = {</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513704; </v>
+      </c>
+      <c r="L9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N9" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1879513641</v>
+      </c>
+      <c r="B10" t="s">
+        <v>385</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513641] = 3, // Bog-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="H10" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [9] = {["ID"] = 1879513641; ["TIER"] = 3; }; -- Bog-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="J10" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [9] = {</v>
+      </c>
+      <c r="K10" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513641; </v>
+      </c>
+      <c r="L10" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N10" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1879513640</v>
+      </c>
+      <c r="B11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513640] = 4, // Bog-slayer of Adagím</v>
+      </c>
+      <c r="H11" t="str">
+        <f t="shared" si="0"/>
+        <v>[10] = {["ID"] = 1879513640; ["TIER"] = 4; }; -- Bog-slayer of Adagím</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="J11" t="str">
+        <f t="shared" si="2"/>
+        <v>[10] = {</v>
+      </c>
+      <c r="K11" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513640; </v>
+      </c>
+      <c r="L11" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N11" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>1879513644</v>
+      </c>
+      <c r="B12" t="s">
+        <v>387</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513644] = 3, // Crocodile-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="H12" t="str">
+        <f t="shared" si="0"/>
+        <v>[11] = {["ID"] = 1879513644; ["TIER"] = 3; }; -- Crocodile-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="J12" t="str">
+        <f t="shared" si="2"/>
+        <v>[11] = {</v>
+      </c>
+      <c r="K12" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513644; </v>
+      </c>
+      <c r="L12" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N12" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1879513647</v>
+      </c>
+      <c r="B13" t="s">
+        <v>388</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513647] = 4, // Crocodile-slayer of Adagím</v>
+      </c>
+      <c r="H13" t="str">
+        <f t="shared" si="0"/>
+        <v>[12] = {["ID"] = 1879513647; ["TIER"] = 4; }; -- Crocodile-slayer of Adagím</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="J13" t="str">
+        <f t="shared" si="2"/>
+        <v>[12] = {</v>
+      </c>
+      <c r="K13" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513647; </v>
+      </c>
+      <c r="L13" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N13" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>1879513663</v>
+      </c>
+      <c r="B14" t="s">
+        <v>389</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513663] = 3, // Huorn-bane of Adagím (Advanced)</v>
+      </c>
+      <c r="H14" t="str">
+        <f t="shared" si="0"/>
+        <v>[13] = {["ID"] = 1879513663; ["TIER"] = 3; }; -- Huorn-bane of Adagím (Advanced)</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="J14" t="str">
+        <f t="shared" si="2"/>
+        <v>[13] = {</v>
+      </c>
+      <c r="K14" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513663; </v>
+      </c>
+      <c r="L14" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N14" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>1879513664</v>
+      </c>
+      <c r="B15" t="s">
+        <v>390</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513664] = 4, // Huorn-bane of Adagím</v>
+      </c>
+      <c r="H15" t="str">
+        <f t="shared" si="0"/>
+        <v>[14] = {["ID"] = 1879513664; ["TIER"] = 4; }; -- Huorn-bane of Adagím</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="J15" t="str">
+        <f t="shared" si="2"/>
+        <v>[14] = {</v>
+      </c>
+      <c r="K15" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513664; </v>
+      </c>
+      <c r="L15" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N15" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1879513659</v>
+      </c>
+      <c r="B16" t="s">
+        <v>391</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513659] = 3, // Orc-bane of Adagím (Advanced)</v>
+      </c>
+      <c r="H16" t="str">
+        <f t="shared" si="0"/>
+        <v>[15] = {["ID"] = 1879513659; ["TIER"] = 3; }; -- Orc-bane of Adagím (Advanced)</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J16" t="str">
+        <f t="shared" si="2"/>
+        <v>[15] = {</v>
+      </c>
+      <c r="K16" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513659; </v>
+      </c>
+      <c r="L16" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N16" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>1879513653</v>
+      </c>
+      <c r="B17" t="s">
+        <v>392</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513653] = 4, // Orc-bane of Adagím</v>
+      </c>
+      <c r="H17" t="str">
+        <f t="shared" si="0"/>
+        <v>[16] = {["ID"] = 1879513653; ["TIER"] = 4; }; -- Orc-bane of Adagím</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="J17" t="str">
+        <f t="shared" si="2"/>
+        <v>[16] = {</v>
+      </c>
+      <c r="K17" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513653; </v>
+      </c>
+      <c r="L17" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N17" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>1879513645</v>
+      </c>
+      <c r="B18" t="s">
+        <v>393</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513645] = 3, // Spider-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="H18" t="str">
+        <f t="shared" si="0"/>
+        <v>[17] = {["ID"] = 1879513645; ["TIER"] = 3; }; -- Spider-slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="J18" t="str">
+        <f t="shared" si="2"/>
+        <v>[17] = {</v>
+      </c>
+      <c r="K18" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513645; </v>
+      </c>
+      <c r="L18" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N18" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>1879513651</v>
+      </c>
+      <c r="B19" t="s">
+        <v>394</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513651] = 4, // Spider-slayer of Adagím</v>
+      </c>
+      <c r="H19" t="str">
+        <f t="shared" si="0"/>
+        <v>[18] = {["ID"] = 1879513651; ["TIER"] = 4; }; -- Spider-slayer of Adagím</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="J19" t="str">
+        <f t="shared" si="2"/>
+        <v>[18] = {</v>
+      </c>
+      <c r="K19" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513651; </v>
+      </c>
+      <c r="L19" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N19" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1879513649</v>
+      </c>
+      <c r="B20" t="s">
+        <v>395</v>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513649] = 3, // Wood-troll Slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="H20" t="str">
+        <f t="shared" si="0"/>
+        <v>[19] = {["ID"] = 1879513649; ["TIER"] = 3; }; -- Wood-troll Slayer of Adagím (Advanced)</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="J20" t="str">
+        <f t="shared" si="2"/>
+        <v>[19] = {</v>
+      </c>
+      <c r="K20" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513649; </v>
+      </c>
+      <c r="L20" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N20" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>1879513650</v>
+      </c>
+      <c r="B21" t="s">
+        <v>396</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513650] = 4, // Wood-troll Slayer of Adagím</v>
+      </c>
+      <c r="H21" t="str">
+        <f t="shared" si="0"/>
+        <v>[20] = {["ID"] = 1879513650; ["TIER"] = 4; }; -- Wood-troll Slayer of Adagím</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="J21" t="str">
+        <f t="shared" si="2"/>
+        <v>[20] = {</v>
+      </c>
+      <c r="K21" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513650; </v>
+      </c>
+      <c r="L21" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N21" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1879513791</v>
+      </c>
+      <c r="B22" t="s">
+        <v>397</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513791] = 2, // Tales of Adagím</v>
+      </c>
+      <c r="H22" t="str">
+        <f t="shared" si="0"/>
+        <v>[21] = {["ID"] = 1879513791; ["TIER"] = 2; }; -- Tales of Adagím</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="J22" t="str">
+        <f t="shared" si="2"/>
+        <v>[21] = {</v>
+      </c>
+      <c r="K22" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513791; </v>
+      </c>
+      <c r="L22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N22" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>338</v>
+      </c>
+      <c r="H23" t="str">
+        <f t="shared" si="0"/>
+        <v>[22] = {["CAT_ID"] = 338; ["TIER"] = 1; }; -- Kighân</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="J23" t="str">
+        <f t="shared" si="2"/>
+        <v>[22] = {</v>
+      </c>
+      <c r="K23" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve">["CAT_ID"] = 338; </v>
+      </c>
+      <c r="M23" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N23" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>1879513787</v>
+      </c>
+      <c r="B24" t="s">
+        <v>398</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513787] = 1, // Rejuvenator of Kighân</v>
+      </c>
+      <c r="H24" t="str">
+        <f t="shared" si="0"/>
+        <v>[23] = {["ID"] = 1879513787; ["TIER"] = 1; }; -- Rejuvenator of Kighân</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="J24" t="str">
+        <f t="shared" si="2"/>
+        <v>[23] = {</v>
+      </c>
+      <c r="K24" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513787; </v>
+      </c>
+      <c r="L24" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N24" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>1879513779</v>
+      </c>
+      <c r="B25" t="s">
+        <v>399</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513779] = 2, // Explorer of Kighân</v>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" si="0"/>
+        <v>[24] = {["ID"] = 1879513779; ["TIER"] = 2; }; -- Explorer of Kighân</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="J25" t="str">
+        <f t="shared" si="2"/>
+        <v>[24] = {</v>
+      </c>
+      <c r="K25" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513779; </v>
+      </c>
+      <c r="L25" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N25" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>1879513781</v>
+      </c>
+      <c r="B26" t="s">
+        <v>400</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513781] = 3, // Dangers in Kighân</v>
+      </c>
+      <c r="H26" t="str">
+        <f t="shared" si="0"/>
+        <v>[25] = {["ID"] = 1879513781; ["TIER"] = 3; }; -- Dangers in Kighân</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="J26" t="str">
+        <f t="shared" si="2"/>
+        <v>[25] = {</v>
+      </c>
+      <c r="K26" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513781; </v>
+      </c>
+      <c r="L26" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N26" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>1879513782</v>
+      </c>
+      <c r="B27" t="s">
+        <v>401</v>
+      </c>
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513782] = 3, // Scouting Kighân</v>
+      </c>
+      <c r="H27" t="str">
+        <f t="shared" si="0"/>
+        <v>[26] = {["ID"] = 1879513782; ["TIER"] = 3; }; -- Scouting Kighân</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="J27" t="str">
+        <f t="shared" si="2"/>
+        <v>[26] = {</v>
+      </c>
+      <c r="K27" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513782; </v>
+      </c>
+      <c r="L27" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N27" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>1879513701</v>
+      </c>
+      <c r="B28" t="s">
+        <v>402</v>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513701] = 3, // Treasure-seeker of Kighân</v>
+      </c>
+      <c r="H28" t="str">
+        <f t="shared" si="0"/>
+        <v>[27] = {["ID"] = 1879513701; ["TIER"] = 3; }; -- Treasure-seeker of Kighân</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" si="2"/>
+        <v>[27] = {</v>
+      </c>
+      <c r="K28" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513701; </v>
+      </c>
+      <c r="L28" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N28" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>1879513706</v>
+      </c>
+      <c r="B29" t="s">
+        <v>403</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513706] = 2, // Slayer of Kighân</v>
+      </c>
+      <c r="H29" t="str">
+        <f t="shared" si="0"/>
+        <v>[28] = {["ID"] = 1879513706; ["TIER"] = 2; }; -- Slayer of Kighân</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="J29" t="str">
+        <f t="shared" si="2"/>
+        <v>[28] = {</v>
+      </c>
+      <c r="K29" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513706; </v>
+      </c>
+      <c r="L29" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N29" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>1879513660</v>
+      </c>
+      <c r="B30" t="s">
+        <v>404</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513660] = 3, // Tarsâri-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="H30" t="str">
+        <f t="shared" si="0"/>
+        <v>[29] = {["ID"] = 1879513660; ["TIER"] = 3; }; -- Tarsâri-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="J30" t="str">
+        <f t="shared" si="2"/>
+        <v>[29] = {</v>
+      </c>
+      <c r="K30" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513660; </v>
+      </c>
+      <c r="L30" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N30" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>1879513655</v>
+      </c>
+      <c r="B31" t="s">
+        <v>405</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513655] = 4, // Tarsâri-bane of Kighân</v>
+      </c>
+      <c r="H31" t="str">
+        <f t="shared" si="0"/>
+        <v>[30] = {["ID"] = 1879513655; ["TIER"] = 4; }; -- Tarsâri-bane of Kighân</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="J31" t="str">
+        <f t="shared" si="2"/>
+        <v>[30] = {</v>
+      </c>
+      <c r="K31" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513655; </v>
+      </c>
+      <c r="L31" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N31" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>1879513656</v>
+      </c>
+      <c r="B32" t="s">
+        <v>406</v>
+      </c>
+      <c r="C32">
+        <v>3</v>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513656] = 3, // Bee-slayer of Kighân (Advanced)</v>
+      </c>
+      <c r="H32" t="str">
+        <f t="shared" si="0"/>
+        <v>[31] = {["ID"] = 1879513656; ["TIER"] = 3; }; -- Bee-slayer of Kighân (Advanced)</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="J32" t="str">
+        <f t="shared" si="2"/>
+        <v>[31] = {</v>
+      </c>
+      <c r="K32" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513656; </v>
+      </c>
+      <c r="L32" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N32" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>1879513654</v>
+      </c>
+      <c r="B33" t="s">
+        <v>407</v>
+      </c>
+      <c r="C33">
+        <v>4</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513654] = 4, // Bee-slayer of Kighân</v>
+      </c>
+      <c r="H33" t="str">
+        <f t="shared" si="0"/>
+        <v>[32] = {["ID"] = 1879513654; ["TIER"] = 4; }; -- Bee-slayer of Kighân</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="J33" t="str">
+        <f t="shared" si="2"/>
+        <v>[32] = {</v>
+      </c>
+      <c r="K33" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513654; </v>
+      </c>
+      <c r="L33" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N33" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>1879513661</v>
+      </c>
+      <c r="B34" t="s">
+        <v>408</v>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513661] = 3, // Brigand-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="H34" t="str">
+        <f t="shared" si="0"/>
+        <v>[33] = {["ID"] = 1879513661; ["TIER"] = 3; }; -- Brigand-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="J34" t="str">
+        <f t="shared" si="2"/>
+        <v>[33] = {</v>
+      </c>
+      <c r="K34" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513661; </v>
+      </c>
+      <c r="L34" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N34" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>1879513657</v>
+      </c>
+      <c r="B35" t="s">
+        <v>409</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513657] = 4, // Brigand-bane of Kighân</v>
+      </c>
+      <c r="H35" t="str">
+        <f t="shared" si="0"/>
+        <v>[34] = {["ID"] = 1879513657; ["TIER"] = 4; }; -- Brigand-bane of Kighân</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="J35" t="str">
+        <f t="shared" si="2"/>
+        <v>[34] = {</v>
+      </c>
+      <c r="K35" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513657; </v>
+      </c>
+      <c r="L35" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N35" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>1879513662</v>
+      </c>
+      <c r="B36" t="s">
+        <v>410</v>
+      </c>
+      <c r="C36">
+        <v>3</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513662] = 3, // Goblin-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="H36" t="str">
+        <f t="shared" si="0"/>
+        <v>[35] = {["ID"] = 1879513662; ["TIER"] = 3; }; -- Goblin-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="J36" t="str">
+        <f t="shared" si="2"/>
+        <v>[35] = {</v>
+      </c>
+      <c r="K36" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513662; </v>
+      </c>
+      <c r="L36" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N36" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>1879513658</v>
+      </c>
+      <c r="B37" t="s">
+        <v>411</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513658] = 4, // Goblin-bane of Kighân</v>
+      </c>
+      <c r="H37" t="str">
+        <f t="shared" si="0"/>
+        <v>[36] = {["ID"] = 1879513658; ["TIER"] = 4; }; -- Goblin-bane of Kighân</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="J37" t="str">
+        <f t="shared" si="2"/>
+        <v>[36] = {</v>
+      </c>
+      <c r="K37" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513658; </v>
+      </c>
+      <c r="L37" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N37" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>1879513648</v>
+      </c>
+      <c r="B38" t="s">
+        <v>412</v>
+      </c>
+      <c r="C38">
+        <v>3</v>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513648] = 3, // Ordâkhai-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="H38" t="str">
+        <f t="shared" si="0"/>
+        <v>[37] = {["ID"] = 1879513648; ["TIER"] = 3; }; -- Ordâkhai-bane of Kighân (Advanced)</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="J38" t="str">
+        <f t="shared" si="2"/>
+        <v>[37] = {</v>
+      </c>
+      <c r="K38" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513648; </v>
+      </c>
+      <c r="L38" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N38" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>1879513652</v>
+      </c>
+      <c r="B39" t="s">
+        <v>413</v>
+      </c>
+      <c r="C39">
+        <v>4</v>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513652] = 4, // Ordâkhai-bane of Kighân</v>
+      </c>
+      <c r="H39" t="str">
+        <f t="shared" si="0"/>
+        <v>[38] = {["ID"] = 1879513652; ["TIER"] = 4; }; -- Ordâkhai-bane of Kighân</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="J39" t="str">
+        <f t="shared" si="2"/>
+        <v>[38] = {</v>
+      </c>
+      <c r="K39" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513652; </v>
+      </c>
+      <c r="L39" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N39" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>1879513643</v>
+      </c>
+      <c r="B40" t="s">
+        <v>414</v>
+      </c>
+      <c r="C40">
+        <v>3</v>
+      </c>
+      <c r="G40" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513643] = 3, // Spider-slayer of Kighân (Advanced)</v>
+      </c>
+      <c r="H40" t="str">
+        <f t="shared" si="0"/>
+        <v>[39] = {["ID"] = 1879513643; ["TIER"] = 3; }; -- Spider-slayer of Kighân (Advanced)</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="J40" t="str">
+        <f t="shared" si="2"/>
+        <v>[39] = {</v>
+      </c>
+      <c r="K40" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513643; </v>
+      </c>
+      <c r="L40" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N40" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>1879513646</v>
+      </c>
+      <c r="B41" t="s">
+        <v>415</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="G41" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513646] = 4, // Spider-slayer of Kighân</v>
+      </c>
+      <c r="H41" t="str">
+        <f t="shared" si="0"/>
+        <v>[40] = {["ID"] = 1879513646; ["TIER"] = 4; }; -- Spider-slayer of Kighân</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="J41" t="str">
+        <f t="shared" si="2"/>
+        <v>[40] = {</v>
+      </c>
+      <c r="K41" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513646; </v>
+      </c>
+      <c r="L41" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N41" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>1879513792</v>
+      </c>
+      <c r="B42" t="s">
+        <v>416</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="H42" t="str">
+        <f t="shared" si="0"/>
+        <v>[41] = {["ID"] = 1879513792; ["TIER"] = 2; }; -- Tales of Kighân</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="2"/>
+        <v>[41] = {</v>
+      </c>
+      <c r="K42" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513792; </v>
+      </c>
+      <c r="L42" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N42" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43">
+        <v>339</v>
+      </c>
+      <c r="H43" t="str">
+        <f t="shared" si="0"/>
+        <v>[42] = {["CAT_ID"] = 339; ["TIER"] = 1; }; -- An Shêru</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="2"/>
+        <v>[42] = {</v>
+      </c>
+      <c r="K43" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve">["CAT_ID"] = 339; </v>
+      </c>
+      <c r="M43" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N43" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>1879513780</v>
+      </c>
+      <c r="B44" t="s">
+        <v>417</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="H44" t="str">
+        <f t="shared" si="0"/>
+        <v>[43] = {["ID"] = 1879513780; ["TIER"] = 1; }; -- Rejuvenator of An Shêru</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+      <c r="J44" t="str">
+        <f t="shared" si="2"/>
+        <v>[43] = {</v>
+      </c>
+      <c r="K44" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513780; </v>
+      </c>
+      <c r="L44" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M44" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N44" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>1879513788</v>
+      </c>
+      <c r="B45" t="s">
+        <v>418</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="H45" t="str">
+        <f t="shared" si="0"/>
+        <v>[44] = {["ID"] = 1879513788; ["TIER"] = 2; }; -- Explorer of An Shêru</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="1"/>
+        <v>44</v>
+      </c>
+      <c r="J45" t="str">
+        <f t="shared" si="2"/>
+        <v>[44] = {</v>
+      </c>
+      <c r="K45" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513788; </v>
+      </c>
+      <c r="L45" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M45" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N45" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>1879513789</v>
+      </c>
+      <c r="B46" t="s">
+        <v>419</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="H46" t="str">
+        <f t="shared" si="0"/>
+        <v>[45] = {["ID"] = 1879513789; ["TIER"] = 3; }; -- New Threats in An Shêru</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="J46" t="str">
+        <f t="shared" si="2"/>
+        <v>[45] = {</v>
+      </c>
+      <c r="K46" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513789; </v>
+      </c>
+      <c r="L46" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M46" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N46" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>1879513775</v>
+      </c>
+      <c r="B47" t="s">
+        <v>420</v>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+      <c r="H47" t="str">
+        <f t="shared" si="0"/>
+        <v>[46] = {["ID"] = 1879513775; ["TIER"] = 3; }; -- Reclaiming An Shêru</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="1"/>
+        <v>46</v>
+      </c>
+      <c r="J47" t="str">
+        <f t="shared" si="2"/>
+        <v>[46] = {</v>
+      </c>
+      <c r="K47" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513775; </v>
+      </c>
+      <c r="L47" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M47" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N47" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>1879513707</v>
+      </c>
+      <c r="B48" t="s">
+        <v>421</v>
+      </c>
+      <c r="C48">
+        <v>3</v>
+      </c>
+      <c r="H48" t="str">
+        <f t="shared" si="0"/>
+        <v>[47] = {["ID"] = 1879513707; ["TIER"] = 3; }; -- Treasure-seeker of An Shêru</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="1"/>
+        <v>47</v>
+      </c>
+      <c r="J48" t="str">
+        <f t="shared" si="2"/>
+        <v>[47] = {</v>
+      </c>
+      <c r="K48" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513707; </v>
+      </c>
+      <c r="L48" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M48" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N48" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>1879513697</v>
+      </c>
+      <c r="B49" t="s">
+        <v>422</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+      <c r="H49" t="str">
+        <f t="shared" si="0"/>
+        <v>[48] = {["ID"] = 1879513697; ["TIER"] = 2; }; -- Slayer of An Shêru</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="1"/>
+        <v>48</v>
+      </c>
+      <c r="J49" t="str">
+        <f t="shared" si="2"/>
+        <v>[48] = {</v>
+      </c>
+      <c r="K49" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513697; </v>
+      </c>
+      <c r="L49" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M49" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N49" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>1879513669</v>
+      </c>
+      <c r="B50" t="s">
+        <v>423</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="H50" t="str">
+        <f t="shared" si="0"/>
+        <v>[49] = {["ID"] = 1879513669; ["TIER"] = 3; }; -- Brigand-bane of An Shêru (Advanced)</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="1"/>
+        <v>49</v>
+      </c>
+      <c r="J50" t="str">
+        <f t="shared" si="2"/>
+        <v>[49] = {</v>
+      </c>
+      <c r="K50" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513669; </v>
+      </c>
+      <c r="L50" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M50" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N50" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>1879513688</v>
+      </c>
+      <c r="B51" t="s">
+        <v>424</v>
+      </c>
+      <c r="C51">
+        <v>4</v>
+      </c>
+      <c r="H51" t="str">
+        <f t="shared" si="0"/>
+        <v>[50] = {["ID"] = 1879513688; ["TIER"] = 4; }; -- Brigand-bane of An Shêru</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="J51" t="str">
+        <f t="shared" si="2"/>
+        <v>[50] = {</v>
+      </c>
+      <c r="K51" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513688; </v>
+      </c>
+      <c r="L51" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N51" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>1879513668</v>
+      </c>
+      <c r="B52" t="s">
+        <v>425</v>
+      </c>
+      <c r="C52">
+        <v>3</v>
+      </c>
+      <c r="H52" t="str">
+        <f t="shared" si="0"/>
+        <v>[51] = {["ID"] = 1879513668; ["TIER"] = 3; }; -- Dead-slayer of An Shêru (Advanced)</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="1"/>
+        <v>51</v>
+      </c>
+      <c r="J52" t="str">
+        <f t="shared" si="2"/>
+        <v>[51] = {</v>
+      </c>
+      <c r="K52" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513668; </v>
+      </c>
+      <c r="L52" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M52" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N52" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>1879513682</v>
+      </c>
+      <c r="B53" t="s">
+        <v>426</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+      <c r="H53" t="str">
+        <f t="shared" si="0"/>
+        <v>[52] = {["ID"] = 1879513682; ["TIER"] = 4; }; -- Dead-slayer of An Shêru</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="1"/>
+        <v>52</v>
+      </c>
+      <c r="J53" t="str">
+        <f t="shared" si="2"/>
+        <v>[52] = {</v>
+      </c>
+      <c r="K53" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513682; </v>
+      </c>
+      <c r="L53" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N53" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>1879513665</v>
+      </c>
+      <c r="B54" t="s">
+        <v>427</v>
+      </c>
+      <c r="C54">
+        <v>3</v>
+      </c>
+      <c r="H54" t="str">
+        <f t="shared" si="0"/>
+        <v>[53] = {["ID"] = 1879513665; ["TIER"] = 3; }; -- Utûgi-bane of An Shêru (Advanced)</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="1"/>
+        <v>53</v>
+      </c>
+      <c r="J54" t="str">
+        <f t="shared" si="2"/>
+        <v>[53] = {</v>
+      </c>
+      <c r="K54" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513665; </v>
+      </c>
+      <c r="L54" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N54" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>1879513674</v>
+      </c>
+      <c r="B55" t="s">
+        <v>428</v>
+      </c>
+      <c r="C55">
+        <v>4</v>
+      </c>
+      <c r="H55" t="str">
+        <f t="shared" si="0"/>
+        <v>[54] = {["ID"] = 1879513674; ["TIER"] = 4; }; -- Utûgi-bane of An Shêru</v>
+      </c>
+      <c r="I55">
+        <f t="shared" si="1"/>
+        <v>54</v>
+      </c>
+      <c r="J55" t="str">
+        <f t="shared" si="2"/>
+        <v>[54] = {</v>
+      </c>
+      <c r="K55" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513674; </v>
+      </c>
+      <c r="L55" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M55" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N55" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>1879513681</v>
+      </c>
+      <c r="B56" t="s">
+        <v>429</v>
+      </c>
+      <c r="C56">
+        <v>3</v>
+      </c>
+      <c r="H56" t="str">
+        <f t="shared" si="0"/>
+        <v>[55] = {["ID"] = 1879513681; ["TIER"] = 3; }; -- Grodbog-slayer of An Shêru (Advanced)</v>
+      </c>
+      <c r="I56">
+        <f t="shared" si="1"/>
+        <v>55</v>
+      </c>
+      <c r="J56" t="str">
+        <f t="shared" si="2"/>
+        <v>[55] = {</v>
+      </c>
+      <c r="K56" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513681; </v>
+      </c>
+      <c r="L56" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M56" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N56" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>1879513673</v>
+      </c>
+      <c r="B57" t="s">
+        <v>430</v>
+      </c>
+      <c r="C57">
+        <v>4</v>
+      </c>
+      <c r="H57" t="str">
+        <f t="shared" si="0"/>
+        <v>[56] = {["ID"] = 1879513673; ["TIER"] = 4; }; -- Grodbog-slayer of An Shêru</v>
+      </c>
+      <c r="I57">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+      <c r="J57" t="str">
+        <f t="shared" si="2"/>
+        <v>[56] = {</v>
+      </c>
+      <c r="K57" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513673; </v>
+      </c>
+      <c r="L57" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M57" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N57" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>1879513686</v>
+      </c>
+      <c r="B58" t="s">
+        <v>431</v>
+      </c>
+      <c r="C58">
+        <v>3</v>
+      </c>
+      <c r="H58" t="str">
+        <f t="shared" si="0"/>
+        <v>[57] = {["ID"] = 1879513686; ["TIER"] = 3; }; -- Ordâkhai-bane of An Shêru (Advanced)</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="J58" t="str">
+        <f t="shared" si="2"/>
+        <v>[57] = {</v>
+      </c>
+      <c r="K58" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513686; </v>
+      </c>
+      <c r="L58" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M58" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N58" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>1879513671</v>
+      </c>
+      <c r="B59" t="s">
+        <v>432</v>
+      </c>
+      <c r="C59">
+        <v>4</v>
+      </c>
+      <c r="H59" t="str">
+        <f t="shared" si="0"/>
+        <v>[58] = {["ID"] = 1879513671; ["TIER"] = 4; }; -- Ordâkhai-bane of An Shêru</v>
+      </c>
+      <c r="I59">
+        <f t="shared" si="1"/>
+        <v>58</v>
+      </c>
+      <c r="J59" t="str">
+        <f t="shared" si="2"/>
+        <v>[58] = {</v>
+      </c>
+      <c r="K59" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513671; </v>
+      </c>
+      <c r="L59" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M59" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N59" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>1879513667</v>
+      </c>
+      <c r="B60" t="s">
+        <v>433</v>
+      </c>
+      <c r="C60">
+        <v>3</v>
+      </c>
+      <c r="H60" t="str">
+        <f t="shared" si="0"/>
+        <v>[59] = {["ID"] = 1879513667; ["TIER"] = 3; }; -- Worm-bane of An Shêru (Advanced)</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="1"/>
+        <v>59</v>
+      </c>
+      <c r="J60" t="str">
+        <f t="shared" si="2"/>
+        <v>[59] = {</v>
+      </c>
+      <c r="K60" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513667; </v>
+      </c>
+      <c r="L60" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M60" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N60" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>1879513684</v>
+      </c>
+      <c r="B61" t="s">
+        <v>434</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+      <c r="H61" t="str">
+        <f t="shared" si="0"/>
+        <v>[60] = {["ID"] = 1879513684; ["TIER"] = 4; }; -- Worm-bane of An Shêru</v>
+      </c>
+      <c r="I61">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" si="2"/>
+        <v>[60] = {</v>
+      </c>
+      <c r="K61" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513684; </v>
+      </c>
+      <c r="L61" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M61" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N61" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>1879513786</v>
+      </c>
+      <c r="B62" t="s">
+        <v>435</v>
+      </c>
+      <c r="C62">
+        <v>2</v>
+      </c>
+      <c r="H62" t="str">
+        <f t="shared" si="0"/>
+        <v>[61] = {["ID"] = 1879513786; ["TIER"] = 2; }; -- Tales of An Shêru</v>
+      </c>
+      <c r="I62">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="J62" t="str">
+        <f t="shared" si="2"/>
+        <v>[61] = {</v>
+      </c>
+      <c r="K62" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513786; </v>
+      </c>
+      <c r="L62" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M62" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N62" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B63" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>340</v>
+      </c>
+      <c r="H63" t="str">
+        <f t="shared" si="0"/>
+        <v>[62] = {["CAT_ID"] = 340; ["TIER"] = 1; }; -- Idagâl</v>
+      </c>
+      <c r="I63">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="J63" t="str">
+        <f t="shared" si="2"/>
+        <v>[62] = {</v>
+      </c>
+      <c r="K63" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve">["CAT_ID"] = 340; </v>
+      </c>
+      <c r="M63" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N63" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>1879513783</v>
+      </c>
+      <c r="B64" t="s">
+        <v>436</v>
+      </c>
+      <c r="C64">
+        <v>1</v>
+      </c>
+      <c r="H64" t="str">
+        <f t="shared" si="0"/>
+        <v>[63] = {["ID"] = 1879513783; ["TIER"] = 1; }; -- Renewer of Idagâl</v>
+      </c>
+      <c r="I64">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="J64" t="str">
+        <f t="shared" si="2"/>
+        <v>[63] = {</v>
+      </c>
+      <c r="K64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513783; </v>
+      </c>
+      <c r="L64" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M64" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N64" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>1879513784</v>
+      </c>
+      <c r="B65" t="s">
+        <v>437</v>
+      </c>
+      <c r="C65">
+        <v>2</v>
+      </c>
+      <c r="H65" t="str">
+        <f t="shared" si="0"/>
+        <v>[64] = {["ID"] = 1879513784; ["TIER"] = 2; }; -- Explorer of Idagâl</v>
+      </c>
+      <c r="I65">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+      <c r="J65" t="str">
+        <f t="shared" si="2"/>
+        <v>[64] = {</v>
+      </c>
+      <c r="K65" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513784; </v>
+      </c>
+      <c r="L65" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M65" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N65" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>1879513793</v>
+      </c>
+      <c r="B66" t="s">
+        <v>438</v>
+      </c>
+      <c r="C66">
+        <v>3</v>
+      </c>
+      <c r="H66" t="str">
+        <f t="shared" si="0"/>
+        <v>[65] = {["ID"] = 1879513793; ["TIER"] = 3; }; -- New Threats in Idagâl</v>
+      </c>
+      <c r="I66">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="J66" t="str">
+        <f t="shared" si="2"/>
+        <v>[65] = {</v>
+      </c>
+      <c r="K66" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513793; </v>
+      </c>
+      <c r="L66" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M66" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N66" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>1879513776</v>
+      </c>
+      <c r="B67" t="s">
+        <v>439</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="H67" t="str">
+        <f t="shared" ref="H67:H103" si="8">CONCATENATE(J67,K67,L67,M67,N67," -- ",B67)</f>
+        <v>[66] = {["ID"] = 1879513776; ["TIER"] = 3; }; -- Reclaiming Idagâl</v>
+      </c>
+      <c r="I67">
+        <f t="shared" ref="I67:I103" si="9">ROW()-1</f>
+        <v>66</v>
+      </c>
+      <c r="J67" t="str">
+        <f t="shared" ref="J67:J103" si="10">CONCATENATE(REPT(" ",2-LEN(I67)),"[",I67,"] = {")</f>
+        <v>[66] = {</v>
+      </c>
+      <c r="K67" t="str">
+        <f t="shared" ref="K67:K103" si="11">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
+        <v xml:space="preserve">["ID"] = 1879513776; </v>
+      </c>
+      <c r="L67" t="str">
+        <f t="shared" ref="L67:L103" si="12">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
+        <v/>
+      </c>
+      <c r="M67" t="str">
+        <f t="shared" ref="M67:M103" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N67" t="str">
+        <f t="shared" ref="N67:N103" si="14">CONCATENATE("};")</f>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>1879513699</v>
+      </c>
+      <c r="B68" t="s">
+        <v>440</v>
+      </c>
+      <c r="C68">
+        <v>3</v>
+      </c>
+      <c r="H68" t="str">
+        <f t="shared" si="8"/>
+        <v>[67] = {["ID"] = 1879513699; ["TIER"] = 3; }; -- Treasure-seeker of Idagâl</v>
+      </c>
+      <c r="I68">
+        <f t="shared" si="9"/>
+        <v>67</v>
+      </c>
+      <c r="J68" t="str">
+        <f t="shared" si="10"/>
+        <v>[67] = {</v>
+      </c>
+      <c r="K68" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513699; </v>
+      </c>
+      <c r="L68" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M68" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N68" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>1879513700</v>
+      </c>
+      <c r="B69" t="s">
+        <v>441</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="H69" t="str">
+        <f t="shared" si="8"/>
+        <v>[68] = {["ID"] = 1879513700; ["TIER"] = 2; }; -- Slayer of Idagâl</v>
+      </c>
+      <c r="I69">
+        <f t="shared" si="9"/>
+        <v>68</v>
+      </c>
+      <c r="J69" t="str">
+        <f t="shared" si="10"/>
+        <v>[68] = {</v>
+      </c>
+      <c r="K69" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513700; </v>
+      </c>
+      <c r="L69" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M69" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N69" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>1879513670</v>
+      </c>
+      <c r="B70" t="s">
+        <v>442</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="H70" t="str">
+        <f t="shared" si="8"/>
+        <v>[69] = {["ID"] = 1879513670; ["TIER"] = 3; }; -- Brigand-bane of Idagâl (Advanced)</v>
+      </c>
+      <c r="I70">
+        <f t="shared" si="9"/>
+        <v>69</v>
+      </c>
+      <c r="J70" t="str">
+        <f t="shared" si="10"/>
+        <v>[69] = {</v>
+      </c>
+      <c r="K70" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513670; </v>
+      </c>
+      <c r="L70" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M70" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N70" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>1879513680</v>
+      </c>
+      <c r="B71" t="s">
+        <v>443</v>
+      </c>
+      <c r="C71">
+        <v>4</v>
+      </c>
+      <c r="H71" t="str">
+        <f t="shared" si="8"/>
+        <v>[70] = {["ID"] = 1879513680; ["TIER"] = 4; }; -- Brigand-bane of Idagâl</v>
+      </c>
+      <c r="I71">
+        <f t="shared" si="9"/>
+        <v>70</v>
+      </c>
+      <c r="J71" t="str">
+        <f t="shared" si="10"/>
+        <v>[70] = {</v>
+      </c>
+      <c r="K71" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513680; </v>
+      </c>
+      <c r="L71" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M71" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N71" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>1879513683</v>
+      </c>
+      <c r="B72" t="s">
+        <v>444</v>
+      </c>
+      <c r="C72">
+        <v>3</v>
+      </c>
+      <c r="H72" t="str">
+        <f t="shared" si="8"/>
+        <v>[71] = {["ID"] = 1879513683; ["TIER"] = 3; }; -- Cobra-slayer of Idagâl (Advanced)</v>
+      </c>
+      <c r="I72">
+        <f t="shared" si="9"/>
+        <v>71</v>
+      </c>
+      <c r="J72" t="str">
+        <f t="shared" si="10"/>
+        <v>[71] = {</v>
+      </c>
+      <c r="K72" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513683; </v>
+      </c>
+      <c r="L72" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M72" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N72" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>1879513676</v>
+      </c>
+      <c r="B73" t="s">
+        <v>445</v>
+      </c>
+      <c r="C73">
+        <v>4</v>
+      </c>
+      <c r="H73" t="str">
+        <f t="shared" si="8"/>
+        <v>[72] = {["ID"] = 1879513676; ["TIER"] = 4; }; -- Cobra-slayer of Idagâl</v>
+      </c>
+      <c r="I73">
+        <f t="shared" si="9"/>
+        <v>72</v>
+      </c>
+      <c r="J73" t="str">
+        <f t="shared" si="10"/>
+        <v>[72] = {</v>
+      </c>
+      <c r="K73" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513676; </v>
+      </c>
+      <c r="L73" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M73" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N73" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>1879513672</v>
+      </c>
+      <c r="B74" t="s">
+        <v>446</v>
+      </c>
+      <c r="C74">
+        <v>3</v>
+      </c>
+      <c r="H74" t="str">
+        <f t="shared" si="8"/>
+        <v>[73] = {["ID"] = 1879513672; ["TIER"] = 3; }; -- Drake-slayer of Idagâl (Advanced)</v>
+      </c>
+      <c r="I74">
+        <f t="shared" si="9"/>
+        <v>73</v>
+      </c>
+      <c r="J74" t="str">
+        <f t="shared" si="10"/>
+        <v>[73] = {</v>
+      </c>
+      <c r="K74" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513672; </v>
+      </c>
+      <c r="L74" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M74" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N74" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>1879513685</v>
+      </c>
+      <c r="B75" t="s">
+        <v>447</v>
+      </c>
+      <c r="C75">
+        <v>4</v>
+      </c>
+      <c r="H75" t="str">
+        <f t="shared" si="8"/>
+        <v>[74] = {["ID"] = 1879513685; ["TIER"] = 4; }; -- Drake-slayer of Idagâl</v>
+      </c>
+      <c r="I75">
+        <f t="shared" si="9"/>
+        <v>74</v>
+      </c>
+      <c r="J75" t="str">
+        <f t="shared" si="10"/>
+        <v>[74] = {</v>
+      </c>
+      <c r="K75" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513685; </v>
+      </c>
+      <c r="L75" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M75" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N75" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>1879513675</v>
+      </c>
+      <c r="B76" t="s">
+        <v>448</v>
+      </c>
+      <c r="C76">
+        <v>3</v>
+      </c>
+      <c r="H76" t="str">
+        <f t="shared" si="8"/>
+        <v>[75] = {["ID"] = 1879513675; ["TIER"] = 3; }; -- Utûgi-bane of Idagâl (Advanced)</v>
+      </c>
+      <c r="I76">
+        <f t="shared" si="9"/>
+        <v>75</v>
+      </c>
+      <c r="J76" t="str">
+        <f t="shared" si="10"/>
+        <v>[75] = {</v>
+      </c>
+      <c r="K76" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513675; </v>
+      </c>
+      <c r="L76" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M76" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N76" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>1879513687</v>
+      </c>
+      <c r="B77" t="s">
+        <v>449</v>
+      </c>
+      <c r="C77">
+        <v>4</v>
+      </c>
+      <c r="H77" t="str">
+        <f t="shared" si="8"/>
+        <v>[76] = {["ID"] = 1879513687; ["TIER"] = 4; }; -- Utûgi-bane of Idagâl</v>
+      </c>
+      <c r="I77">
+        <f t="shared" si="9"/>
+        <v>76</v>
+      </c>
+      <c r="J77" t="str">
+        <f t="shared" si="10"/>
+        <v>[76] = {</v>
+      </c>
+      <c r="K77" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513687; </v>
+      </c>
+      <c r="L77" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M77" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N77" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>1879513677</v>
+      </c>
+      <c r="B78" t="s">
+        <v>450</v>
+      </c>
+      <c r="C78">
+        <v>3</v>
+      </c>
+      <c r="H78" t="str">
+        <f t="shared" si="8"/>
+        <v>[77] = {["ID"] = 1879513677; ["TIER"] = 3; }; -- Kergrim-slayer of Idagâl (Advanced)</v>
+      </c>
+      <c r="I78">
+        <f t="shared" si="9"/>
+        <v>77</v>
+      </c>
+      <c r="J78" t="str">
+        <f t="shared" si="10"/>
+        <v>[77] = {</v>
+      </c>
+      <c r="K78" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513677; </v>
+      </c>
+      <c r="L78" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M78" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N78" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>1879513678</v>
+      </c>
+      <c r="B79" t="s">
+        <v>451</v>
+      </c>
+      <c r="C79">
+        <v>4</v>
+      </c>
+      <c r="H79" t="str">
+        <f t="shared" si="8"/>
+        <v>[78] = {["ID"] = 1879513678; ["TIER"] = 4; }; -- Kergrim-slayer of Idagâl</v>
+      </c>
+      <c r="I79">
+        <f t="shared" si="9"/>
+        <v>78</v>
+      </c>
+      <c r="J79" t="str">
+        <f t="shared" si="10"/>
+        <v>[78] = {</v>
+      </c>
+      <c r="K79" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513678; </v>
+      </c>
+      <c r="L79" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M79" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N79" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>1879513679</v>
+      </c>
+      <c r="B80" t="s">
+        <v>452</v>
+      </c>
+      <c r="C80">
+        <v>3</v>
+      </c>
+      <c r="H80" t="str">
+        <f t="shared" si="8"/>
+        <v>[79] = {["ID"] = 1879513679; ["TIER"] = 3; }; -- Ordâkhai-bane of Idagâl (Advanced)</v>
+      </c>
+      <c r="I80">
+        <f t="shared" si="9"/>
+        <v>79</v>
+      </c>
+      <c r="J80" t="str">
+        <f t="shared" si="10"/>
+        <v>[79] = {</v>
+      </c>
+      <c r="K80" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513679; </v>
+      </c>
+      <c r="L80" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M80" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N80" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>1879513666</v>
+      </c>
+      <c r="B81" t="s">
+        <v>453</v>
+      </c>
+      <c r="C81">
+        <v>4</v>
+      </c>
+      <c r="H81" t="str">
+        <f t="shared" si="8"/>
+        <v>[80] = {["ID"] = 1879513666; ["TIER"] = 4; }; -- Ordâkhai-bane of Idagâl</v>
+      </c>
+      <c r="I81">
+        <f t="shared" si="9"/>
+        <v>80</v>
+      </c>
+      <c r="J81" t="str">
+        <f t="shared" si="10"/>
+        <v>[80] = {</v>
+      </c>
+      <c r="K81" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513666; </v>
+      </c>
+      <c r="L81" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M81" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N81" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>1879513777</v>
+      </c>
+      <c r="B82" t="s">
+        <v>454</v>
+      </c>
+      <c r="C82">
+        <v>2</v>
+      </c>
+      <c r="H82" t="str">
+        <f t="shared" si="8"/>
+        <v>[81] = {["ID"] = 1879513777; ["TIER"] = 2; }; -- Tales of Idagâl</v>
+      </c>
+      <c r="I82">
+        <f t="shared" si="9"/>
+        <v>81</v>
+      </c>
+      <c r="J82" t="str">
+        <f t="shared" si="10"/>
+        <v>[81] = {</v>
+      </c>
+      <c r="K82" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513777; </v>
+      </c>
+      <c r="L82" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M82" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N82" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B83" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D83">
+        <v>341</v>
+      </c>
+      <c r="H83" t="str">
+        <f t="shared" si="8"/>
+        <v>[82] = {["CAT_ID"] = 341; }; -- Mûr Ghala</v>
+      </c>
+      <c r="I83">
+        <f t="shared" si="9"/>
+        <v>82</v>
+      </c>
+      <c r="J83" t="str">
+        <f t="shared" si="10"/>
+        <v>[82] = {</v>
+      </c>
+      <c r="K83" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L83" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">["CAT_ID"] = 341; </v>
+      </c>
+      <c r="M83" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N83" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>1879514041</v>
+      </c>
+      <c r="B84" t="s">
+        <v>460</v>
+      </c>
+      <c r="H84" t="str">
+        <f t="shared" si="8"/>
+        <v>[83] = {["ID"] = 1879514041; }; -- Hunter of Mûr Ghala</v>
+      </c>
+      <c r="I84">
+        <f t="shared" si="9"/>
+        <v>83</v>
+      </c>
+      <c r="J84" t="str">
+        <f t="shared" si="10"/>
+        <v>[83] = {</v>
+      </c>
+      <c r="K84" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514041; </v>
+      </c>
+      <c r="L84" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M84" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N84" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>1879514045</v>
+      </c>
+      <c r="B85" t="s">
+        <v>461</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="H85" t="str">
+        <f t="shared" si="8"/>
+        <v>[84] = {["ID"] = 1879514045; ["TIER"] = 1; }; -- Adversaries of Adagím</v>
+      </c>
+      <c r="I85">
+        <f t="shared" si="9"/>
+        <v>84</v>
+      </c>
+      <c r="J85" t="str">
+        <f t="shared" si="10"/>
+        <v>[84] = {</v>
+      </c>
+      <c r="K85" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514045; </v>
+      </c>
+      <c r="L85" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M85" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N85" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>1879514044</v>
+      </c>
+      <c r="B86" t="s">
+        <v>462</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="H86" t="str">
+        <f t="shared" si="8"/>
+        <v>[85] = {["ID"] = 1879514044; ["TIER"] = 1; }; -- Combatants of Kighân</v>
+      </c>
+      <c r="I86">
+        <f t="shared" si="9"/>
+        <v>85</v>
+      </c>
+      <c r="J86" t="str">
+        <f t="shared" si="10"/>
+        <v>[85] = {</v>
+      </c>
+      <c r="K86" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514044; </v>
+      </c>
+      <c r="L86" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M86" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N86" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>1879514039</v>
+      </c>
+      <c r="B87" t="s">
+        <v>463</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="H87" t="str">
+        <f t="shared" si="8"/>
+        <v>[86] = {["ID"] = 1879514039; ["TIER"] = 1; }; -- Enemies of An Shêru</v>
+      </c>
+      <c r="I87">
+        <f t="shared" si="9"/>
+        <v>86</v>
+      </c>
+      <c r="J87" t="str">
+        <f t="shared" si="10"/>
+        <v>[86] = {</v>
+      </c>
+      <c r="K87" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514039; </v>
+      </c>
+      <c r="L87" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M87" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N87" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>1879514047</v>
+      </c>
+      <c r="B88" t="s">
+        <v>464</v>
+      </c>
+      <c r="C88">
+        <v>1</v>
+      </c>
+      <c r="H88" t="str">
+        <f t="shared" si="8"/>
+        <v>[87] = {["ID"] = 1879514047; ["TIER"] = 1; }; -- Invaders of Idagâl</v>
+      </c>
+      <c r="I88">
+        <f t="shared" si="9"/>
+        <v>87</v>
+      </c>
+      <c r="J88" t="str">
+        <f t="shared" si="10"/>
+        <v>[87] = {</v>
+      </c>
+      <c r="K88" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514047; </v>
+      </c>
+      <c r="L88" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M88" t="str">
+        <f t="shared" si="13"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N88" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>1879514046</v>
+      </c>
+      <c r="B89" t="s">
+        <v>473</v>
+      </c>
+      <c r="H89" t="str">
+        <f t="shared" si="8"/>
+        <v>[88] = {["ID"] = 1879514046; }; -- Defender of Adagím</v>
+      </c>
+      <c r="I89">
+        <f t="shared" si="9"/>
+        <v>88</v>
+      </c>
+      <c r="J89" t="str">
+        <f t="shared" si="10"/>
+        <v>[88] = {</v>
+      </c>
+      <c r="K89" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514046; </v>
+      </c>
+      <c r="L89" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M89" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N89" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>1879514040</v>
+      </c>
+      <c r="B90" t="s">
+        <v>474</v>
+      </c>
+      <c r="H90" t="str">
+        <f t="shared" si="8"/>
+        <v>[89] = {["ID"] = 1879514040; }; -- Defender of Kighân</v>
+      </c>
+      <c r="I90">
+        <f t="shared" si="9"/>
+        <v>89</v>
+      </c>
+      <c r="J90" t="str">
+        <f t="shared" si="10"/>
+        <v>[89] = {</v>
+      </c>
+      <c r="K90" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514040; </v>
+      </c>
+      <c r="L90" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M90" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N90" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>1879514042</v>
+      </c>
+      <c r="B91" t="s">
+        <v>475</v>
+      </c>
+      <c r="H91" t="str">
+        <f t="shared" si="8"/>
+        <v>[90] = {["ID"] = 1879514042; }; -- Defender of An Shêru</v>
+      </c>
+      <c r="I91">
+        <f t="shared" si="9"/>
+        <v>90</v>
+      </c>
+      <c r="J91" t="str">
+        <f t="shared" si="10"/>
+        <v>[90] = {</v>
+      </c>
+      <c r="K91" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514042; </v>
+      </c>
+      <c r="L91" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M91" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N91" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>1879514043</v>
+      </c>
+      <c r="B92" t="s">
+        <v>476</v>
+      </c>
+      <c r="H92" t="str">
+        <f t="shared" si="8"/>
+        <v>[91] = {["ID"] = 1879514043; }; -- Defender of Idagâl</v>
+      </c>
+      <c r="I92">
+        <f t="shared" si="9"/>
+        <v>91</v>
+      </c>
+      <c r="J92" t="str">
+        <f t="shared" si="10"/>
+        <v>[91] = {</v>
+      </c>
+      <c r="K92" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879514043; </v>
+      </c>
+      <c r="L92" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M92" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N92" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>1879513808</v>
+      </c>
+      <c r="B93" t="s">
+        <v>472</v>
+      </c>
+      <c r="H93" t="str">
+        <f t="shared" si="8"/>
+        <v>[92] = {["ID"] = 1879513808; }; -- Explorer of Mûr Ghala</v>
+      </c>
+      <c r="I93">
+        <f t="shared" si="9"/>
+        <v>92</v>
+      </c>
+      <c r="J93" t="str">
+        <f t="shared" si="10"/>
+        <v>[92] = {</v>
+      </c>
+      <c r="K93" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513808; </v>
+      </c>
+      <c r="L93" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M93" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N93" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>1879513705</v>
+      </c>
+      <c r="B94" t="s">
+        <v>470</v>
+      </c>
+      <c r="H94" t="str">
+        <f t="shared" si="8"/>
+        <v>[93] = {["ID"] = 1879513705; }; -- Treasure-seeker of Mûr Ghala</v>
+      </c>
+      <c r="I94">
+        <f t="shared" si="9"/>
+        <v>93</v>
+      </c>
+      <c r="J94" t="str">
+        <f t="shared" si="10"/>
+        <v>[93] = {</v>
+      </c>
+      <c r="K94" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513705; </v>
+      </c>
+      <c r="L94" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M94" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N94" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>1879513698</v>
+      </c>
+      <c r="B95" t="s">
+        <v>468</v>
+      </c>
+      <c r="H95" t="str">
+        <f t="shared" si="8"/>
+        <v>[94] = {["ID"] = 1879513698; }; -- Slayer of Mûr Ghala</v>
+      </c>
+      <c r="I95">
+        <f t="shared" si="9"/>
+        <v>94</v>
+      </c>
+      <c r="J95" t="str">
+        <f t="shared" si="10"/>
+        <v>[94] = {</v>
+      </c>
+      <c r="K95" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513698; </v>
+      </c>
+      <c r="L95" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M95" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N95" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>1879513807</v>
+      </c>
+      <c r="B96" t="s">
+        <v>471</v>
+      </c>
+      <c r="H96" t="str">
+        <f t="shared" si="8"/>
+        <v>[95] = {["ID"] = 1879513807; }; -- Tales of Mûr Ghala</v>
+      </c>
+      <c r="I96">
+        <f t="shared" si="9"/>
+        <v>95</v>
+      </c>
+      <c r="J96" t="str">
+        <f t="shared" si="10"/>
+        <v>[95] = {</v>
+      </c>
+      <c r="K96" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513807; </v>
+      </c>
+      <c r="L96" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M96" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N96" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>1879513694</v>
+      </c>
+      <c r="B97" t="s">
+        <v>465</v>
+      </c>
+      <c r="H97" t="str">
+        <f t="shared" si="8"/>
+        <v>[96] = {["ID"] = 1879513694; }; -- Brigand-bane of Mûr Ghala</v>
+      </c>
+      <c r="I97">
+        <f t="shared" si="9"/>
+        <v>96</v>
+      </c>
+      <c r="J97" t="str">
+        <f t="shared" si="10"/>
+        <v>[96] = {</v>
+      </c>
+      <c r="K97" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513694; </v>
+      </c>
+      <c r="L97" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M97" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N97" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>1879513695</v>
+      </c>
+      <c r="B98" t="s">
+        <v>466</v>
+      </c>
+      <c r="H98" t="str">
+        <f t="shared" si="8"/>
+        <v>[97] = {["ID"] = 1879513695; }; -- Nightmare of the Ordâkhai</v>
+      </c>
+      <c r="I98">
+        <f t="shared" si="9"/>
+        <v>97</v>
+      </c>
+      <c r="J98" t="str">
+        <f t="shared" si="10"/>
+        <v>[97] = {</v>
+      </c>
+      <c r="K98" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513695; </v>
+      </c>
+      <c r="L98" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M98" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N98" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>1879513696</v>
+      </c>
+      <c r="B99" t="s">
+        <v>467</v>
+      </c>
+      <c r="H99" t="str">
+        <f t="shared" si="8"/>
+        <v>[98] = {["ID"] = 1879513696; }; -- Spider-slayer of Mûr Ghala</v>
+      </c>
+      <c r="I99">
+        <f t="shared" si="9"/>
+        <v>98</v>
+      </c>
+      <c r="J99" t="str">
+        <f t="shared" si="10"/>
+        <v>[98] = {</v>
+      </c>
+      <c r="K99" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513696; </v>
+      </c>
+      <c r="L99" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M99" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N99" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>1879513703</v>
+      </c>
+      <c r="B100" t="s">
+        <v>469</v>
+      </c>
+      <c r="H100" t="str">
+        <f t="shared" si="8"/>
+        <v>[99] = {["ID"] = 1879513703; }; -- Orc-slayer of Mûr Ghala</v>
+      </c>
+      <c r="I100">
+        <f t="shared" si="9"/>
+        <v>99</v>
+      </c>
+      <c r="J100" t="str">
+        <f t="shared" si="10"/>
+        <v>[99] = {</v>
+      </c>
+      <c r="K100" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513703; </v>
+      </c>
+      <c r="L100" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M100" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N100" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H101" t="e">
+        <f t="shared" si="8"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I101">
+        <f t="shared" si="9"/>
+        <v>100</v>
+      </c>
+      <c r="J101" t="e">
+        <f t="shared" si="10"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K101" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L101" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M101" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N101" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H102" t="e">
+        <f t="shared" si="8"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I102">
+        <f t="shared" si="9"/>
+        <v>101</v>
+      </c>
+      <c r="J102" t="e">
+        <f t="shared" si="10"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K102" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L102" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M102" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N102" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H103" t="e">
+        <f t="shared" si="8"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I103">
+        <f t="shared" si="9"/>
+        <v>102</v>
+      </c>
+      <c r="J103" t="e">
+        <f t="shared" si="10"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K103" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L103" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M103" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N103" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8910B2F7-82CE-4F8E-A600-0933F0B541F5}">
   <dimension ref="A1:B77"/>

</xml_diff>

<commit_message>
Added new deeds: Conqueror of the Legion of Lhaereth, PvMP season 6, Spring Festival pies, Persistent Defenders
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
+++ b/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F472B9-C877-4EBE-BBB3-9E792CFC15AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9A3386-751D-4CCE-8841-432ABFA6536B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="870" windowWidth="21285" windowHeight="14325" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="481">
   <si>
     <t>TIER</t>
   </si>
@@ -1477,6 +1477,18 @@
   </si>
   <si>
     <t>Defender of Idagâl</t>
+  </si>
+  <si>
+    <t>Persistent Defender of Adagím</t>
+  </si>
+  <si>
+    <t>Persistent Defender of Kighân</t>
+  </si>
+  <si>
+    <t>Persistent Defender of An Shêru</t>
+  </si>
+  <si>
+    <t>Persistent Defender of Idagâl</t>
   </si>
 </sst>
 </file>
@@ -5930,7 +5942,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D727EC7-6195-47C5-8CEB-067AA7EF5F9D}">
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -5995,15 +6007,15 @@
       </c>
       <c r="H2" t="str">
         <f>CONCATENATE(J2,K2,L2,M2,N2," -- ",B2)</f>
-        <v xml:space="preserve"> [1] = {["ID"] = 1879513802; }; -- Rejuvenator of Mûr Ghala</v>
+        <v xml:space="preserve">  [1] = {["ID"] = 1879513802; }; -- Rejuvenator of Mûr Ghala</v>
       </c>
       <c r="I2">
         <f>ROW()-1</f>
         <v>1</v>
       </c>
       <c r="J2" t="str">
-        <f>CONCATENATE(REPT(" ",2-LEN(I2)),"[",I2,"] = {")</f>
-        <v xml:space="preserve"> [1] = {</v>
+        <f>CONCATENATE(REPT(" ",3-LEN(I2)),"[",I2,"] = {")</f>
+        <v xml:space="preserve">  [1] = {</v>
       </c>
       <c r="K2" t="str">
         <f>IF(LEN(A2)&gt;0,CONCATENATE("[""ID""] = ",A2,"; "),"")</f>
@@ -6034,15 +6046,15 @@
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H66" si="0">CONCATENATE(J3,K3,L3,M3,N3," -- ",B3)</f>
-        <v xml:space="preserve"> [2] = {["CAT_ID"] = 337; ["TIER"] = 1; }; -- Adagím</v>
+        <v xml:space="preserve">  [2] = {["CAT_ID"] = 337; ["TIER"] = 1; }; -- Adagím</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I66" si="1">ROW()-1</f>
         <v>2</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J3:J66" si="2">CONCATENATE(REPT(" ",2-LEN(I3)),"[",I3,"] = {")</f>
-        <v xml:space="preserve"> [2] = {</v>
+        <f t="shared" ref="J3:J66" si="2">CONCATENATE(REPT(" ",3-LEN(I3)),"[",I3,"] = {")</f>
+        <v xml:space="preserve">  [2] = {</v>
       </c>
       <c r="K3" t="str">
         <f t="shared" ref="K3:K66" si="3">IF(LEN(A3)&gt;0,CONCATENATE("[""ID""] = ",A3,"; "),"")</f>
@@ -6072,12 +6084,12 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <f t="shared" ref="G4:G41" si="7">IF(AND(A4&gt;0,C4&gt;0),CONCATENATE("[",A4,"] = ",C4,", // ",B4),"")</f>
+        <f t="shared" ref="G4:G42" si="7">IF(AND(A4&gt;0,C4&gt;0),CONCATENATE("[",A4,"] = ",C4,", // ",B4),"")</f>
         <v>[1879513774] = 1, // Renewing Adagím</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [3] = {["ID"] = 1879513774; ["TIER"] = 1; }; -- Renewing Adagím</v>
+        <v xml:space="preserve">  [3] = {["ID"] = 1879513774; ["TIER"] = 1; }; -- Renewing Adagím</v>
       </c>
       <c r="I4">
         <f t="shared" si="1"/>
@@ -6085,7 +6097,7 @@
       </c>
       <c r="J4" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [3] = {</v>
+        <v xml:space="preserve">  [3] = {</v>
       </c>
       <c r="K4" t="str">
         <f t="shared" si="3"/>
@@ -6120,7 +6132,7 @@
       </c>
       <c r="H5" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [4] = {["ID"] = 1879513785; ["TIER"] = 2; }; -- Exploring Adagím</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879513785; ["TIER"] = 2; }; -- Exploring Adagím</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
@@ -6128,7 +6140,7 @@
       </c>
       <c r="J5" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [4] = {</v>
+        <v xml:space="preserve">  [4] = {</v>
       </c>
       <c r="K5" t="str">
         <f t="shared" si="3"/>
@@ -6163,7 +6175,7 @@
       </c>
       <c r="H6" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [5] = {["ID"] = 1879513778; ["TIER"] = 3; }; -- New Threats in Adagím</v>
+        <v xml:space="preserve">  [5] = {["ID"] = 1879513778; ["TIER"] = 3; }; -- New Threats in Adagím</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
@@ -6171,7 +6183,7 @@
       </c>
       <c r="J6" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [5] = {</v>
+        <v xml:space="preserve">  [5] = {</v>
       </c>
       <c r="K6" t="str">
         <f t="shared" si="3"/>
@@ -6206,7 +6218,7 @@
       </c>
       <c r="H7" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [6] = {["ID"] = 1879513790; ["TIER"] = 3; }; -- Scouting Adagím</v>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879513790; ["TIER"] = 3; }; -- Scouting Adagím</v>
       </c>
       <c r="I7">
         <f t="shared" si="1"/>
@@ -6214,7 +6226,7 @@
       </c>
       <c r="J7" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [6] = {</v>
+        <v xml:space="preserve">  [6] = {</v>
       </c>
       <c r="K7" t="str">
         <f t="shared" si="3"/>
@@ -6249,7 +6261,7 @@
       </c>
       <c r="H8" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [7] = {["ID"] = 1879513702; ["TIER"] = 3; }; -- Treasure-seeker of Adagím</v>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879513702; ["TIER"] = 3; }; -- Treasure-seeker of Adagím</v>
       </c>
       <c r="I8">
         <f t="shared" si="1"/>
@@ -6257,7 +6269,7 @@
       </c>
       <c r="J8" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [7] = {</v>
+        <v xml:space="preserve">  [7] = {</v>
       </c>
       <c r="K8" t="str">
         <f t="shared" si="3"/>
@@ -6292,7 +6304,7 @@
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [8] = {["ID"] = 1879513704; ["TIER"] = 2; }; -- Slayer of Adagím</v>
+        <v xml:space="preserve">  [8] = {["ID"] = 1879513704; ["TIER"] = 2; }; -- Slayer of Adagím</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
@@ -6300,7 +6312,7 @@
       </c>
       <c r="J9" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [8] = {</v>
+        <v xml:space="preserve">  [8] = {</v>
       </c>
       <c r="K9" t="str">
         <f t="shared" si="3"/>
@@ -6335,7 +6347,7 @@
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> [9] = {["ID"] = 1879513641; ["TIER"] = 3; }; -- Bog-slayer of Adagím (Advanced)</v>
+        <v xml:space="preserve">  [9] = {["ID"] = 1879513641; ["TIER"] = 3; }; -- Bog-slayer of Adagím (Advanced)</v>
       </c>
       <c r="I10">
         <f t="shared" si="1"/>
@@ -6343,7 +6355,7 @@
       </c>
       <c r="J10" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> [9] = {</v>
+        <v xml:space="preserve">  [9] = {</v>
       </c>
       <c r="K10" t="str">
         <f t="shared" si="3"/>
@@ -6378,7 +6390,7 @@
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
-        <v>[10] = {["ID"] = 1879513640; ["TIER"] = 4; }; -- Bog-slayer of Adagím</v>
+        <v xml:space="preserve"> [10] = {["ID"] = 1879513640; ["TIER"] = 4; }; -- Bog-slayer of Adagím</v>
       </c>
       <c r="I11">
         <f t="shared" si="1"/>
@@ -6386,7 +6398,7 @@
       </c>
       <c r="J11" t="str">
         <f t="shared" si="2"/>
-        <v>[10] = {</v>
+        <v xml:space="preserve"> [10] = {</v>
       </c>
       <c r="K11" t="str">
         <f t="shared" si="3"/>
@@ -6421,7 +6433,7 @@
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
-        <v>[11] = {["ID"] = 1879513644; ["TIER"] = 3; }; -- Crocodile-slayer of Adagím (Advanced)</v>
+        <v xml:space="preserve"> [11] = {["ID"] = 1879513644; ["TIER"] = 3; }; -- Crocodile-slayer of Adagím (Advanced)</v>
       </c>
       <c r="I12">
         <f t="shared" si="1"/>
@@ -6429,7 +6441,7 @@
       </c>
       <c r="J12" t="str">
         <f t="shared" si="2"/>
-        <v>[11] = {</v>
+        <v xml:space="preserve"> [11] = {</v>
       </c>
       <c r="K12" t="str">
         <f t="shared" si="3"/>
@@ -6464,7 +6476,7 @@
       </c>
       <c r="H13" t="str">
         <f t="shared" si="0"/>
-        <v>[12] = {["ID"] = 1879513647; ["TIER"] = 4; }; -- Crocodile-slayer of Adagím</v>
+        <v xml:space="preserve"> [12] = {["ID"] = 1879513647; ["TIER"] = 4; }; -- Crocodile-slayer of Adagím</v>
       </c>
       <c r="I13">
         <f t="shared" si="1"/>
@@ -6472,7 +6484,7 @@
       </c>
       <c r="J13" t="str">
         <f t="shared" si="2"/>
-        <v>[12] = {</v>
+        <v xml:space="preserve"> [12] = {</v>
       </c>
       <c r="K13" t="str">
         <f t="shared" si="3"/>
@@ -6507,7 +6519,7 @@
       </c>
       <c r="H14" t="str">
         <f t="shared" si="0"/>
-        <v>[13] = {["ID"] = 1879513663; ["TIER"] = 3; }; -- Huorn-bane of Adagím (Advanced)</v>
+        <v xml:space="preserve"> [13] = {["ID"] = 1879513663; ["TIER"] = 3; }; -- Huorn-bane of Adagím (Advanced)</v>
       </c>
       <c r="I14">
         <f t="shared" si="1"/>
@@ -6515,7 +6527,7 @@
       </c>
       <c r="J14" t="str">
         <f t="shared" si="2"/>
-        <v>[13] = {</v>
+        <v xml:space="preserve"> [13] = {</v>
       </c>
       <c r="K14" t="str">
         <f t="shared" si="3"/>
@@ -6550,7 +6562,7 @@
       </c>
       <c r="H15" t="str">
         <f t="shared" si="0"/>
-        <v>[14] = {["ID"] = 1879513664; ["TIER"] = 4; }; -- Huorn-bane of Adagím</v>
+        <v xml:space="preserve"> [14] = {["ID"] = 1879513664; ["TIER"] = 4; }; -- Huorn-bane of Adagím</v>
       </c>
       <c r="I15">
         <f t="shared" si="1"/>
@@ -6558,7 +6570,7 @@
       </c>
       <c r="J15" t="str">
         <f t="shared" si="2"/>
-        <v>[14] = {</v>
+        <v xml:space="preserve"> [14] = {</v>
       </c>
       <c r="K15" t="str">
         <f t="shared" si="3"/>
@@ -6593,7 +6605,7 @@
       </c>
       <c r="H16" t="str">
         <f t="shared" si="0"/>
-        <v>[15] = {["ID"] = 1879513659; ["TIER"] = 3; }; -- Orc-bane of Adagím (Advanced)</v>
+        <v xml:space="preserve"> [15] = {["ID"] = 1879513659; ["TIER"] = 3; }; -- Orc-bane of Adagím (Advanced)</v>
       </c>
       <c r="I16">
         <f t="shared" si="1"/>
@@ -6601,7 +6613,7 @@
       </c>
       <c r="J16" t="str">
         <f t="shared" si="2"/>
-        <v>[15] = {</v>
+        <v xml:space="preserve"> [15] = {</v>
       </c>
       <c r="K16" t="str">
         <f t="shared" si="3"/>
@@ -6636,7 +6648,7 @@
       </c>
       <c r="H17" t="str">
         <f t="shared" si="0"/>
-        <v>[16] = {["ID"] = 1879513653; ["TIER"] = 4; }; -- Orc-bane of Adagím</v>
+        <v xml:space="preserve"> [16] = {["ID"] = 1879513653; ["TIER"] = 4; }; -- Orc-bane of Adagím</v>
       </c>
       <c r="I17">
         <f t="shared" si="1"/>
@@ -6644,7 +6656,7 @@
       </c>
       <c r="J17" t="str">
         <f t="shared" si="2"/>
-        <v>[16] = {</v>
+        <v xml:space="preserve"> [16] = {</v>
       </c>
       <c r="K17" t="str">
         <f t="shared" si="3"/>
@@ -6679,7 +6691,7 @@
       </c>
       <c r="H18" t="str">
         <f t="shared" si="0"/>
-        <v>[17] = {["ID"] = 1879513645; ["TIER"] = 3; }; -- Spider-slayer of Adagím (Advanced)</v>
+        <v xml:space="preserve"> [17] = {["ID"] = 1879513645; ["TIER"] = 3; }; -- Spider-slayer of Adagím (Advanced)</v>
       </c>
       <c r="I18">
         <f t="shared" si="1"/>
@@ -6687,7 +6699,7 @@
       </c>
       <c r="J18" t="str">
         <f t="shared" si="2"/>
-        <v>[17] = {</v>
+        <v xml:space="preserve"> [17] = {</v>
       </c>
       <c r="K18" t="str">
         <f t="shared" si="3"/>
@@ -6722,7 +6734,7 @@
       </c>
       <c r="H19" t="str">
         <f t="shared" si="0"/>
-        <v>[18] = {["ID"] = 1879513651; ["TIER"] = 4; }; -- Spider-slayer of Adagím</v>
+        <v xml:space="preserve"> [18] = {["ID"] = 1879513651; ["TIER"] = 4; }; -- Spider-slayer of Adagím</v>
       </c>
       <c r="I19">
         <f t="shared" si="1"/>
@@ -6730,7 +6742,7 @@
       </c>
       <c r="J19" t="str">
         <f t="shared" si="2"/>
-        <v>[18] = {</v>
+        <v xml:space="preserve"> [18] = {</v>
       </c>
       <c r="K19" t="str">
         <f t="shared" si="3"/>
@@ -6765,7 +6777,7 @@
       </c>
       <c r="H20" t="str">
         <f t="shared" si="0"/>
-        <v>[19] = {["ID"] = 1879513649; ["TIER"] = 3; }; -- Wood-troll Slayer of Adagím (Advanced)</v>
+        <v xml:space="preserve"> [19] = {["ID"] = 1879513649; ["TIER"] = 3; }; -- Wood-troll Slayer of Adagím (Advanced)</v>
       </c>
       <c r="I20">
         <f t="shared" si="1"/>
@@ -6773,7 +6785,7 @@
       </c>
       <c r="J20" t="str">
         <f t="shared" si="2"/>
-        <v>[19] = {</v>
+        <v xml:space="preserve"> [19] = {</v>
       </c>
       <c r="K20" t="str">
         <f t="shared" si="3"/>
@@ -6808,7 +6820,7 @@
       </c>
       <c r="H21" t="str">
         <f t="shared" si="0"/>
-        <v>[20] = {["ID"] = 1879513650; ["TIER"] = 4; }; -- Wood-troll Slayer of Adagím</v>
+        <v xml:space="preserve"> [20] = {["ID"] = 1879513650; ["TIER"] = 4; }; -- Wood-troll Slayer of Adagím</v>
       </c>
       <c r="I21">
         <f t="shared" si="1"/>
@@ -6816,7 +6828,7 @@
       </c>
       <c r="J21" t="str">
         <f t="shared" si="2"/>
-        <v>[20] = {</v>
+        <v xml:space="preserve"> [20] = {</v>
       </c>
       <c r="K21" t="str">
         <f t="shared" si="3"/>
@@ -6851,7 +6863,7 @@
       </c>
       <c r="H22" t="str">
         <f t="shared" si="0"/>
-        <v>[21] = {["ID"] = 1879513791; ["TIER"] = 2; }; -- Tales of Adagím</v>
+        <v xml:space="preserve"> [21] = {["ID"] = 1879513791; ["TIER"] = 2; }; -- Tales of Adagím</v>
       </c>
       <c r="I22">
         <f t="shared" si="1"/>
@@ -6859,7 +6871,7 @@
       </c>
       <c r="J22" t="str">
         <f t="shared" si="2"/>
-        <v>[21] = {</v>
+        <v xml:space="preserve"> [21] = {</v>
       </c>
       <c r="K22" t="str">
         <f t="shared" si="3"/>
@@ -6879,18 +6891,22 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
-        <v>456</v>
+      <c r="A23">
+        <v>1879521611</v>
+      </c>
+      <c r="B23" t="s">
+        <v>477</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
-      <c r="D23">
-        <v>338</v>
+      <c r="G23" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879521611] = 1, // Persistent Defender of Adagím</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="0"/>
-        <v>[22] = {["CAT_ID"] = 338; ["TIER"] = 1; }; -- Kighân</v>
+        <v xml:space="preserve"> [22] = {["ID"] = 1879521611; ["TIER"] = 1; }; -- Persistent Defender of Adagím</v>
       </c>
       <c r="I23">
         <f t="shared" si="1"/>
@@ -6898,15 +6914,15 @@
       </c>
       <c r="J23" t="str">
         <f t="shared" si="2"/>
-        <v>[22] = {</v>
+        <v xml:space="preserve"> [22] = {</v>
       </c>
       <c r="K23" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879521611; </v>
       </c>
       <c r="L23" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">["CAT_ID"] = 338; </v>
+        <v/>
       </c>
       <c r="M23" t="str">
         <f t="shared" si="5"/>
@@ -6918,22 +6934,18 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>1879513787</v>
-      </c>
-      <c r="B24" t="s">
-        <v>398</v>
+      <c r="B24" s="1" t="s">
+        <v>456</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
-      <c r="G24" t="str">
-        <f t="shared" si="7"/>
-        <v>[1879513787] = 1, // Rejuvenator of Kighân</v>
+      <c r="D24">
+        <v>338</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="0"/>
-        <v>[23] = {["ID"] = 1879513787; ["TIER"] = 1; }; -- Rejuvenator of Kighân</v>
+        <v xml:space="preserve"> [23] = {["CAT_ID"] = 338; ["TIER"] = 1; }; -- Kighân</v>
       </c>
       <c r="I24">
         <f t="shared" si="1"/>
@@ -6941,15 +6953,15 @@
       </c>
       <c r="J24" t="str">
         <f t="shared" si="2"/>
-        <v>[23] = {</v>
+        <v xml:space="preserve"> [23] = {</v>
       </c>
       <c r="K24" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513787; </v>
+        <v/>
       </c>
       <c r="L24" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["CAT_ID"] = 338; </v>
       </c>
       <c r="M24" t="str">
         <f t="shared" si="5"/>
@@ -6962,21 +6974,21 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>1879513779</v>
+        <v>1879513787</v>
       </c>
       <c r="B25" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513779] = 2, // Explorer of Kighân</v>
+        <v>[1879513787] = 1, // Rejuvenator of Kighân</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="0"/>
-        <v>[24] = {["ID"] = 1879513779; ["TIER"] = 2; }; -- Explorer of Kighân</v>
+        <v xml:space="preserve"> [24] = {["ID"] = 1879513787; ["TIER"] = 1; }; -- Rejuvenator of Kighân</v>
       </c>
       <c r="I25">
         <f t="shared" si="1"/>
@@ -6984,11 +6996,11 @@
       </c>
       <c r="J25" t="str">
         <f t="shared" si="2"/>
-        <v>[24] = {</v>
+        <v xml:space="preserve"> [24] = {</v>
       </c>
       <c r="K25" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513779; </v>
+        <v xml:space="preserve">["ID"] = 1879513787; </v>
       </c>
       <c r="L25" t="str">
         <f t="shared" si="4"/>
@@ -6996,7 +7008,7 @@
       </c>
       <c r="M25" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N25" t="str">
         <f t="shared" si="6"/>
@@ -7005,21 +7017,21 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>1879513781</v>
+        <v>1879513779</v>
       </c>
       <c r="B26" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513781] = 3, // Dangers in Kighân</v>
+        <v>[1879513779] = 2, // Explorer of Kighân</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="0"/>
-        <v>[25] = {["ID"] = 1879513781; ["TIER"] = 3; }; -- Dangers in Kighân</v>
+        <v xml:space="preserve"> [25] = {["ID"] = 1879513779; ["TIER"] = 2; }; -- Explorer of Kighân</v>
       </c>
       <c r="I26">
         <f t="shared" si="1"/>
@@ -7027,11 +7039,11 @@
       </c>
       <c r="J26" t="str">
         <f t="shared" si="2"/>
-        <v>[25] = {</v>
+        <v xml:space="preserve"> [25] = {</v>
       </c>
       <c r="K26" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513781; </v>
+        <v xml:space="preserve">["ID"] = 1879513779; </v>
       </c>
       <c r="L26" t="str">
         <f t="shared" si="4"/>
@@ -7039,7 +7051,7 @@
       </c>
       <c r="M26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N26" t="str">
         <f t="shared" si="6"/>
@@ -7048,21 +7060,21 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>1879513782</v>
+        <v>1879513781</v>
       </c>
       <c r="B27" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C27">
         <v>3</v>
       </c>
       <c r="G27" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513782] = 3, // Scouting Kighân</v>
+        <v>[1879513781] = 3, // Dangers in Kighân</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" si="0"/>
-        <v>[26] = {["ID"] = 1879513782; ["TIER"] = 3; }; -- Scouting Kighân</v>
+        <v xml:space="preserve"> [26] = {["ID"] = 1879513781; ["TIER"] = 3; }; -- Dangers in Kighân</v>
       </c>
       <c r="I27">
         <f t="shared" si="1"/>
@@ -7070,11 +7082,11 @@
       </c>
       <c r="J27" t="str">
         <f t="shared" si="2"/>
-        <v>[26] = {</v>
+        <v xml:space="preserve"> [26] = {</v>
       </c>
       <c r="K27" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513782; </v>
+        <v xml:space="preserve">["ID"] = 1879513781; </v>
       </c>
       <c r="L27" t="str">
         <f t="shared" si="4"/>
@@ -7091,21 +7103,21 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>1879513701</v>
+        <v>1879513782</v>
       </c>
       <c r="B28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="G28" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513701] = 3, // Treasure-seeker of Kighân</v>
+        <v>[1879513782] = 3, // Scouting Kighân</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="0"/>
-        <v>[27] = {["ID"] = 1879513701; ["TIER"] = 3; }; -- Treasure-seeker of Kighân</v>
+        <v xml:space="preserve"> [27] = {["ID"] = 1879513782; ["TIER"] = 3; }; -- Scouting Kighân</v>
       </c>
       <c r="I28">
         <f t="shared" si="1"/>
@@ -7113,11 +7125,11 @@
       </c>
       <c r="J28" t="str">
         <f t="shared" si="2"/>
-        <v>[27] = {</v>
+        <v xml:space="preserve"> [27] = {</v>
       </c>
       <c r="K28" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513701; </v>
+        <v xml:space="preserve">["ID"] = 1879513782; </v>
       </c>
       <c r="L28" t="str">
         <f t="shared" si="4"/>
@@ -7134,21 +7146,21 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>1879513706</v>
+        <v>1879513701</v>
       </c>
       <c r="B29" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513706] = 2, // Slayer of Kighân</v>
+        <v>[1879513701] = 3, // Treasure-seeker of Kighân</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="0"/>
-        <v>[28] = {["ID"] = 1879513706; ["TIER"] = 2; }; -- Slayer of Kighân</v>
+        <v xml:space="preserve"> [28] = {["ID"] = 1879513701; ["TIER"] = 3; }; -- Treasure-seeker of Kighân</v>
       </c>
       <c r="I29">
         <f t="shared" si="1"/>
@@ -7156,11 +7168,11 @@
       </c>
       <c r="J29" t="str">
         <f t="shared" si="2"/>
-        <v>[28] = {</v>
+        <v xml:space="preserve"> [28] = {</v>
       </c>
       <c r="K29" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513706; </v>
+        <v xml:space="preserve">["ID"] = 1879513701; </v>
       </c>
       <c r="L29" t="str">
         <f t="shared" si="4"/>
@@ -7168,7 +7180,7 @@
       </c>
       <c r="M29" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N29" t="str">
         <f t="shared" si="6"/>
@@ -7177,21 +7189,21 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>1879513660</v>
+        <v>1879513706</v>
       </c>
       <c r="B30" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G30" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513660] = 3, // Tarsâri-bane of Kighân (Advanced)</v>
+        <v>[1879513706] = 2, // Slayer of Kighân</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="0"/>
-        <v>[29] = {["ID"] = 1879513660; ["TIER"] = 3; }; -- Tarsâri-bane of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [29] = {["ID"] = 1879513706; ["TIER"] = 2; }; -- Slayer of Kighân</v>
       </c>
       <c r="I30">
         <f t="shared" si="1"/>
@@ -7199,11 +7211,11 @@
       </c>
       <c r="J30" t="str">
         <f t="shared" si="2"/>
-        <v>[29] = {</v>
+        <v xml:space="preserve"> [29] = {</v>
       </c>
       <c r="K30" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513660; </v>
+        <v xml:space="preserve">["ID"] = 1879513706; </v>
       </c>
       <c r="L30" t="str">
         <f t="shared" si="4"/>
@@ -7211,7 +7223,7 @@
       </c>
       <c r="M30" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N30" t="str">
         <f t="shared" si="6"/>
@@ -7220,21 +7232,21 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>1879513655</v>
+        <v>1879513660</v>
       </c>
       <c r="B31" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G31" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513655] = 4, // Tarsâri-bane of Kighân</v>
+        <v>[1879513660] = 3, // Tarsâri-bane of Kighân (Advanced)</v>
       </c>
       <c r="H31" t="str">
         <f t="shared" si="0"/>
-        <v>[30] = {["ID"] = 1879513655; ["TIER"] = 4; }; -- Tarsâri-bane of Kighân</v>
+        <v xml:space="preserve"> [30] = {["ID"] = 1879513660; ["TIER"] = 3; }; -- Tarsâri-bane of Kighân (Advanced)</v>
       </c>
       <c r="I31">
         <f t="shared" si="1"/>
@@ -7242,11 +7254,11 @@
       </c>
       <c r="J31" t="str">
         <f t="shared" si="2"/>
-        <v>[30] = {</v>
+        <v xml:space="preserve"> [30] = {</v>
       </c>
       <c r="K31" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513655; </v>
+        <v xml:space="preserve">["ID"] = 1879513660; </v>
       </c>
       <c r="L31" t="str">
         <f t="shared" si="4"/>
@@ -7254,7 +7266,7 @@
       </c>
       <c r="M31" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N31" t="str">
         <f t="shared" si="6"/>
@@ -7263,21 +7275,21 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>1879513656</v>
+        <v>1879513655</v>
       </c>
       <c r="B32" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513656] = 3, // Bee-slayer of Kighân (Advanced)</v>
+        <v>[1879513655] = 4, // Tarsâri-bane of Kighân</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="0"/>
-        <v>[31] = {["ID"] = 1879513656; ["TIER"] = 3; }; -- Bee-slayer of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [31] = {["ID"] = 1879513655; ["TIER"] = 4; }; -- Tarsâri-bane of Kighân</v>
       </c>
       <c r="I32">
         <f t="shared" si="1"/>
@@ -7285,11 +7297,11 @@
       </c>
       <c r="J32" t="str">
         <f t="shared" si="2"/>
-        <v>[31] = {</v>
+        <v xml:space="preserve"> [31] = {</v>
       </c>
       <c r="K32" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513656; </v>
+        <v xml:space="preserve">["ID"] = 1879513655; </v>
       </c>
       <c r="L32" t="str">
         <f t="shared" si="4"/>
@@ -7297,7 +7309,7 @@
       </c>
       <c r="M32" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N32" t="str">
         <f t="shared" si="6"/>
@@ -7306,21 +7318,21 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>1879513654</v>
+        <v>1879513656</v>
       </c>
       <c r="B33" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C33">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G33" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513654] = 4, // Bee-slayer of Kighân</v>
+        <v>[1879513656] = 3, // Bee-slayer of Kighân (Advanced)</v>
       </c>
       <c r="H33" t="str">
         <f t="shared" si="0"/>
-        <v>[32] = {["ID"] = 1879513654; ["TIER"] = 4; }; -- Bee-slayer of Kighân</v>
+        <v xml:space="preserve"> [32] = {["ID"] = 1879513656; ["TIER"] = 3; }; -- Bee-slayer of Kighân (Advanced)</v>
       </c>
       <c r="I33">
         <f t="shared" si="1"/>
@@ -7328,11 +7340,11 @@
       </c>
       <c r="J33" t="str">
         <f t="shared" si="2"/>
-        <v>[32] = {</v>
+        <v xml:space="preserve"> [32] = {</v>
       </c>
       <c r="K33" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513654; </v>
+        <v xml:space="preserve">["ID"] = 1879513656; </v>
       </c>
       <c r="L33" t="str">
         <f t="shared" si="4"/>
@@ -7340,7 +7352,7 @@
       </c>
       <c r="M33" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N33" t="str">
         <f t="shared" si="6"/>
@@ -7349,21 +7361,21 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>1879513661</v>
+        <v>1879513654</v>
       </c>
       <c r="B34" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513661] = 3, // Brigand-bane of Kighân (Advanced)</v>
+        <v>[1879513654] = 4, // Bee-slayer of Kighân</v>
       </c>
       <c r="H34" t="str">
         <f t="shared" si="0"/>
-        <v>[33] = {["ID"] = 1879513661; ["TIER"] = 3; }; -- Brigand-bane of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [33] = {["ID"] = 1879513654; ["TIER"] = 4; }; -- Bee-slayer of Kighân</v>
       </c>
       <c r="I34">
         <f t="shared" si="1"/>
@@ -7371,11 +7383,11 @@
       </c>
       <c r="J34" t="str">
         <f t="shared" si="2"/>
-        <v>[33] = {</v>
+        <v xml:space="preserve"> [33] = {</v>
       </c>
       <c r="K34" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513661; </v>
+        <v xml:space="preserve">["ID"] = 1879513654; </v>
       </c>
       <c r="L34" t="str">
         <f t="shared" si="4"/>
@@ -7383,7 +7395,7 @@
       </c>
       <c r="M34" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N34" t="str">
         <f t="shared" si="6"/>
@@ -7392,21 +7404,21 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>1879513657</v>
+        <v>1879513661</v>
       </c>
       <c r="B35" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G35" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513657] = 4, // Brigand-bane of Kighân</v>
+        <v>[1879513661] = 3, // Brigand-bane of Kighân (Advanced)</v>
       </c>
       <c r="H35" t="str">
         <f t="shared" si="0"/>
-        <v>[34] = {["ID"] = 1879513657; ["TIER"] = 4; }; -- Brigand-bane of Kighân</v>
+        <v xml:space="preserve"> [34] = {["ID"] = 1879513661; ["TIER"] = 3; }; -- Brigand-bane of Kighân (Advanced)</v>
       </c>
       <c r="I35">
         <f t="shared" si="1"/>
@@ -7414,11 +7426,11 @@
       </c>
       <c r="J35" t="str">
         <f t="shared" si="2"/>
-        <v>[34] = {</v>
+        <v xml:space="preserve"> [34] = {</v>
       </c>
       <c r="K35" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513657; </v>
+        <v xml:space="preserve">["ID"] = 1879513661; </v>
       </c>
       <c r="L35" t="str">
         <f t="shared" si="4"/>
@@ -7426,7 +7438,7 @@
       </c>
       <c r="M35" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N35" t="str">
         <f t="shared" si="6"/>
@@ -7435,21 +7447,21 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>1879513662</v>
+        <v>1879513657</v>
       </c>
       <c r="B36" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G36" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513662] = 3, // Goblin-bane of Kighân (Advanced)</v>
+        <v>[1879513657] = 4, // Brigand-bane of Kighân</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="0"/>
-        <v>[35] = {["ID"] = 1879513662; ["TIER"] = 3; }; -- Goblin-bane of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [35] = {["ID"] = 1879513657; ["TIER"] = 4; }; -- Brigand-bane of Kighân</v>
       </c>
       <c r="I36">
         <f t="shared" si="1"/>
@@ -7457,11 +7469,11 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="2"/>
-        <v>[35] = {</v>
+        <v xml:space="preserve"> [35] = {</v>
       </c>
       <c r="K36" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513662; </v>
+        <v xml:space="preserve">["ID"] = 1879513657; </v>
       </c>
       <c r="L36" t="str">
         <f t="shared" si="4"/>
@@ -7469,7 +7481,7 @@
       </c>
       <c r="M36" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N36" t="str">
         <f t="shared" si="6"/>
@@ -7478,21 +7490,21 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>1879513658</v>
+        <v>1879513662</v>
       </c>
       <c r="B37" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C37">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G37" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513658] = 4, // Goblin-bane of Kighân</v>
+        <v>[1879513662] = 3, // Goblin-bane of Kighân (Advanced)</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="0"/>
-        <v>[36] = {["ID"] = 1879513658; ["TIER"] = 4; }; -- Goblin-bane of Kighân</v>
+        <v xml:space="preserve"> [36] = {["ID"] = 1879513662; ["TIER"] = 3; }; -- Goblin-bane of Kighân (Advanced)</v>
       </c>
       <c r="I37">
         <f t="shared" si="1"/>
@@ -7500,11 +7512,11 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="2"/>
-        <v>[36] = {</v>
+        <v xml:space="preserve"> [36] = {</v>
       </c>
       <c r="K37" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513658; </v>
+        <v xml:space="preserve">["ID"] = 1879513662; </v>
       </c>
       <c r="L37" t="str">
         <f t="shared" si="4"/>
@@ -7512,7 +7524,7 @@
       </c>
       <c r="M37" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N37" t="str">
         <f t="shared" si="6"/>
@@ -7521,21 +7533,21 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>1879513648</v>
+        <v>1879513658</v>
       </c>
       <c r="B38" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513648] = 3, // Ordâkhai-bane of Kighân (Advanced)</v>
+        <v>[1879513658] = 4, // Goblin-bane of Kighân</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="0"/>
-        <v>[37] = {["ID"] = 1879513648; ["TIER"] = 3; }; -- Ordâkhai-bane of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [37] = {["ID"] = 1879513658; ["TIER"] = 4; }; -- Goblin-bane of Kighân</v>
       </c>
       <c r="I38">
         <f t="shared" si="1"/>
@@ -7543,11 +7555,11 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="2"/>
-        <v>[37] = {</v>
+        <v xml:space="preserve"> [37] = {</v>
       </c>
       <c r="K38" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513648; </v>
+        <v xml:space="preserve">["ID"] = 1879513658; </v>
       </c>
       <c r="L38" t="str">
         <f t="shared" si="4"/>
@@ -7555,7 +7567,7 @@
       </c>
       <c r="M38" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N38" t="str">
         <f t="shared" si="6"/>
@@ -7564,21 +7576,21 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>1879513652</v>
+        <v>1879513648</v>
       </c>
       <c r="B39" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C39">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G39" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513652] = 4, // Ordâkhai-bane of Kighân</v>
+        <v>[1879513648] = 3, // Ordâkhai-bane of Kighân (Advanced)</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="0"/>
-        <v>[38] = {["ID"] = 1879513652; ["TIER"] = 4; }; -- Ordâkhai-bane of Kighân</v>
+        <v xml:space="preserve"> [38] = {["ID"] = 1879513648; ["TIER"] = 3; }; -- Ordâkhai-bane of Kighân (Advanced)</v>
       </c>
       <c r="I39">
         <f t="shared" si="1"/>
@@ -7586,11 +7598,11 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="2"/>
-        <v>[38] = {</v>
+        <v xml:space="preserve"> [38] = {</v>
       </c>
       <c r="K39" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513652; </v>
+        <v xml:space="preserve">["ID"] = 1879513648; </v>
       </c>
       <c r="L39" t="str">
         <f t="shared" si="4"/>
@@ -7598,7 +7610,7 @@
       </c>
       <c r="M39" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N39" t="str">
         <f t="shared" si="6"/>
@@ -7607,21 +7619,21 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>1879513643</v>
+        <v>1879513652</v>
       </c>
       <c r="B40" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513643] = 3, // Spider-slayer of Kighân (Advanced)</v>
+        <v>[1879513652] = 4, // Ordâkhai-bane of Kighân</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="0"/>
-        <v>[39] = {["ID"] = 1879513643; ["TIER"] = 3; }; -- Spider-slayer of Kighân (Advanced)</v>
+        <v xml:space="preserve"> [39] = {["ID"] = 1879513652; ["TIER"] = 4; }; -- Ordâkhai-bane of Kighân</v>
       </c>
       <c r="I40">
         <f t="shared" si="1"/>
@@ -7629,11 +7641,11 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="2"/>
-        <v>[39] = {</v>
+        <v xml:space="preserve"> [39] = {</v>
       </c>
       <c r="K40" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513643; </v>
+        <v xml:space="preserve">["ID"] = 1879513652; </v>
       </c>
       <c r="L40" t="str">
         <f t="shared" si="4"/>
@@ -7641,7 +7653,7 @@
       </c>
       <c r="M40" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N40" t="str">
         <f t="shared" si="6"/>
@@ -7650,21 +7662,21 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>1879513646</v>
+        <v>1879513643</v>
       </c>
       <c r="B41" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G41" t="str">
         <f t="shared" si="7"/>
-        <v>[1879513646] = 4, // Spider-slayer of Kighân</v>
+        <v>[1879513643] = 3, // Spider-slayer of Kighân (Advanced)</v>
       </c>
       <c r="H41" t="str">
         <f t="shared" si="0"/>
-        <v>[40] = {["ID"] = 1879513646; ["TIER"] = 4; }; -- Spider-slayer of Kighân</v>
+        <v xml:space="preserve"> [40] = {["ID"] = 1879513643; ["TIER"] = 3; }; -- Spider-slayer of Kighân (Advanced)</v>
       </c>
       <c r="I41">
         <f t="shared" si="1"/>
@@ -7672,11 +7684,11 @@
       </c>
       <c r="J41" t="str">
         <f t="shared" si="2"/>
-        <v>[40] = {</v>
+        <v xml:space="preserve"> [40] = {</v>
       </c>
       <c r="K41" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513646; </v>
+        <v xml:space="preserve">["ID"] = 1879513643; </v>
       </c>
       <c r="L41" t="str">
         <f t="shared" si="4"/>
@@ -7684,7 +7696,7 @@
       </c>
       <c r="M41" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N41" t="str">
         <f t="shared" si="6"/>
@@ -7693,76 +7705,80 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42">
+        <v>1879513646</v>
+      </c>
+      <c r="B42" t="s">
+        <v>415</v>
+      </c>
+      <c r="C42">
+        <v>4</v>
+      </c>
+      <c r="G42" t="str">
+        <f t="shared" si="7"/>
+        <v>[1879513646] = 4, // Spider-slayer of Kighân</v>
+      </c>
+      <c r="H42" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [41] = {["ID"] = 1879513646; ["TIER"] = 4; }; -- Spider-slayer of Kighân</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [41] = {</v>
+      </c>
+      <c r="K42" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve">["ID"] = 1879513646; </v>
+      </c>
+      <c r="L42" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
+      </c>
+      <c r="N42" t="str">
+        <f t="shared" si="6"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>1879513792</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>416</v>
       </c>
-      <c r="C42">
+      <c r="C43">
         <v>2</v>
       </c>
-      <c r="H42" t="str">
-        <f t="shared" si="0"/>
-        <v>[41] = {["ID"] = 1879513792; ["TIER"] = 2; }; -- Tales of Kighân</v>
-      </c>
-      <c r="I42">
-        <f t="shared" si="1"/>
-        <v>41</v>
-      </c>
-      <c r="J42" t="str">
-        <f t="shared" si="2"/>
-        <v>[41] = {</v>
-      </c>
-      <c r="K42" t="str">
+      <c r="H43" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> [42] = {["ID"] = 1879513792; ["TIER"] = 2; }; -- Tales of Kighân</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> [42] = {</v>
+      </c>
+      <c r="K43" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve">["ID"] = 1879513792; </v>
       </c>
-      <c r="L42" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="M42" t="str">
+      <c r="L43" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="M43" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve">["TIER"] = 2; </v>
-      </c>
-      <c r="N42" t="str">
-        <f t="shared" si="6"/>
-        <v>};</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="C43">
-        <v>1</v>
-      </c>
-      <c r="D43">
-        <v>339</v>
-      </c>
-      <c r="H43" t="str">
-        <f t="shared" si="0"/>
-        <v>[42] = {["CAT_ID"] = 339; ["TIER"] = 1; }; -- An Shêru</v>
-      </c>
-      <c r="I43">
-        <f t="shared" si="1"/>
-        <v>42</v>
-      </c>
-      <c r="J43" t="str">
-        <f t="shared" si="2"/>
-        <v>[42] = {</v>
-      </c>
-      <c r="K43" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L43" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve">["CAT_ID"] = 339; </v>
-      </c>
-      <c r="M43" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N43" t="str">
         <f t="shared" si="6"/>
@@ -7771,17 +7787,17 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>1879513780</v>
+        <v>1879521612</v>
       </c>
       <c r="B44" t="s">
-        <v>417</v>
+        <v>478</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
       <c r="H44" t="str">
         <f t="shared" si="0"/>
-        <v>[43] = {["ID"] = 1879513780; ["TIER"] = 1; }; -- Rejuvenator of An Shêru</v>
+        <v xml:space="preserve"> [43] = {["ID"] = 1879521612; ["TIER"] = 1; }; -- Persistent Defender of Kighân</v>
       </c>
       <c r="I44">
         <f t="shared" si="1"/>
@@ -7789,11 +7805,11 @@
       </c>
       <c r="J44" t="str">
         <f t="shared" si="2"/>
-        <v>[43] = {</v>
+        <v xml:space="preserve"> [43] = {</v>
       </c>
       <c r="K44" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513780; </v>
+        <v xml:space="preserve">["ID"] = 1879521612; </v>
       </c>
       <c r="L44" t="str">
         <f t="shared" si="4"/>
@@ -7809,18 +7825,18 @@
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>1879513788</v>
-      </c>
-      <c r="B45" t="s">
-        <v>418</v>
+      <c r="B45" s="1" t="s">
+        <v>457</v>
       </c>
       <c r="C45">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D45">
+        <v>339</v>
       </c>
       <c r="H45" t="str">
         <f t="shared" si="0"/>
-        <v>[44] = {["ID"] = 1879513788; ["TIER"] = 2; }; -- Explorer of An Shêru</v>
+        <v xml:space="preserve"> [44] = {["CAT_ID"] = 339; ["TIER"] = 1; }; -- An Shêru</v>
       </c>
       <c r="I45">
         <f t="shared" si="1"/>
@@ -7828,19 +7844,19 @@
       </c>
       <c r="J45" t="str">
         <f t="shared" si="2"/>
-        <v>[44] = {</v>
+        <v xml:space="preserve"> [44] = {</v>
       </c>
       <c r="K45" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513788; </v>
+        <v/>
       </c>
       <c r="L45" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["CAT_ID"] = 339; </v>
       </c>
       <c r="M45" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N45" t="str">
         <f t="shared" si="6"/>
@@ -7849,17 +7865,17 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>1879513789</v>
+        <v>1879513780</v>
       </c>
       <c r="B46" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H46" t="str">
         <f t="shared" si="0"/>
-        <v>[45] = {["ID"] = 1879513789; ["TIER"] = 3; }; -- New Threats in An Shêru</v>
+        <v xml:space="preserve"> [45] = {["ID"] = 1879513780; ["TIER"] = 1; }; -- Rejuvenator of An Shêru</v>
       </c>
       <c r="I46">
         <f t="shared" si="1"/>
@@ -7867,11 +7883,11 @@
       </c>
       <c r="J46" t="str">
         <f t="shared" si="2"/>
-        <v>[45] = {</v>
+        <v xml:space="preserve"> [45] = {</v>
       </c>
       <c r="K46" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513789; </v>
+        <v xml:space="preserve">["ID"] = 1879513780; </v>
       </c>
       <c r="L46" t="str">
         <f t="shared" si="4"/>
@@ -7879,7 +7895,7 @@
       </c>
       <c r="M46" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N46" t="str">
         <f t="shared" si="6"/>
@@ -7888,17 +7904,17 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>1879513775</v>
+        <v>1879513788</v>
       </c>
       <c r="B47" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="0"/>
-        <v>[46] = {["ID"] = 1879513775; ["TIER"] = 3; }; -- Reclaiming An Shêru</v>
+        <v xml:space="preserve"> [46] = {["ID"] = 1879513788; ["TIER"] = 2; }; -- Explorer of An Shêru</v>
       </c>
       <c r="I47">
         <f t="shared" si="1"/>
@@ -7906,11 +7922,11 @@
       </c>
       <c r="J47" t="str">
         <f t="shared" si="2"/>
-        <v>[46] = {</v>
+        <v xml:space="preserve"> [46] = {</v>
       </c>
       <c r="K47" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513775; </v>
+        <v xml:space="preserve">["ID"] = 1879513788; </v>
       </c>
       <c r="L47" t="str">
         <f t="shared" si="4"/>
@@ -7918,7 +7934,7 @@
       </c>
       <c r="M47" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N47" t="str">
         <f t="shared" si="6"/>
@@ -7927,17 +7943,17 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>1879513707</v>
+        <v>1879513789</v>
       </c>
       <c r="B48" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C48">
         <v>3</v>
       </c>
       <c r="H48" t="str">
         <f t="shared" si="0"/>
-        <v>[47] = {["ID"] = 1879513707; ["TIER"] = 3; }; -- Treasure-seeker of An Shêru</v>
+        <v xml:space="preserve"> [47] = {["ID"] = 1879513789; ["TIER"] = 3; }; -- New Threats in An Shêru</v>
       </c>
       <c r="I48">
         <f t="shared" si="1"/>
@@ -7945,11 +7961,11 @@
       </c>
       <c r="J48" t="str">
         <f t="shared" si="2"/>
-        <v>[47] = {</v>
+        <v xml:space="preserve"> [47] = {</v>
       </c>
       <c r="K48" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513707; </v>
+        <v xml:space="preserve">["ID"] = 1879513789; </v>
       </c>
       <c r="L48" t="str">
         <f t="shared" si="4"/>
@@ -7966,17 +7982,17 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>1879513697</v>
+        <v>1879513775</v>
       </c>
       <c r="B49" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H49" t="str">
         <f t="shared" si="0"/>
-        <v>[48] = {["ID"] = 1879513697; ["TIER"] = 2; }; -- Slayer of An Shêru</v>
+        <v xml:space="preserve"> [48] = {["ID"] = 1879513775; ["TIER"] = 3; }; -- Reclaiming An Shêru</v>
       </c>
       <c r="I49">
         <f t="shared" si="1"/>
@@ -7984,11 +8000,11 @@
       </c>
       <c r="J49" t="str">
         <f t="shared" si="2"/>
-        <v>[48] = {</v>
+        <v xml:space="preserve"> [48] = {</v>
       </c>
       <c r="K49" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513697; </v>
+        <v xml:space="preserve">["ID"] = 1879513775; </v>
       </c>
       <c r="L49" t="str">
         <f t="shared" si="4"/>
@@ -7996,7 +8012,7 @@
       </c>
       <c r="M49" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N49" t="str">
         <f t="shared" si="6"/>
@@ -8005,17 +8021,17 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>1879513669</v>
+        <v>1879513707</v>
       </c>
       <c r="B50" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C50">
         <v>3</v>
       </c>
       <c r="H50" t="str">
         <f t="shared" si="0"/>
-        <v>[49] = {["ID"] = 1879513669; ["TIER"] = 3; }; -- Brigand-bane of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [49] = {["ID"] = 1879513707; ["TIER"] = 3; }; -- Treasure-seeker of An Shêru</v>
       </c>
       <c r="I50">
         <f t="shared" si="1"/>
@@ -8023,11 +8039,11 @@
       </c>
       <c r="J50" t="str">
         <f t="shared" si="2"/>
-        <v>[49] = {</v>
+        <v xml:space="preserve"> [49] = {</v>
       </c>
       <c r="K50" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513669; </v>
+        <v xml:space="preserve">["ID"] = 1879513707; </v>
       </c>
       <c r="L50" t="str">
         <f t="shared" si="4"/>
@@ -8044,17 +8060,17 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>1879513688</v>
+        <v>1879513697</v>
       </c>
       <c r="B51" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C51">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H51" t="str">
         <f t="shared" si="0"/>
-        <v>[50] = {["ID"] = 1879513688; ["TIER"] = 4; }; -- Brigand-bane of An Shêru</v>
+        <v xml:space="preserve"> [50] = {["ID"] = 1879513697; ["TIER"] = 2; }; -- Slayer of An Shêru</v>
       </c>
       <c r="I51">
         <f t="shared" si="1"/>
@@ -8062,11 +8078,11 @@
       </c>
       <c r="J51" t="str">
         <f t="shared" si="2"/>
-        <v>[50] = {</v>
+        <v xml:space="preserve"> [50] = {</v>
       </c>
       <c r="K51" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513688; </v>
+        <v xml:space="preserve">["ID"] = 1879513697; </v>
       </c>
       <c r="L51" t="str">
         <f t="shared" si="4"/>
@@ -8074,7 +8090,7 @@
       </c>
       <c r="M51" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N51" t="str">
         <f t="shared" si="6"/>
@@ -8083,17 +8099,17 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>1879513668</v>
+        <v>1879513669</v>
       </c>
       <c r="B52" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C52">
         <v>3</v>
       </c>
       <c r="H52" t="str">
         <f t="shared" si="0"/>
-        <v>[51] = {["ID"] = 1879513668; ["TIER"] = 3; }; -- Dead-slayer of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [51] = {["ID"] = 1879513669; ["TIER"] = 3; }; -- Brigand-bane of An Shêru (Advanced)</v>
       </c>
       <c r="I52">
         <f t="shared" si="1"/>
@@ -8101,11 +8117,11 @@
       </c>
       <c r="J52" t="str">
         <f t="shared" si="2"/>
-        <v>[51] = {</v>
+        <v xml:space="preserve"> [51] = {</v>
       </c>
       <c r="K52" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513668; </v>
+        <v xml:space="preserve">["ID"] = 1879513669; </v>
       </c>
       <c r="L52" t="str">
         <f t="shared" si="4"/>
@@ -8122,17 +8138,17 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>1879513682</v>
+        <v>1879513688</v>
       </c>
       <c r="B53" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C53">
         <v>4</v>
       </c>
       <c r="H53" t="str">
         <f t="shared" si="0"/>
-        <v>[52] = {["ID"] = 1879513682; ["TIER"] = 4; }; -- Dead-slayer of An Shêru</v>
+        <v xml:space="preserve"> [52] = {["ID"] = 1879513688; ["TIER"] = 4; }; -- Brigand-bane of An Shêru</v>
       </c>
       <c r="I53">
         <f t="shared" si="1"/>
@@ -8140,11 +8156,11 @@
       </c>
       <c r="J53" t="str">
         <f t="shared" si="2"/>
-        <v>[52] = {</v>
+        <v xml:space="preserve"> [52] = {</v>
       </c>
       <c r="K53" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513682; </v>
+        <v xml:space="preserve">["ID"] = 1879513688; </v>
       </c>
       <c r="L53" t="str">
         <f t="shared" si="4"/>
@@ -8161,17 +8177,17 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>1879513665</v>
+        <v>1879513668</v>
       </c>
       <c r="B54" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C54">
         <v>3</v>
       </c>
       <c r="H54" t="str">
         <f t="shared" si="0"/>
-        <v>[53] = {["ID"] = 1879513665; ["TIER"] = 3; }; -- Utûgi-bane of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [53] = {["ID"] = 1879513668; ["TIER"] = 3; }; -- Dead-slayer of An Shêru (Advanced)</v>
       </c>
       <c r="I54">
         <f t="shared" si="1"/>
@@ -8179,11 +8195,11 @@
       </c>
       <c r="J54" t="str">
         <f t="shared" si="2"/>
-        <v>[53] = {</v>
+        <v xml:space="preserve"> [53] = {</v>
       </c>
       <c r="K54" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513665; </v>
+        <v xml:space="preserve">["ID"] = 1879513668; </v>
       </c>
       <c r="L54" t="str">
         <f t="shared" si="4"/>
@@ -8200,17 +8216,17 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>1879513674</v>
+        <v>1879513682</v>
       </c>
       <c r="B55" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C55">
         <v>4</v>
       </c>
       <c r="H55" t="str">
         <f t="shared" si="0"/>
-        <v>[54] = {["ID"] = 1879513674; ["TIER"] = 4; }; -- Utûgi-bane of An Shêru</v>
+        <v xml:space="preserve"> [54] = {["ID"] = 1879513682; ["TIER"] = 4; }; -- Dead-slayer of An Shêru</v>
       </c>
       <c r="I55">
         <f t="shared" si="1"/>
@@ -8218,11 +8234,11 @@
       </c>
       <c r="J55" t="str">
         <f t="shared" si="2"/>
-        <v>[54] = {</v>
+        <v xml:space="preserve"> [54] = {</v>
       </c>
       <c r="K55" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513674; </v>
+        <v xml:space="preserve">["ID"] = 1879513682; </v>
       </c>
       <c r="L55" t="str">
         <f t="shared" si="4"/>
@@ -8239,17 +8255,17 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>1879513681</v>
+        <v>1879513665</v>
       </c>
       <c r="B56" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C56">
         <v>3</v>
       </c>
       <c r="H56" t="str">
         <f t="shared" si="0"/>
-        <v>[55] = {["ID"] = 1879513681; ["TIER"] = 3; }; -- Grodbog-slayer of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [55] = {["ID"] = 1879513665; ["TIER"] = 3; }; -- Utûgi-bane of An Shêru (Advanced)</v>
       </c>
       <c r="I56">
         <f t="shared" si="1"/>
@@ -8257,11 +8273,11 @@
       </c>
       <c r="J56" t="str">
         <f t="shared" si="2"/>
-        <v>[55] = {</v>
+        <v xml:space="preserve"> [55] = {</v>
       </c>
       <c r="K56" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513681; </v>
+        <v xml:space="preserve">["ID"] = 1879513665; </v>
       </c>
       <c r="L56" t="str">
         <f t="shared" si="4"/>
@@ -8278,17 +8294,17 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>1879513673</v>
+        <v>1879513674</v>
       </c>
       <c r="B57" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C57">
         <v>4</v>
       </c>
       <c r="H57" t="str">
         <f t="shared" si="0"/>
-        <v>[56] = {["ID"] = 1879513673; ["TIER"] = 4; }; -- Grodbog-slayer of An Shêru</v>
+        <v xml:space="preserve"> [56] = {["ID"] = 1879513674; ["TIER"] = 4; }; -- Utûgi-bane of An Shêru</v>
       </c>
       <c r="I57">
         <f t="shared" si="1"/>
@@ -8296,11 +8312,11 @@
       </c>
       <c r="J57" t="str">
         <f t="shared" si="2"/>
-        <v>[56] = {</v>
+        <v xml:space="preserve"> [56] = {</v>
       </c>
       <c r="K57" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513673; </v>
+        <v xml:space="preserve">["ID"] = 1879513674; </v>
       </c>
       <c r="L57" t="str">
         <f t="shared" si="4"/>
@@ -8317,17 +8333,17 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>1879513686</v>
+        <v>1879513681</v>
       </c>
       <c r="B58" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C58">
         <v>3</v>
       </c>
       <c r="H58" t="str">
         <f t="shared" si="0"/>
-        <v>[57] = {["ID"] = 1879513686; ["TIER"] = 3; }; -- Ordâkhai-bane of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [57] = {["ID"] = 1879513681; ["TIER"] = 3; }; -- Grodbog-slayer of An Shêru (Advanced)</v>
       </c>
       <c r="I58">
         <f t="shared" si="1"/>
@@ -8335,11 +8351,11 @@
       </c>
       <c r="J58" t="str">
         <f t="shared" si="2"/>
-        <v>[57] = {</v>
+        <v xml:space="preserve"> [57] = {</v>
       </c>
       <c r="K58" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513686; </v>
+        <v xml:space="preserve">["ID"] = 1879513681; </v>
       </c>
       <c r="L58" t="str">
         <f t="shared" si="4"/>
@@ -8356,17 +8372,17 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>1879513671</v>
+        <v>1879513673</v>
       </c>
       <c r="B59" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C59">
         <v>4</v>
       </c>
       <c r="H59" t="str">
         <f t="shared" si="0"/>
-        <v>[58] = {["ID"] = 1879513671; ["TIER"] = 4; }; -- Ordâkhai-bane of An Shêru</v>
+        <v xml:space="preserve"> [58] = {["ID"] = 1879513673; ["TIER"] = 4; }; -- Grodbog-slayer of An Shêru</v>
       </c>
       <c r="I59">
         <f t="shared" si="1"/>
@@ -8374,11 +8390,11 @@
       </c>
       <c r="J59" t="str">
         <f t="shared" si="2"/>
-        <v>[58] = {</v>
+        <v xml:space="preserve"> [58] = {</v>
       </c>
       <c r="K59" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513671; </v>
+        <v xml:space="preserve">["ID"] = 1879513673; </v>
       </c>
       <c r="L59" t="str">
         <f t="shared" si="4"/>
@@ -8395,17 +8411,17 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>1879513667</v>
+        <v>1879513686</v>
       </c>
       <c r="B60" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C60">
         <v>3</v>
       </c>
       <c r="H60" t="str">
         <f t="shared" si="0"/>
-        <v>[59] = {["ID"] = 1879513667; ["TIER"] = 3; }; -- Worm-bane of An Shêru (Advanced)</v>
+        <v xml:space="preserve"> [59] = {["ID"] = 1879513686; ["TIER"] = 3; }; -- Ordâkhai-bane of An Shêru (Advanced)</v>
       </c>
       <c r="I60">
         <f t="shared" si="1"/>
@@ -8413,11 +8429,11 @@
       </c>
       <c r="J60" t="str">
         <f t="shared" si="2"/>
-        <v>[59] = {</v>
+        <v xml:space="preserve"> [59] = {</v>
       </c>
       <c r="K60" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513667; </v>
+        <v xml:space="preserve">["ID"] = 1879513686; </v>
       </c>
       <c r="L60" t="str">
         <f t="shared" si="4"/>
@@ -8434,17 +8450,17 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>1879513684</v>
+        <v>1879513671</v>
       </c>
       <c r="B61" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C61">
         <v>4</v>
       </c>
       <c r="H61" t="str">
         <f t="shared" si="0"/>
-        <v>[60] = {["ID"] = 1879513684; ["TIER"] = 4; }; -- Worm-bane of An Shêru</v>
+        <v xml:space="preserve"> [60] = {["ID"] = 1879513671; ["TIER"] = 4; }; -- Ordâkhai-bane of An Shêru</v>
       </c>
       <c r="I61">
         <f t="shared" si="1"/>
@@ -8452,11 +8468,11 @@
       </c>
       <c r="J61" t="str">
         <f t="shared" si="2"/>
-        <v>[60] = {</v>
+        <v xml:space="preserve"> [60] = {</v>
       </c>
       <c r="K61" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513684; </v>
+        <v xml:space="preserve">["ID"] = 1879513671; </v>
       </c>
       <c r="L61" t="str">
         <f t="shared" si="4"/>
@@ -8473,17 +8489,17 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>1879513786</v>
+        <v>1879513667</v>
       </c>
       <c r="B62" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H62" t="str">
         <f t="shared" si="0"/>
-        <v>[61] = {["ID"] = 1879513786; ["TIER"] = 2; }; -- Tales of An Shêru</v>
+        <v xml:space="preserve"> [61] = {["ID"] = 1879513667; ["TIER"] = 3; }; -- Worm-bane of An Shêru (Advanced)</v>
       </c>
       <c r="I62">
         <f t="shared" si="1"/>
@@ -8491,11 +8507,11 @@
       </c>
       <c r="J62" t="str">
         <f t="shared" si="2"/>
-        <v>[61] = {</v>
+        <v xml:space="preserve"> [61] = {</v>
       </c>
       <c r="K62" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513786; </v>
+        <v xml:space="preserve">["ID"] = 1879513667; </v>
       </c>
       <c r="L62" t="str">
         <f t="shared" si="4"/>
@@ -8503,7 +8519,7 @@
       </c>
       <c r="M62" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N62" t="str">
         <f t="shared" si="6"/>
@@ -8511,18 +8527,18 @@
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B63" s="1" t="s">
-        <v>458</v>
+      <c r="A63">
+        <v>1879513684</v>
+      </c>
+      <c r="B63" t="s">
+        <v>434</v>
       </c>
       <c r="C63">
-        <v>1</v>
-      </c>
-      <c r="D63">
-        <v>340</v>
+        <v>4</v>
       </c>
       <c r="H63" t="str">
         <f t="shared" si="0"/>
-        <v>[62] = {["CAT_ID"] = 340; ["TIER"] = 1; }; -- Idagâl</v>
+        <v xml:space="preserve"> [62] = {["ID"] = 1879513684; ["TIER"] = 4; }; -- Worm-bane of An Shêru</v>
       </c>
       <c r="I63">
         <f t="shared" si="1"/>
@@ -8530,19 +8546,19 @@
       </c>
       <c r="J63" t="str">
         <f t="shared" si="2"/>
-        <v>[62] = {</v>
+        <v xml:space="preserve"> [62] = {</v>
       </c>
       <c r="K63" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879513684; </v>
       </c>
       <c r="L63" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">["CAT_ID"] = 340; </v>
+        <v/>
       </c>
       <c r="M63" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N63" t="str">
         <f t="shared" si="6"/>
@@ -8551,17 +8567,17 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>1879513783</v>
+        <v>1879513786</v>
       </c>
       <c r="B64" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H64" t="str">
         <f t="shared" si="0"/>
-        <v>[63] = {["ID"] = 1879513783; ["TIER"] = 1; }; -- Renewer of Idagâl</v>
+        <v xml:space="preserve"> [63] = {["ID"] = 1879513786; ["TIER"] = 2; }; -- Tales of An Shêru</v>
       </c>
       <c r="I64">
         <f t="shared" si="1"/>
@@ -8569,11 +8585,11 @@
       </c>
       <c r="J64" t="str">
         <f t="shared" si="2"/>
-        <v>[63] = {</v>
+        <v xml:space="preserve"> [63] = {</v>
       </c>
       <c r="K64" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513783; </v>
+        <v xml:space="preserve">["ID"] = 1879513786; </v>
       </c>
       <c r="L64" t="str">
         <f t="shared" si="4"/>
@@ -8581,7 +8597,7 @@
       </c>
       <c r="M64" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N64" t="str">
         <f t="shared" si="6"/>
@@ -8590,17 +8606,17 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>1879513784</v>
+        <v>1879521613</v>
       </c>
       <c r="B65" t="s">
-        <v>437</v>
+        <v>479</v>
       </c>
       <c r="C65">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H65" t="str">
         <f t="shared" si="0"/>
-        <v>[64] = {["ID"] = 1879513784; ["TIER"] = 2; }; -- Explorer of Idagâl</v>
+        <v xml:space="preserve"> [64] = {["ID"] = 1879521613; ["TIER"] = 1; }; -- Persistent Defender of An Shêru</v>
       </c>
       <c r="I65">
         <f t="shared" si="1"/>
@@ -8608,11 +8624,11 @@
       </c>
       <c r="J65" t="str">
         <f t="shared" si="2"/>
-        <v>[64] = {</v>
+        <v xml:space="preserve"> [64] = {</v>
       </c>
       <c r="K65" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513784; </v>
+        <v xml:space="preserve">["ID"] = 1879521613; </v>
       </c>
       <c r="L65" t="str">
         <f t="shared" si="4"/>
@@ -8620,7 +8636,7 @@
       </c>
       <c r="M65" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N65" t="str">
         <f t="shared" si="6"/>
@@ -8628,18 +8644,18 @@
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>1879513793</v>
-      </c>
-      <c r="B66" t="s">
-        <v>438</v>
+      <c r="B66" s="1" t="s">
+        <v>458</v>
       </c>
       <c r="C66">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>340</v>
       </c>
       <c r="H66" t="str">
         <f t="shared" si="0"/>
-        <v>[65] = {["ID"] = 1879513793; ["TIER"] = 3; }; -- New Threats in Idagâl</v>
+        <v xml:space="preserve"> [65] = {["CAT_ID"] = 340; ["TIER"] = 1; }; -- Idagâl</v>
       </c>
       <c r="I66">
         <f t="shared" si="1"/>
@@ -8647,19 +8663,19 @@
       </c>
       <c r="J66" t="str">
         <f t="shared" si="2"/>
-        <v>[65] = {</v>
+        <v xml:space="preserve"> [65] = {</v>
       </c>
       <c r="K66" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">["ID"] = 1879513793; </v>
+        <v/>
       </c>
       <c r="L66" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v xml:space="preserve">["CAT_ID"] = 340; </v>
       </c>
       <c r="M66" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N66" t="str">
         <f t="shared" si="6"/>
@@ -8668,56 +8684,56 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>1879513776</v>
+        <v>1879513783</v>
       </c>
       <c r="B67" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C67">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H67" t="str">
-        <f t="shared" ref="H67:H103" si="8">CONCATENATE(J67,K67,L67,M67,N67," -- ",B67)</f>
-        <v>[66] = {["ID"] = 1879513776; ["TIER"] = 3; }; -- Reclaiming Idagâl</v>
+        <f t="shared" ref="H67:H107" si="8">CONCATENATE(J67,K67,L67,M67,N67," -- ",B67)</f>
+        <v xml:space="preserve"> [66] = {["ID"] = 1879513783; ["TIER"] = 1; }; -- Renewer of Idagâl</v>
       </c>
       <c r="I67">
-        <f t="shared" ref="I67:I103" si="9">ROW()-1</f>
+        <f t="shared" ref="I67:I107" si="9">ROW()-1</f>
         <v>66</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" ref="J67:J103" si="10">CONCATENATE(REPT(" ",2-LEN(I67)),"[",I67,"] = {")</f>
-        <v>[66] = {</v>
+        <f t="shared" ref="J67:J107" si="10">CONCATENATE(REPT(" ",3-LEN(I67)),"[",I67,"] = {")</f>
+        <v xml:space="preserve"> [66] = {</v>
       </c>
       <c r="K67" t="str">
-        <f t="shared" ref="K67:K103" si="11">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
-        <v xml:space="preserve">["ID"] = 1879513776; </v>
+        <f t="shared" ref="K67:K107" si="11">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
+        <v xml:space="preserve">["ID"] = 1879513783; </v>
       </c>
       <c r="L67" t="str">
-        <f t="shared" ref="L67:L103" si="12">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
+        <f t="shared" ref="L67:L107" si="12">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
         <v/>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M103" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <f t="shared" ref="M67:M107" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N67" t="str">
-        <f t="shared" ref="N67:N103" si="14">CONCATENATE("};")</f>
+        <f t="shared" ref="N67:N107" si="14">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>1879513699</v>
+        <v>1879513784</v>
       </c>
       <c r="B68" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H68" t="str">
         <f t="shared" si="8"/>
-        <v>[67] = {["ID"] = 1879513699; ["TIER"] = 3; }; -- Treasure-seeker of Idagâl</v>
+        <v xml:space="preserve"> [67] = {["ID"] = 1879513784; ["TIER"] = 2; }; -- Explorer of Idagâl</v>
       </c>
       <c r="I68">
         <f t="shared" si="9"/>
@@ -8725,11 +8741,11 @@
       </c>
       <c r="J68" t="str">
         <f t="shared" si="10"/>
-        <v>[67] = {</v>
+        <v xml:space="preserve"> [67] = {</v>
       </c>
       <c r="K68" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513699; </v>
+        <v xml:space="preserve">["ID"] = 1879513784; </v>
       </c>
       <c r="L68" t="str">
         <f t="shared" si="12"/>
@@ -8737,7 +8753,7 @@
       </c>
       <c r="M68" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N68" t="str">
         <f t="shared" si="14"/>
@@ -8746,17 +8762,17 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>1879513700</v>
+        <v>1879513793</v>
       </c>
       <c r="B69" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H69" t="str">
         <f t="shared" si="8"/>
-        <v>[68] = {["ID"] = 1879513700; ["TIER"] = 2; }; -- Slayer of Idagâl</v>
+        <v xml:space="preserve"> [68] = {["ID"] = 1879513793; ["TIER"] = 3; }; -- New Threats in Idagâl</v>
       </c>
       <c r="I69">
         <f t="shared" si="9"/>
@@ -8764,11 +8780,11 @@
       </c>
       <c r="J69" t="str">
         <f t="shared" si="10"/>
-        <v>[68] = {</v>
+        <v xml:space="preserve"> [68] = {</v>
       </c>
       <c r="K69" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513700; </v>
+        <v xml:space="preserve">["ID"] = 1879513793; </v>
       </c>
       <c r="L69" t="str">
         <f t="shared" si="12"/>
@@ -8776,7 +8792,7 @@
       </c>
       <c r="M69" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N69" t="str">
         <f t="shared" si="14"/>
@@ -8785,17 +8801,17 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>1879513670</v>
+        <v>1879513776</v>
       </c>
       <c r="B70" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="C70">
         <v>3</v>
       </c>
       <c r="H70" t="str">
         <f t="shared" si="8"/>
-        <v>[69] = {["ID"] = 1879513670; ["TIER"] = 3; }; -- Brigand-bane of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [69] = {["ID"] = 1879513776; ["TIER"] = 3; }; -- Reclaiming Idagâl</v>
       </c>
       <c r="I70">
         <f t="shared" si="9"/>
@@ -8803,11 +8819,11 @@
       </c>
       <c r="J70" t="str">
         <f t="shared" si="10"/>
-        <v>[69] = {</v>
+        <v xml:space="preserve"> [69] = {</v>
       </c>
       <c r="K70" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513670; </v>
+        <v xml:space="preserve">["ID"] = 1879513776; </v>
       </c>
       <c r="L70" t="str">
         <f t="shared" si="12"/>
@@ -8824,17 +8840,17 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>1879513680</v>
+        <v>1879513699</v>
       </c>
       <c r="B71" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H71" t="str">
         <f t="shared" si="8"/>
-        <v>[70] = {["ID"] = 1879513680; ["TIER"] = 4; }; -- Brigand-bane of Idagâl</v>
+        <v xml:space="preserve"> [70] = {["ID"] = 1879513699; ["TIER"] = 3; }; -- Treasure-seeker of Idagâl</v>
       </c>
       <c r="I71">
         <f t="shared" si="9"/>
@@ -8842,11 +8858,11 @@
       </c>
       <c r="J71" t="str">
         <f t="shared" si="10"/>
-        <v>[70] = {</v>
+        <v xml:space="preserve"> [70] = {</v>
       </c>
       <c r="K71" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513680; </v>
+        <v xml:space="preserve">["ID"] = 1879513699; </v>
       </c>
       <c r="L71" t="str">
         <f t="shared" si="12"/>
@@ -8854,7 +8870,7 @@
       </c>
       <c r="M71" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N71" t="str">
         <f t="shared" si="14"/>
@@ -8863,17 +8879,17 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>1879513683</v>
+        <v>1879513700</v>
       </c>
       <c r="B72" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="C72">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H72" t="str">
         <f t="shared" si="8"/>
-        <v>[71] = {["ID"] = 1879513683; ["TIER"] = 3; }; -- Cobra-slayer of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [71] = {["ID"] = 1879513700; ["TIER"] = 2; }; -- Slayer of Idagâl</v>
       </c>
       <c r="I72">
         <f t="shared" si="9"/>
@@ -8881,11 +8897,11 @@
       </c>
       <c r="J72" t="str">
         <f t="shared" si="10"/>
-        <v>[71] = {</v>
+        <v xml:space="preserve"> [71] = {</v>
       </c>
       <c r="K72" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513683; </v>
+        <v xml:space="preserve">["ID"] = 1879513700; </v>
       </c>
       <c r="L72" t="str">
         <f t="shared" si="12"/>
@@ -8893,7 +8909,7 @@
       </c>
       <c r="M72" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N72" t="str">
         <f t="shared" si="14"/>
@@ -8902,17 +8918,17 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>1879513676</v>
+        <v>1879513670</v>
       </c>
       <c r="B73" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="C73">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H73" t="str">
         <f t="shared" si="8"/>
-        <v>[72] = {["ID"] = 1879513676; ["TIER"] = 4; }; -- Cobra-slayer of Idagâl</v>
+        <v xml:space="preserve"> [72] = {["ID"] = 1879513670; ["TIER"] = 3; }; -- Brigand-bane of Idagâl (Advanced)</v>
       </c>
       <c r="I73">
         <f t="shared" si="9"/>
@@ -8920,11 +8936,11 @@
       </c>
       <c r="J73" t="str">
         <f t="shared" si="10"/>
-        <v>[72] = {</v>
+        <v xml:space="preserve"> [72] = {</v>
       </c>
       <c r="K73" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513676; </v>
+        <v xml:space="preserve">["ID"] = 1879513670; </v>
       </c>
       <c r="L73" t="str">
         <f t="shared" si="12"/>
@@ -8932,7 +8948,7 @@
       </c>
       <c r="M73" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N73" t="str">
         <f t="shared" si="14"/>
@@ -8941,17 +8957,17 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>1879513672</v>
+        <v>1879513680</v>
       </c>
       <c r="B74" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H74" t="str">
         <f t="shared" si="8"/>
-        <v>[73] = {["ID"] = 1879513672; ["TIER"] = 3; }; -- Drake-slayer of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [73] = {["ID"] = 1879513680; ["TIER"] = 4; }; -- Brigand-bane of Idagâl</v>
       </c>
       <c r="I74">
         <f t="shared" si="9"/>
@@ -8959,11 +8975,11 @@
       </c>
       <c r="J74" t="str">
         <f t="shared" si="10"/>
-        <v>[73] = {</v>
+        <v xml:space="preserve"> [73] = {</v>
       </c>
       <c r="K74" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513672; </v>
+        <v xml:space="preserve">["ID"] = 1879513680; </v>
       </c>
       <c r="L74" t="str">
         <f t="shared" si="12"/>
@@ -8971,7 +8987,7 @@
       </c>
       <c r="M74" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N74" t="str">
         <f t="shared" si="14"/>
@@ -8980,17 +8996,17 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>1879513685</v>
+        <v>1879513683</v>
       </c>
       <c r="B75" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C75">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H75" t="str">
         <f t="shared" si="8"/>
-        <v>[74] = {["ID"] = 1879513685; ["TIER"] = 4; }; -- Drake-slayer of Idagâl</v>
+        <v xml:space="preserve"> [74] = {["ID"] = 1879513683; ["TIER"] = 3; }; -- Cobra-slayer of Idagâl (Advanced)</v>
       </c>
       <c r="I75">
         <f t="shared" si="9"/>
@@ -8998,11 +9014,11 @@
       </c>
       <c r="J75" t="str">
         <f t="shared" si="10"/>
-        <v>[74] = {</v>
+        <v xml:space="preserve"> [74] = {</v>
       </c>
       <c r="K75" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513685; </v>
+        <v xml:space="preserve">["ID"] = 1879513683; </v>
       </c>
       <c r="L75" t="str">
         <f t="shared" si="12"/>
@@ -9010,7 +9026,7 @@
       </c>
       <c r="M75" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N75" t="str">
         <f t="shared" si="14"/>
@@ -9019,17 +9035,17 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>1879513675</v>
+        <v>1879513676</v>
       </c>
       <c r="B76" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="C76">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H76" t="str">
         <f t="shared" si="8"/>
-        <v>[75] = {["ID"] = 1879513675; ["TIER"] = 3; }; -- Utûgi-bane of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [75] = {["ID"] = 1879513676; ["TIER"] = 4; }; -- Cobra-slayer of Idagâl</v>
       </c>
       <c r="I76">
         <f t="shared" si="9"/>
@@ -9037,11 +9053,11 @@
       </c>
       <c r="J76" t="str">
         <f t="shared" si="10"/>
-        <v>[75] = {</v>
+        <v xml:space="preserve"> [75] = {</v>
       </c>
       <c r="K76" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513675; </v>
+        <v xml:space="preserve">["ID"] = 1879513676; </v>
       </c>
       <c r="L76" t="str">
         <f t="shared" si="12"/>
@@ -9049,7 +9065,7 @@
       </c>
       <c r="M76" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N76" t="str">
         <f t="shared" si="14"/>
@@ -9058,17 +9074,17 @@
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>1879513687</v>
+        <v>1879513672</v>
       </c>
       <c r="B77" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="C77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H77" t="str">
         <f t="shared" si="8"/>
-        <v>[76] = {["ID"] = 1879513687; ["TIER"] = 4; }; -- Utûgi-bane of Idagâl</v>
+        <v xml:space="preserve"> [76] = {["ID"] = 1879513672; ["TIER"] = 3; }; -- Drake-slayer of Idagâl (Advanced)</v>
       </c>
       <c r="I77">
         <f t="shared" si="9"/>
@@ -9076,11 +9092,11 @@
       </c>
       <c r="J77" t="str">
         <f t="shared" si="10"/>
-        <v>[76] = {</v>
+        <v xml:space="preserve"> [76] = {</v>
       </c>
       <c r="K77" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513687; </v>
+        <v xml:space="preserve">["ID"] = 1879513672; </v>
       </c>
       <c r="L77" t="str">
         <f t="shared" si="12"/>
@@ -9088,7 +9104,7 @@
       </c>
       <c r="M77" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N77" t="str">
         <f t="shared" si="14"/>
@@ -9097,17 +9113,17 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>1879513677</v>
+        <v>1879513685</v>
       </c>
       <c r="B78" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C78">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H78" t="str">
         <f t="shared" si="8"/>
-        <v>[77] = {["ID"] = 1879513677; ["TIER"] = 3; }; -- Kergrim-slayer of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [77] = {["ID"] = 1879513685; ["TIER"] = 4; }; -- Drake-slayer of Idagâl</v>
       </c>
       <c r="I78">
         <f t="shared" si="9"/>
@@ -9115,11 +9131,11 @@
       </c>
       <c r="J78" t="str">
         <f t="shared" si="10"/>
-        <v>[77] = {</v>
+        <v xml:space="preserve"> [77] = {</v>
       </c>
       <c r="K78" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513677; </v>
+        <v xml:space="preserve">["ID"] = 1879513685; </v>
       </c>
       <c r="L78" t="str">
         <f t="shared" si="12"/>
@@ -9127,7 +9143,7 @@
       </c>
       <c r="M78" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N78" t="str">
         <f t="shared" si="14"/>
@@ -9136,17 +9152,17 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>1879513678</v>
+        <v>1879513675</v>
       </c>
       <c r="B79" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="C79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H79" t="str">
         <f t="shared" si="8"/>
-        <v>[78] = {["ID"] = 1879513678; ["TIER"] = 4; }; -- Kergrim-slayer of Idagâl</v>
+        <v xml:space="preserve"> [78] = {["ID"] = 1879513675; ["TIER"] = 3; }; -- Utûgi-bane of Idagâl (Advanced)</v>
       </c>
       <c r="I79">
         <f t="shared" si="9"/>
@@ -9154,11 +9170,11 @@
       </c>
       <c r="J79" t="str">
         <f t="shared" si="10"/>
-        <v>[78] = {</v>
+        <v xml:space="preserve"> [78] = {</v>
       </c>
       <c r="K79" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513678; </v>
+        <v xml:space="preserve">["ID"] = 1879513675; </v>
       </c>
       <c r="L79" t="str">
         <f t="shared" si="12"/>
@@ -9166,7 +9182,7 @@
       </c>
       <c r="M79" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N79" t="str">
         <f t="shared" si="14"/>
@@ -9175,17 +9191,17 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>1879513679</v>
+        <v>1879513687</v>
       </c>
       <c r="B80" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="C80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H80" t="str">
         <f t="shared" si="8"/>
-        <v>[79] = {["ID"] = 1879513679; ["TIER"] = 3; }; -- Ordâkhai-bane of Idagâl (Advanced)</v>
+        <v xml:space="preserve"> [79] = {["ID"] = 1879513687; ["TIER"] = 4; }; -- Utûgi-bane of Idagâl</v>
       </c>
       <c r="I80">
         <f t="shared" si="9"/>
@@ -9193,11 +9209,11 @@
       </c>
       <c r="J80" t="str">
         <f t="shared" si="10"/>
-        <v>[79] = {</v>
+        <v xml:space="preserve"> [79] = {</v>
       </c>
       <c r="K80" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513679; </v>
+        <v xml:space="preserve">["ID"] = 1879513687; </v>
       </c>
       <c r="L80" t="str">
         <f t="shared" si="12"/>
@@ -9205,7 +9221,7 @@
       </c>
       <c r="M80" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 3; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N80" t="str">
         <f t="shared" si="14"/>
@@ -9214,17 +9230,17 @@
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>1879513666</v>
+        <v>1879513677</v>
       </c>
       <c r="B81" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="C81">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H81" t="str">
         <f t="shared" si="8"/>
-        <v>[80] = {["ID"] = 1879513666; ["TIER"] = 4; }; -- Ordâkhai-bane of Idagâl</v>
+        <v xml:space="preserve"> [80] = {["ID"] = 1879513677; ["TIER"] = 3; }; -- Kergrim-slayer of Idagâl (Advanced)</v>
       </c>
       <c r="I81">
         <f t="shared" si="9"/>
@@ -9232,11 +9248,11 @@
       </c>
       <c r="J81" t="str">
         <f t="shared" si="10"/>
-        <v>[80] = {</v>
+        <v xml:space="preserve"> [80] = {</v>
       </c>
       <c r="K81" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513666; </v>
+        <v xml:space="preserve">["ID"] = 1879513677; </v>
       </c>
       <c r="L81" t="str">
         <f t="shared" si="12"/>
@@ -9244,7 +9260,7 @@
       </c>
       <c r="M81" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 4; </v>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N81" t="str">
         <f t="shared" si="14"/>
@@ -9253,17 +9269,17 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>1879513777</v>
+        <v>1879513678</v>
       </c>
       <c r="B82" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C82">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H82" t="str">
         <f t="shared" si="8"/>
-        <v>[81] = {["ID"] = 1879513777; ["TIER"] = 2; }; -- Tales of Idagâl</v>
+        <v xml:space="preserve"> [81] = {["ID"] = 1879513678; ["TIER"] = 4; }; -- Kergrim-slayer of Idagâl</v>
       </c>
       <c r="I82">
         <f t="shared" si="9"/>
@@ -9271,11 +9287,11 @@
       </c>
       <c r="J82" t="str">
         <f t="shared" si="10"/>
-        <v>[81] = {</v>
+        <v xml:space="preserve"> [81] = {</v>
       </c>
       <c r="K82" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513777; </v>
+        <v xml:space="preserve">["ID"] = 1879513678; </v>
       </c>
       <c r="L82" t="str">
         <f t="shared" si="12"/>
@@ -9283,7 +9299,7 @@
       </c>
       <c r="M82" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 2; </v>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N82" t="str">
         <f t="shared" si="14"/>
@@ -9291,15 +9307,18 @@
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B83" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D83">
-        <v>341</v>
+      <c r="A83">
+        <v>1879513679</v>
+      </c>
+      <c r="B83" t="s">
+        <v>452</v>
+      </c>
+      <c r="C83">
+        <v>3</v>
       </c>
       <c r="H83" t="str">
         <f t="shared" si="8"/>
-        <v>[82] = {["CAT_ID"] = 341; }; -- Mûr Ghala</v>
+        <v xml:space="preserve"> [82] = {["ID"] = 1879513679; ["TIER"] = 3; }; -- Ordâkhai-bane of Idagâl (Advanced)</v>
       </c>
       <c r="I83">
         <f t="shared" si="9"/>
@@ -9307,19 +9326,19 @@
       </c>
       <c r="J83" t="str">
         <f t="shared" si="10"/>
-        <v>[82] = {</v>
+        <v xml:space="preserve"> [82] = {</v>
       </c>
       <c r="K83" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879513679; </v>
       </c>
       <c r="L83" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve">["CAT_ID"] = 341; </v>
+        <v/>
       </c>
       <c r="M83" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
       </c>
       <c r="N83" t="str">
         <f t="shared" si="14"/>
@@ -9328,14 +9347,17 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>1879514041</v>
+        <v>1879513666</v>
       </c>
       <c r="B84" t="s">
-        <v>460</v>
+        <v>453</v>
+      </c>
+      <c r="C84">
+        <v>4</v>
       </c>
       <c r="H84" t="str">
         <f t="shared" si="8"/>
-        <v>[83] = {["ID"] = 1879514041; }; -- Hunter of Mûr Ghala</v>
+        <v xml:space="preserve"> [83] = {["ID"] = 1879513666; ["TIER"] = 4; }; -- Ordâkhai-bane of Idagâl</v>
       </c>
       <c r="I84">
         <f t="shared" si="9"/>
@@ -9343,11 +9365,11 @@
       </c>
       <c r="J84" t="str">
         <f t="shared" si="10"/>
-        <v>[83] = {</v>
+        <v xml:space="preserve"> [83] = {</v>
       </c>
       <c r="K84" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514041; </v>
+        <v xml:space="preserve">["ID"] = 1879513666; </v>
       </c>
       <c r="L84" t="str">
         <f t="shared" si="12"/>
@@ -9355,7 +9377,7 @@
       </c>
       <c r="M84" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 4; </v>
       </c>
       <c r="N84" t="str">
         <f t="shared" si="14"/>
@@ -9364,17 +9386,17 @@
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>1879514045</v>
+        <v>1879513777</v>
       </c>
       <c r="B85" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="C85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H85" t="str">
         <f t="shared" si="8"/>
-        <v>[84] = {["ID"] = 1879514045; ["TIER"] = 1; }; -- Adversaries of Adagím</v>
+        <v xml:space="preserve"> [84] = {["ID"] = 1879513777; ["TIER"] = 2; }; -- Tales of Idagâl</v>
       </c>
       <c r="I85">
         <f t="shared" si="9"/>
@@ -9382,11 +9404,11 @@
       </c>
       <c r="J85" t="str">
         <f t="shared" si="10"/>
-        <v>[84] = {</v>
+        <v xml:space="preserve"> [84] = {</v>
       </c>
       <c r="K85" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514045; </v>
+        <v xml:space="preserve">["ID"] = 1879513777; </v>
       </c>
       <c r="L85" t="str">
         <f t="shared" si="12"/>
@@ -9394,7 +9416,7 @@
       </c>
       <c r="M85" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
+        <v xml:space="preserve">["TIER"] = 2; </v>
       </c>
       <c r="N85" t="str">
         <f t="shared" si="14"/>
@@ -9403,17 +9425,17 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>1879514044</v>
+        <v>1879521614</v>
       </c>
       <c r="B86" t="s">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="H86" t="str">
         <f t="shared" si="8"/>
-        <v>[85] = {["ID"] = 1879514044; ["TIER"] = 1; }; -- Combatants of Kighân</v>
+        <v xml:space="preserve"> [85] = {["ID"] = 1879521614; ["TIER"] = 1; }; -- Persistent Defender of Idagâl</v>
       </c>
       <c r="I86">
         <f t="shared" si="9"/>
@@ -9421,11 +9443,11 @@
       </c>
       <c r="J86" t="str">
         <f t="shared" si="10"/>
-        <v>[85] = {</v>
+        <v xml:space="preserve"> [85] = {</v>
       </c>
       <c r="K86" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514044; </v>
+        <v xml:space="preserve">["ID"] = 1879521614; </v>
       </c>
       <c r="L86" t="str">
         <f t="shared" si="12"/>
@@ -9441,18 +9463,15 @@
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A87">
-        <v>1879514039</v>
-      </c>
-      <c r="B87" t="s">
-        <v>463</v>
-      </c>
-      <c r="C87">
-        <v>1</v>
+      <c r="B87" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D87">
+        <v>341</v>
       </c>
       <c r="H87" t="str">
         <f t="shared" si="8"/>
-        <v>[86] = {["ID"] = 1879514039; ["TIER"] = 1; }; -- Enemies of An Shêru</v>
+        <v xml:space="preserve"> [86] = {["CAT_ID"] = 341; }; -- Mûr Ghala</v>
       </c>
       <c r="I87">
         <f t="shared" si="9"/>
@@ -9460,19 +9479,19 @@
       </c>
       <c r="J87" t="str">
         <f t="shared" si="10"/>
-        <v>[86] = {</v>
+        <v xml:space="preserve"> [86] = {</v>
       </c>
       <c r="K87" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514039; </v>
+        <v/>
       </c>
       <c r="L87" t="str">
         <f t="shared" si="12"/>
-        <v/>
+        <v xml:space="preserve">["CAT_ID"] = 341; </v>
       </c>
       <c r="M87" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
+        <v/>
       </c>
       <c r="N87" t="str">
         <f t="shared" si="14"/>
@@ -9481,17 +9500,14 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>1879514047</v>
+        <v>1879514041</v>
       </c>
       <c r="B88" t="s">
-        <v>464</v>
-      </c>
-      <c r="C88">
-        <v>1</v>
+        <v>460</v>
       </c>
       <c r="H88" t="str">
         <f t="shared" si="8"/>
-        <v>[87] = {["ID"] = 1879514047; ["TIER"] = 1; }; -- Invaders of Idagâl</v>
+        <v xml:space="preserve"> [87] = {["ID"] = 1879514041; }; -- Hunter of Mûr Ghala</v>
       </c>
       <c r="I88">
         <f t="shared" si="9"/>
@@ -9499,11 +9515,11 @@
       </c>
       <c r="J88" t="str">
         <f t="shared" si="10"/>
-        <v>[87] = {</v>
+        <v xml:space="preserve"> [87] = {</v>
       </c>
       <c r="K88" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514047; </v>
+        <v xml:space="preserve">["ID"] = 1879514041; </v>
       </c>
       <c r="L88" t="str">
         <f t="shared" si="12"/>
@@ -9511,7 +9527,7 @@
       </c>
       <c r="M88" t="str">
         <f t="shared" si="13"/>
-        <v xml:space="preserve">["TIER"] = 1; </v>
+        <v/>
       </c>
       <c r="N88" t="str">
         <f t="shared" si="14"/>
@@ -9520,14 +9536,17 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>1879514046</v>
+        <v>1879514045</v>
       </c>
       <c r="B89" t="s">
-        <v>473</v>
+        <v>461</v>
+      </c>
+      <c r="C89">
+        <v>1</v>
       </c>
       <c r="H89" t="str">
         <f t="shared" si="8"/>
-        <v>[88] = {["ID"] = 1879514046; }; -- Defender of Adagím</v>
+        <v xml:space="preserve"> [88] = {["ID"] = 1879514045; ["TIER"] = 1; }; -- Adversaries of Adagím</v>
       </c>
       <c r="I89">
         <f t="shared" si="9"/>
@@ -9535,11 +9554,11 @@
       </c>
       <c r="J89" t="str">
         <f t="shared" si="10"/>
-        <v>[88] = {</v>
+        <v xml:space="preserve"> [88] = {</v>
       </c>
       <c r="K89" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514046; </v>
+        <v xml:space="preserve">["ID"] = 1879514045; </v>
       </c>
       <c r="L89" t="str">
         <f t="shared" si="12"/>
@@ -9547,7 +9566,7 @@
       </c>
       <c r="M89" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N89" t="str">
         <f t="shared" si="14"/>
@@ -9556,14 +9575,17 @@
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>1879514040</v>
+        <v>1879514044</v>
       </c>
       <c r="B90" t="s">
-        <v>474</v>
+        <v>462</v>
+      </c>
+      <c r="C90">
+        <v>1</v>
       </c>
       <c r="H90" t="str">
         <f t="shared" si="8"/>
-        <v>[89] = {["ID"] = 1879514040; }; -- Defender of Kighân</v>
+        <v xml:space="preserve"> [89] = {["ID"] = 1879514044; ["TIER"] = 1; }; -- Combatants of Kighân</v>
       </c>
       <c r="I90">
         <f t="shared" si="9"/>
@@ -9571,11 +9593,11 @@
       </c>
       <c r="J90" t="str">
         <f t="shared" si="10"/>
-        <v>[89] = {</v>
+        <v xml:space="preserve"> [89] = {</v>
       </c>
       <c r="K90" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514040; </v>
+        <v xml:space="preserve">["ID"] = 1879514044; </v>
       </c>
       <c r="L90" t="str">
         <f t="shared" si="12"/>
@@ -9583,7 +9605,7 @@
       </c>
       <c r="M90" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N90" t="str">
         <f t="shared" si="14"/>
@@ -9592,14 +9614,17 @@
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>1879514042</v>
+        <v>1879514039</v>
       </c>
       <c r="B91" t="s">
-        <v>475</v>
+        <v>463</v>
+      </c>
+      <c r="C91">
+        <v>1</v>
       </c>
       <c r="H91" t="str">
         <f t="shared" si="8"/>
-        <v>[90] = {["ID"] = 1879514042; }; -- Defender of An Shêru</v>
+        <v xml:space="preserve"> [90] = {["ID"] = 1879514039; ["TIER"] = 1; }; -- Enemies of An Shêru</v>
       </c>
       <c r="I91">
         <f t="shared" si="9"/>
@@ -9607,11 +9632,11 @@
       </c>
       <c r="J91" t="str">
         <f t="shared" si="10"/>
-        <v>[90] = {</v>
+        <v xml:space="preserve"> [90] = {</v>
       </c>
       <c r="K91" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514042; </v>
+        <v xml:space="preserve">["ID"] = 1879514039; </v>
       </c>
       <c r="L91" t="str">
         <f t="shared" si="12"/>
@@ -9619,7 +9644,7 @@
       </c>
       <c r="M91" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N91" t="str">
         <f t="shared" si="14"/>
@@ -9628,14 +9653,17 @@
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>1879514043</v>
+        <v>1879514047</v>
       </c>
       <c r="B92" t="s">
-        <v>476</v>
+        <v>464</v>
+      </c>
+      <c r="C92">
+        <v>1</v>
       </c>
       <c r="H92" t="str">
         <f t="shared" si="8"/>
-        <v>[91] = {["ID"] = 1879514043; }; -- Defender of Idagâl</v>
+        <v xml:space="preserve"> [91] = {["ID"] = 1879514047; ["TIER"] = 1; }; -- Invaders of Idagâl</v>
       </c>
       <c r="I92">
         <f t="shared" si="9"/>
@@ -9643,11 +9671,11 @@
       </c>
       <c r="J92" t="str">
         <f t="shared" si="10"/>
-        <v>[91] = {</v>
+        <v xml:space="preserve"> [91] = {</v>
       </c>
       <c r="K92" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879514043; </v>
+        <v xml:space="preserve">["ID"] = 1879514047; </v>
       </c>
       <c r="L92" t="str">
         <f t="shared" si="12"/>
@@ -9655,7 +9683,7 @@
       </c>
       <c r="M92" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N92" t="str">
         <f t="shared" si="14"/>
@@ -9664,14 +9692,14 @@
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>1879513808</v>
+        <v>1879514046</v>
       </c>
       <c r="B93" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="H93" t="str">
         <f t="shared" si="8"/>
-        <v>[92] = {["ID"] = 1879513808; }; -- Explorer of Mûr Ghala</v>
+        <v xml:space="preserve"> [92] = {["ID"] = 1879514046; }; -- Defender of Adagím</v>
       </c>
       <c r="I93">
         <f t="shared" si="9"/>
@@ -9679,11 +9707,11 @@
       </c>
       <c r="J93" t="str">
         <f t="shared" si="10"/>
-        <v>[92] = {</v>
+        <v xml:space="preserve"> [92] = {</v>
       </c>
       <c r="K93" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513808; </v>
+        <v xml:space="preserve">["ID"] = 1879514046; </v>
       </c>
       <c r="L93" t="str">
         <f t="shared" si="12"/>
@@ -9700,14 +9728,14 @@
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>1879513705</v>
+        <v>1879514040</v>
       </c>
       <c r="B94" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="H94" t="str">
         <f t="shared" si="8"/>
-        <v>[93] = {["ID"] = 1879513705; }; -- Treasure-seeker of Mûr Ghala</v>
+        <v xml:space="preserve"> [93] = {["ID"] = 1879514040; }; -- Defender of Kighân</v>
       </c>
       <c r="I94">
         <f t="shared" si="9"/>
@@ -9715,11 +9743,11 @@
       </c>
       <c r="J94" t="str">
         <f t="shared" si="10"/>
-        <v>[93] = {</v>
+        <v xml:space="preserve"> [93] = {</v>
       </c>
       <c r="K94" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513705; </v>
+        <v xml:space="preserve">["ID"] = 1879514040; </v>
       </c>
       <c r="L94" t="str">
         <f t="shared" si="12"/>
@@ -9736,14 +9764,14 @@
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>1879513698</v>
+        <v>1879514042</v>
       </c>
       <c r="B95" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="H95" t="str">
         <f t="shared" si="8"/>
-        <v>[94] = {["ID"] = 1879513698; }; -- Slayer of Mûr Ghala</v>
+        <v xml:space="preserve"> [94] = {["ID"] = 1879514042; }; -- Defender of An Shêru</v>
       </c>
       <c r="I95">
         <f t="shared" si="9"/>
@@ -9751,11 +9779,11 @@
       </c>
       <c r="J95" t="str">
         <f t="shared" si="10"/>
-        <v>[94] = {</v>
+        <v xml:space="preserve"> [94] = {</v>
       </c>
       <c r="K95" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513698; </v>
+        <v xml:space="preserve">["ID"] = 1879514042; </v>
       </c>
       <c r="L95" t="str">
         <f t="shared" si="12"/>
@@ -9772,14 +9800,14 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>1879513807</v>
+        <v>1879514043</v>
       </c>
       <c r="B96" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="H96" t="str">
         <f t="shared" si="8"/>
-        <v>[95] = {["ID"] = 1879513807; }; -- Tales of Mûr Ghala</v>
+        <v xml:space="preserve"> [95] = {["ID"] = 1879514043; }; -- Defender of Idagâl</v>
       </c>
       <c r="I96">
         <f t="shared" si="9"/>
@@ -9787,11 +9815,11 @@
       </c>
       <c r="J96" t="str">
         <f t="shared" si="10"/>
-        <v>[95] = {</v>
+        <v xml:space="preserve"> [95] = {</v>
       </c>
       <c r="K96" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513807; </v>
+        <v xml:space="preserve">["ID"] = 1879514043; </v>
       </c>
       <c r="L96" t="str">
         <f t="shared" si="12"/>
@@ -9808,14 +9836,14 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>1879513694</v>
+        <v>1879513808</v>
       </c>
       <c r="B97" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="H97" t="str">
         <f t="shared" si="8"/>
-        <v>[96] = {["ID"] = 1879513694; }; -- Brigand-bane of Mûr Ghala</v>
+        <v xml:space="preserve"> [96] = {["ID"] = 1879513808; }; -- Explorer of Mûr Ghala</v>
       </c>
       <c r="I97">
         <f t="shared" si="9"/>
@@ -9823,11 +9851,11 @@
       </c>
       <c r="J97" t="str">
         <f t="shared" si="10"/>
-        <v>[96] = {</v>
+        <v xml:space="preserve"> [96] = {</v>
       </c>
       <c r="K97" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513694; </v>
+        <v xml:space="preserve">["ID"] = 1879513808; </v>
       </c>
       <c r="L97" t="str">
         <f t="shared" si="12"/>
@@ -9844,14 +9872,14 @@
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>1879513695</v>
+        <v>1879513705</v>
       </c>
       <c r="B98" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="H98" t="str">
         <f t="shared" si="8"/>
-        <v>[97] = {["ID"] = 1879513695; }; -- Nightmare of the Ordâkhai</v>
+        <v xml:space="preserve"> [97] = {["ID"] = 1879513705; }; -- Treasure-seeker of Mûr Ghala</v>
       </c>
       <c r="I98">
         <f t="shared" si="9"/>
@@ -9859,11 +9887,11 @@
       </c>
       <c r="J98" t="str">
         <f t="shared" si="10"/>
-        <v>[97] = {</v>
+        <v xml:space="preserve"> [97] = {</v>
       </c>
       <c r="K98" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513695; </v>
+        <v xml:space="preserve">["ID"] = 1879513705; </v>
       </c>
       <c r="L98" t="str">
         <f t="shared" si="12"/>
@@ -9880,14 +9908,14 @@
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>1879513696</v>
+        <v>1879513698</v>
       </c>
       <c r="B99" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="H99" t="str">
         <f t="shared" si="8"/>
-        <v>[98] = {["ID"] = 1879513696; }; -- Spider-slayer of Mûr Ghala</v>
+        <v xml:space="preserve"> [98] = {["ID"] = 1879513698; }; -- Slayer of Mûr Ghala</v>
       </c>
       <c r="I99">
         <f t="shared" si="9"/>
@@ -9895,11 +9923,11 @@
       </c>
       <c r="J99" t="str">
         <f t="shared" si="10"/>
-        <v>[98] = {</v>
+        <v xml:space="preserve"> [98] = {</v>
       </c>
       <c r="K99" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513696; </v>
+        <v xml:space="preserve">["ID"] = 1879513698; </v>
       </c>
       <c r="L99" t="str">
         <f t="shared" si="12"/>
@@ -9916,14 +9944,14 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>1879513703</v>
+        <v>1879513807</v>
       </c>
       <c r="B100" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="H100" t="str">
         <f t="shared" si="8"/>
-        <v>[99] = {["ID"] = 1879513703; }; -- Orc-slayer of Mûr Ghala</v>
+        <v xml:space="preserve"> [99] = {["ID"] = 1879513807; }; -- Tales of Mûr Ghala</v>
       </c>
       <c r="I100">
         <f t="shared" si="9"/>
@@ -9931,11 +9959,11 @@
       </c>
       <c r="J100" t="str">
         <f t="shared" si="10"/>
-        <v>[99] = {</v>
+        <v xml:space="preserve"> [99] = {</v>
       </c>
       <c r="K100" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve">["ID"] = 1879513703; </v>
+        <v xml:space="preserve">["ID"] = 1879513807; </v>
       </c>
       <c r="L100" t="str">
         <f t="shared" si="12"/>
@@ -9951,21 +9979,27 @@
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H101" t="e">
+      <c r="A101">
+        <v>1879513694</v>
+      </c>
+      <c r="B101" t="s">
+        <v>465</v>
+      </c>
+      <c r="H101" t="str">
         <f t="shared" si="8"/>
-        <v>#VALUE!</v>
+        <v>[100] = {["ID"] = 1879513694; }; -- Brigand-bane of Mûr Ghala</v>
       </c>
       <c r="I101">
         <f t="shared" si="9"/>
         <v>100</v>
       </c>
-      <c r="J101" t="e">
+      <c r="J101" t="str">
         <f t="shared" si="10"/>
-        <v>#VALUE!</v>
+        <v>[100] = {</v>
       </c>
       <c r="K101" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879513694; </v>
       </c>
       <c r="L101" t="str">
         <f t="shared" si="12"/>
@@ -9981,21 +10015,27 @@
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H102" t="e">
+      <c r="A102">
+        <v>1879513695</v>
+      </c>
+      <c r="B102" t="s">
+        <v>466</v>
+      </c>
+      <c r="H102" t="str">
         <f t="shared" si="8"/>
-        <v>#VALUE!</v>
+        <v>[101] = {["ID"] = 1879513695; }; -- Nightmare of the Ordâkhai</v>
       </c>
       <c r="I102">
         <f t="shared" si="9"/>
         <v>101</v>
       </c>
-      <c r="J102" t="e">
+      <c r="J102" t="str">
         <f t="shared" si="10"/>
-        <v>#VALUE!</v>
+        <v>[101] = {</v>
       </c>
       <c r="K102" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879513695; </v>
       </c>
       <c r="L102" t="str">
         <f t="shared" si="12"/>
@@ -10011,21 +10051,27 @@
       </c>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H103" t="e">
+      <c r="A103">
+        <v>1879513696</v>
+      </c>
+      <c r="B103" t="s">
+        <v>467</v>
+      </c>
+      <c r="H103" t="str">
         <f t="shared" si="8"/>
-        <v>#VALUE!</v>
+        <v>[102] = {["ID"] = 1879513696; }; -- Spider-slayer of Mûr Ghala</v>
       </c>
       <c r="I103">
         <f t="shared" si="9"/>
         <v>102</v>
       </c>
-      <c r="J103" t="e">
+      <c r="J103" t="str">
         <f t="shared" si="10"/>
-        <v>#VALUE!</v>
+        <v>[102] = {</v>
       </c>
       <c r="K103" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879513696; </v>
       </c>
       <c r="L103" t="str">
         <f t="shared" si="12"/>
@@ -10036,6 +10082,132 @@
         <v/>
       </c>
       <c r="N103" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>1879513703</v>
+      </c>
+      <c r="B104" t="s">
+        <v>469</v>
+      </c>
+      <c r="H104" t="str">
+        <f t="shared" si="8"/>
+        <v>[103] = {["ID"] = 1879513703; }; -- Orc-slayer of Mûr Ghala</v>
+      </c>
+      <c r="I104">
+        <f t="shared" si="9"/>
+        <v>103</v>
+      </c>
+      <c r="J104" t="str">
+        <f t="shared" si="10"/>
+        <v>[103] = {</v>
+      </c>
+      <c r="K104" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">["ID"] = 1879513703; </v>
+      </c>
+      <c r="L104" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M104" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N104" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H105" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">[104] = {}; -- </v>
+      </c>
+      <c r="I105">
+        <f t="shared" si="9"/>
+        <v>104</v>
+      </c>
+      <c r="J105" t="str">
+        <f t="shared" si="10"/>
+        <v>[104] = {</v>
+      </c>
+      <c r="K105" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L105" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M105" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N105" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H106" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">[105] = {}; -- </v>
+      </c>
+      <c r="I106">
+        <f t="shared" si="9"/>
+        <v>105</v>
+      </c>
+      <c r="J106" t="str">
+        <f t="shared" si="10"/>
+        <v>[105] = {</v>
+      </c>
+      <c r="K106" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L106" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M106" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N106" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H107" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">[106] = {}; -- </v>
+      </c>
+      <c r="I107">
+        <f t="shared" si="9"/>
+        <v>106</v>
+      </c>
+      <c r="J107" t="str">
+        <f t="shared" si="10"/>
+        <v>[106] = {</v>
+      </c>
+      <c r="K107" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="L107" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M107" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N107" t="str">
         <f t="shared" si="14"/>
         <v>};</v>
       </c>

</xml_diff>

<commit_message>
Added U48 deeds - Additional Hamât Renewed, Veil of the Nine - Baubles, and Mûr Ghala/Hatokáli Fells
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
+++ b/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9A3386-751D-4CCE-8841-432ABFA6536B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D79FD5-75AC-4C55-8702-4B8CA8ACC0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="210" yWindow="270" windowWidth="22875" windowHeight="14685" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="505">
   <si>
     <t>TIER</t>
   </si>
@@ -1489,6 +1489,78 @@
   </si>
   <si>
     <t>Persistent Defender of Idagâl</t>
+  </si>
+  <si>
+    <t>Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Rejuvenator of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Explorer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Dangers in Pahar Hatokáli</t>
+  </si>
+  <si>
+    <t>Scouting Pahar Hatokáli</t>
+  </si>
+  <si>
+    <t>Treasure-seeker of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Slayer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Brigand-bane of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Kergrim-bane of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Kergrim-bane of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Orc-slayer of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Orc-slayer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Ordâkhai-bane of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Scorpion-slayer of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Scorpion-slayer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Snake-slayer of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Snake-slayer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Zizanu-slayer of Hatokáli Fells (Advanced)</t>
+  </si>
+  <si>
+    <t>Zizanu-slayer of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Tales of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Defender of Hatokáli Fells</t>
+  </si>
+  <si>
+    <t>Hatokáli Scouting</t>
   </si>
 </sst>
 </file>
@@ -5942,7 +6014,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D727EC7-6195-47C5-8CEB-067AA7EF5F9D}">
-  <dimension ref="A1:N107"/>
+  <dimension ref="A1:N129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -8697,7 +8769,7 @@
         <v xml:space="preserve"> [66] = {["ID"] = 1879513783; ["TIER"] = 1; }; -- Renewer of Idagâl</v>
       </c>
       <c r="I67">
-        <f t="shared" ref="I67:I107" si="9">ROW()-1</f>
+        <f t="shared" ref="I67:I129" si="9">ROW()-1</f>
         <v>66</v>
       </c>
       <c r="J67" t="str">
@@ -8713,11 +8785,11 @@
         <v/>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M107" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
+        <f t="shared" ref="M67:M128" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
         <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N67" t="str">
-        <f t="shared" ref="N67:N107" si="14">CONCATENATE("};")</f>
+        <f t="shared" ref="N67:N129" si="14">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
@@ -10094,7 +10166,7 @@
         <v>469</v>
       </c>
       <c r="H104" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="H104:H129" si="15">CONCATENATE(J104,K104,L104,M104,N104," -- ",B104)</f>
         <v>[103] = {["ID"] = 1879513703; }; -- Orc-slayer of Mûr Ghala</v>
       </c>
       <c r="I104">
@@ -10102,19 +10174,19 @@
         <v>103</v>
       </c>
       <c r="J104" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="J104:J129" si="16">CONCATENATE(REPT(" ",3-LEN(I104)),"[",I104,"] = {")</f>
         <v>[103] = {</v>
       </c>
       <c r="K104" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="K104:K129" si="17">IF(LEN(A104)&gt;0,CONCATENATE("[""ID""] = ",A104,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879513703; </v>
       </c>
       <c r="L104" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="L104:L129" si="18">IF(LEN(D104)&gt;0,CONCATENATE("[""CAT_ID""] = ",D104,"; "),"")</f>
         <v/>
       </c>
       <c r="M104" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="M104:M129" si="19">IF(C104&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C104,"0"),"; "),"")</f>
         <v/>
       </c>
       <c r="N104" t="str">
@@ -10123,28 +10195,37 @@
       </c>
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>481</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+      <c r="D105">
+        <v>343</v>
+      </c>
       <c r="H105" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">[104] = {}; -- </v>
+        <f t="shared" si="15"/>
+        <v>[104] = {["CAT_ID"] = 343; }; -- Hatokáli Fells</v>
       </c>
       <c r="I105">
         <f t="shared" si="9"/>
         <v>104</v>
       </c>
       <c r="J105" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>[104] = {</v>
       </c>
       <c r="K105" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="L105" t="str">
-        <f t="shared" si="12"/>
-        <v/>
+        <f t="shared" si="18"/>
+        <v xml:space="preserve">["CAT_ID"] = 343; </v>
       </c>
       <c r="M105" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="N105" t="str">
@@ -10153,28 +10234,37 @@
       </c>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>1879524266</v>
+      </c>
+      <c r="B106" t="s">
+        <v>482</v>
+      </c>
+      <c r="C106">
+        <v>0</v>
+      </c>
       <c r="H106" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">[105] = {}; -- </v>
+        <f t="shared" si="15"/>
+        <v>[105] = {["ID"] = 1879524266; }; -- Rejuvenator of Hatokáli Fells</v>
       </c>
       <c r="I106">
         <f t="shared" si="9"/>
         <v>105</v>
       </c>
       <c r="J106" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>[105] = {</v>
       </c>
       <c r="K106" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524266; </v>
       </c>
       <c r="L106" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="M106" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="N106" t="str">
@@ -10183,31 +10273,889 @@
       </c>
     </row>
     <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>1879524262</v>
+      </c>
+      <c r="B107" t="s">
+        <v>483</v>
+      </c>
+      <c r="C107">
+        <v>1</v>
+      </c>
       <c r="H107" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">[106] = {}; -- </v>
+        <f t="shared" si="15"/>
+        <v>[106] = {["ID"] = 1879524262; ["TIER"] = 1; }; -- Explorer of Hatokáli Fells</v>
       </c>
       <c r="I107">
         <f t="shared" si="9"/>
         <v>106</v>
       </c>
       <c r="J107" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>[106] = {</v>
       </c>
       <c r="K107" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524262; </v>
       </c>
       <c r="L107" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="M107" t="str">
-        <f t="shared" si="13"/>
-        <v/>
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N107" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>1879524270</v>
+      </c>
+      <c r="B108" t="s">
+        <v>484</v>
+      </c>
+      <c r="C108">
+        <v>2</v>
+      </c>
+      <c r="H108" t="str">
+        <f t="shared" si="15"/>
+        <v>[107] = {["ID"] = 1879524270; ["TIER"] = 2; }; -- Dangers in Pahar Hatokáli</v>
+      </c>
+      <c r="I108">
+        <f t="shared" si="9"/>
+        <v>107</v>
+      </c>
+      <c r="J108" t="str">
+        <f t="shared" si="16"/>
+        <v>[107] = {</v>
+      </c>
+      <c r="K108" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524270; </v>
+      </c>
+      <c r="L108" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M108" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N108" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>1879524271</v>
+      </c>
+      <c r="B109" t="s">
+        <v>485</v>
+      </c>
+      <c r="C109">
+        <v>2</v>
+      </c>
+      <c r="H109" t="str">
+        <f t="shared" si="15"/>
+        <v>[108] = {["ID"] = 1879524271; ["TIER"] = 2; }; -- Scouting Pahar Hatokáli</v>
+      </c>
+      <c r="I109">
+        <f t="shared" si="9"/>
+        <v>108</v>
+      </c>
+      <c r="J109" t="str">
+        <f t="shared" si="16"/>
+        <v>[108] = {</v>
+      </c>
+      <c r="K109" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524271; </v>
+      </c>
+      <c r="L109" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M109" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N109" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>1879524264</v>
+      </c>
+      <c r="B110" t="s">
+        <v>486</v>
+      </c>
+      <c r="C110">
+        <v>2</v>
+      </c>
+      <c r="H110" t="str">
+        <f t="shared" si="15"/>
+        <v>[109] = {["ID"] = 1879524264; ["TIER"] = 2; }; -- Treasure-seeker of Hatokáli Fells</v>
+      </c>
+      <c r="I110">
+        <f t="shared" si="9"/>
+        <v>109</v>
+      </c>
+      <c r="J110" t="str">
+        <f t="shared" si="16"/>
+        <v>[109] = {</v>
+      </c>
+      <c r="K110" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524264; </v>
+      </c>
+      <c r="L110" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M110" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N110" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>1879524261</v>
+      </c>
+      <c r="B111" t="s">
+        <v>487</v>
+      </c>
+      <c r="C111">
+        <v>1</v>
+      </c>
+      <c r="H111" t="str">
+        <f t="shared" si="15"/>
+        <v>[110] = {["ID"] = 1879524261; ["TIER"] = 1; }; -- Slayer of Hatokáli Fells</v>
+      </c>
+      <c r="I111">
+        <f t="shared" si="9"/>
+        <v>110</v>
+      </c>
+      <c r="J111" t="str">
+        <f t="shared" si="16"/>
+        <v>[110] = {</v>
+      </c>
+      <c r="K111" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524261; </v>
+      </c>
+      <c r="L111" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M111" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N111" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>1879524249</v>
+      </c>
+      <c r="B112" t="s">
+        <v>488</v>
+      </c>
+      <c r="C112">
+        <v>2</v>
+      </c>
+      <c r="H112" t="str">
+        <f t="shared" si="15"/>
+        <v>[111] = {["ID"] = 1879524249; ["TIER"] = 2; }; -- Brigand-bane of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I112">
+        <f t="shared" si="9"/>
+        <v>111</v>
+      </c>
+      <c r="J112" t="str">
+        <f t="shared" si="16"/>
+        <v>[111] = {</v>
+      </c>
+      <c r="K112" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524249; </v>
+      </c>
+      <c r="L112" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M112" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N112" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>1879524240</v>
+      </c>
+      <c r="B113" t="s">
+        <v>489</v>
+      </c>
+      <c r="C113">
+        <v>3</v>
+      </c>
+      <c r="H113" t="str">
+        <f t="shared" si="15"/>
+        <v>[112] = {["ID"] = 1879524240; ["TIER"] = 3; }; -- Brigand-bane of Hatokáli Fells</v>
+      </c>
+      <c r="I113">
+        <f t="shared" si="9"/>
+        <v>112</v>
+      </c>
+      <c r="J113" t="str">
+        <f t="shared" si="16"/>
+        <v>[112] = {</v>
+      </c>
+      <c r="K113" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524240; </v>
+      </c>
+      <c r="L113" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M113" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N113" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>1879524265</v>
+      </c>
+      <c r="B114" t="s">
+        <v>490</v>
+      </c>
+      <c r="C114">
+        <v>2</v>
+      </c>
+      <c r="H114" t="str">
+        <f t="shared" si="15"/>
+        <v>[113] = {["ID"] = 1879524265; ["TIER"] = 2; }; -- Kergrim-bane of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I114">
+        <f t="shared" si="9"/>
+        <v>113</v>
+      </c>
+      <c r="J114" t="str">
+        <f t="shared" si="16"/>
+        <v>[113] = {</v>
+      </c>
+      <c r="K114" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524265; </v>
+      </c>
+      <c r="L114" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M114" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N114" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>1879524257</v>
+      </c>
+      <c r="B115" t="s">
+        <v>491</v>
+      </c>
+      <c r="C115">
+        <v>3</v>
+      </c>
+      <c r="H115" t="str">
+        <f t="shared" si="15"/>
+        <v>[114] = {["ID"] = 1879524257; ["TIER"] = 3; }; -- Kergrim-bane of Hatokáli Fells</v>
+      </c>
+      <c r="I115">
+        <f t="shared" si="9"/>
+        <v>114</v>
+      </c>
+      <c r="J115" t="str">
+        <f t="shared" si="16"/>
+        <v>[114] = {</v>
+      </c>
+      <c r="K115" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524257; </v>
+      </c>
+      <c r="L115" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M115" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N115" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>1879524256</v>
+      </c>
+      <c r="B116" t="s">
+        <v>492</v>
+      </c>
+      <c r="C116">
+        <v>2</v>
+      </c>
+      <c r="H116" t="str">
+        <f t="shared" si="15"/>
+        <v>[115] = {["ID"] = 1879524256; ["TIER"] = 2; }; -- Orc-slayer of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I116">
+        <f t="shared" si="9"/>
+        <v>115</v>
+      </c>
+      <c r="J116" t="str">
+        <f t="shared" si="16"/>
+        <v>[115] = {</v>
+      </c>
+      <c r="K116" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524256; </v>
+      </c>
+      <c r="L116" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M116" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N116" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>1879524260</v>
+      </c>
+      <c r="B117" t="s">
+        <v>493</v>
+      </c>
+      <c r="C117">
+        <v>3</v>
+      </c>
+      <c r="H117" t="str">
+        <f t="shared" si="15"/>
+        <v>[116] = {["ID"] = 1879524260; ["TIER"] = 3; }; -- Orc-slayer of Hatokáli Fells</v>
+      </c>
+      <c r="I117">
+        <f t="shared" si="9"/>
+        <v>116</v>
+      </c>
+      <c r="J117" t="str">
+        <f t="shared" si="16"/>
+        <v>[116] = {</v>
+      </c>
+      <c r="K117" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524260; </v>
+      </c>
+      <c r="L117" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M117" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N117" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>1879524255</v>
+      </c>
+      <c r="B118" t="s">
+        <v>494</v>
+      </c>
+      <c r="C118">
+        <v>2</v>
+      </c>
+      <c r="H118" t="str">
+        <f t="shared" si="15"/>
+        <v>[117] = {["ID"] = 1879524255; ["TIER"] = 2; }; -- Ordâkhai-bane of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I118">
+        <f t="shared" si="9"/>
+        <v>117</v>
+      </c>
+      <c r="J118" t="str">
+        <f t="shared" si="16"/>
+        <v>[117] = {</v>
+      </c>
+      <c r="K118" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524255; </v>
+      </c>
+      <c r="L118" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M118" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N118" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>1879524252</v>
+      </c>
+      <c r="B119" t="s">
+        <v>495</v>
+      </c>
+      <c r="C119">
+        <v>3</v>
+      </c>
+      <c r="H119" t="str">
+        <f t="shared" si="15"/>
+        <v>[118] = {["ID"] = 1879524252; ["TIER"] = 3; }; -- Ordâkhai-bane of Hatokáli Fells</v>
+      </c>
+      <c r="I119">
+        <f t="shared" si="9"/>
+        <v>118</v>
+      </c>
+      <c r="J119" t="str">
+        <f t="shared" si="16"/>
+        <v>[118] = {</v>
+      </c>
+      <c r="K119" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524252; </v>
+      </c>
+      <c r="L119" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M119" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N119" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>1879524254</v>
+      </c>
+      <c r="B120" t="s">
+        <v>496</v>
+      </c>
+      <c r="C120">
+        <v>2</v>
+      </c>
+      <c r="H120" t="str">
+        <f t="shared" si="15"/>
+        <v>[119] = {["ID"] = 1879524254; ["TIER"] = 2; }; -- Scorpion-slayer of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I120">
+        <f t="shared" si="9"/>
+        <v>119</v>
+      </c>
+      <c r="J120" t="str">
+        <f t="shared" si="16"/>
+        <v>[119] = {</v>
+      </c>
+      <c r="K120" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524254; </v>
+      </c>
+      <c r="L120" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M120" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N120" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>1879524258</v>
+      </c>
+      <c r="B121" t="s">
+        <v>497</v>
+      </c>
+      <c r="C121">
+        <v>3</v>
+      </c>
+      <c r="H121" t="str">
+        <f t="shared" si="15"/>
+        <v>[120] = {["ID"] = 1879524258; ["TIER"] = 3; }; -- Scorpion-slayer of Hatokáli Fells</v>
+      </c>
+      <c r="I121">
+        <f t="shared" si="9"/>
+        <v>120</v>
+      </c>
+      <c r="J121" t="str">
+        <f t="shared" si="16"/>
+        <v>[120] = {</v>
+      </c>
+      <c r="K121" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524258; </v>
+      </c>
+      <c r="L121" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M121" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N121" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>1879524263</v>
+      </c>
+      <c r="B122" t="s">
+        <v>498</v>
+      </c>
+      <c r="C122">
+        <v>2</v>
+      </c>
+      <c r="H122" t="str">
+        <f t="shared" si="15"/>
+        <v>[121] = {["ID"] = 1879524263; ["TIER"] = 2; }; -- Snake-slayer of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I122">
+        <f t="shared" si="9"/>
+        <v>121</v>
+      </c>
+      <c r="J122" t="str">
+        <f t="shared" si="16"/>
+        <v>[121] = {</v>
+      </c>
+      <c r="K122" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524263; </v>
+      </c>
+      <c r="L122" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M122" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N122" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>1879524269</v>
+      </c>
+      <c r="B123" t="s">
+        <v>499</v>
+      </c>
+      <c r="C123">
+        <v>3</v>
+      </c>
+      <c r="H123" t="str">
+        <f t="shared" si="15"/>
+        <v>[122] = {["ID"] = 1879524269; ["TIER"] = 3; }; -- Snake-slayer of Hatokáli Fells</v>
+      </c>
+      <c r="I123">
+        <f t="shared" si="9"/>
+        <v>122</v>
+      </c>
+      <c r="J123" t="str">
+        <f t="shared" si="16"/>
+        <v>[122] = {</v>
+      </c>
+      <c r="K123" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524269; </v>
+      </c>
+      <c r="L123" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M123" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N123" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>1879524268</v>
+      </c>
+      <c r="B124" t="s">
+        <v>500</v>
+      </c>
+      <c r="C124">
+        <v>2</v>
+      </c>
+      <c r="H124" t="str">
+        <f t="shared" si="15"/>
+        <v>[123] = {["ID"] = 1879524268; ["TIER"] = 2; }; -- Zizanu-slayer of Hatokáli Fells (Advanced)</v>
+      </c>
+      <c r="I124">
+        <f t="shared" si="9"/>
+        <v>123</v>
+      </c>
+      <c r="J124" t="str">
+        <f t="shared" si="16"/>
+        <v>[123] = {</v>
+      </c>
+      <c r="K124" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524268; </v>
+      </c>
+      <c r="L124" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M124" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 2; </v>
+      </c>
+      <c r="N124" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>1879524253</v>
+      </c>
+      <c r="B125" t="s">
+        <v>501</v>
+      </c>
+      <c r="C125">
+        <v>3</v>
+      </c>
+      <c r="H125" t="str">
+        <f t="shared" si="15"/>
+        <v>[124] = {["ID"] = 1879524253; ["TIER"] = 3; }; -- Zizanu-slayer of Hatokáli Fells</v>
+      </c>
+      <c r="I125">
+        <f t="shared" si="9"/>
+        <v>124</v>
+      </c>
+      <c r="J125" t="str">
+        <f t="shared" si="16"/>
+        <v>[124] = {</v>
+      </c>
+      <c r="K125" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524253; </v>
+      </c>
+      <c r="L125" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M125" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 3; </v>
+      </c>
+      <c r="N125" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>1879524267</v>
+      </c>
+      <c r="B126" t="s">
+        <v>502</v>
+      </c>
+      <c r="C126">
+        <v>1</v>
+      </c>
+      <c r="H126" t="str">
+        <f t="shared" si="15"/>
+        <v>[125] = {["ID"] = 1879524267; ["TIER"] = 1; }; -- Tales of Hatokáli Fells</v>
+      </c>
+      <c r="I126">
+        <f t="shared" si="9"/>
+        <v>125</v>
+      </c>
+      <c r="J126" t="str">
+        <f t="shared" si="16"/>
+        <v>[125] = {</v>
+      </c>
+      <c r="K126" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524267; </v>
+      </c>
+      <c r="L126" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M126" t="str">
+        <f t="shared" si="19"/>
+        <v xml:space="preserve">["TIER"] = 1; </v>
+      </c>
+      <c r="N126" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>1879524259</v>
+      </c>
+      <c r="B127" t="s">
+        <v>503</v>
+      </c>
+      <c r="C127">
+        <v>0</v>
+      </c>
+      <c r="H127" t="str">
+        <f t="shared" si="15"/>
+        <v>[126] = {["ID"] = 1879524259; }; -- Defender of Hatokáli Fells</v>
+      </c>
+      <c r="I127">
+        <f t="shared" si="9"/>
+        <v>126</v>
+      </c>
+      <c r="J127" t="str">
+        <f t="shared" si="16"/>
+        <v>[126] = {</v>
+      </c>
+      <c r="K127" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879524259; </v>
+      </c>
+      <c r="L127" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M127" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="N127" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>1879525229</v>
+      </c>
+      <c r="B128" t="s">
+        <v>504</v>
+      </c>
+      <c r="C128">
+        <v>0</v>
+      </c>
+      <c r="H128" t="str">
+        <f t="shared" si="15"/>
+        <v>[127] = {["ID"] = 1879525229; }; -- Hatokáli Scouting</v>
+      </c>
+      <c r="I128">
+        <f t="shared" si="9"/>
+        <v>127</v>
+      </c>
+      <c r="J128" t="str">
+        <f t="shared" si="16"/>
+        <v>[127] = {</v>
+      </c>
+      <c r="K128" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">["ID"] = 1879525229; </v>
+      </c>
+      <c r="L128" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M128" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="N128" t="str">
+        <f t="shared" si="14"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="129" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H129" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve">[128] = {}; -- </v>
+      </c>
+      <c r="I129">
+        <f t="shared" si="9"/>
+        <v>128</v>
+      </c>
+      <c r="J129" t="str">
+        <f t="shared" si="16"/>
+        <v>[128] = {</v>
+      </c>
+      <c r="K129" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="L129" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="M129" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="N129" t="str">
         <f t="shared" si="14"/>
         <v>};</v>
       </c>

</xml_diff>

<commit_message>
Re-added Tales for the Storyteller
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
+++ b/_SourceFiles/DeedInfo-10-Haradwaith.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D79FD5-75AC-4C55-8702-4B8CA8ACC0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C6B633-F687-4C48-84B7-3CE37133B0D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="210" yWindow="270" windowWidth="22875" windowHeight="14685" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="869" firstSheet="9" activeTab="12" xr2:uid="{CDC9C16A-58F0-4807-B5CD-F77FF9D2EA43}"/>
   </bookViews>
   <sheets>
     <sheet name="Type" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="506">
   <si>
     <t>TIER</t>
   </si>
@@ -1561,6 +1561,9 @@
   </si>
   <si>
     <t>Hatokáli Scouting</t>
+  </si>
+  <si>
+    <t>Tales for the Storyteller</t>
   </si>
 </sst>
 </file>
@@ -8765,7 +8768,7 @@
         <v>1</v>
       </c>
       <c r="H67" t="str">
-        <f t="shared" ref="H67:H107" si="8">CONCATENATE(J67,K67,L67,M67,N67," -- ",B67)</f>
+        <f t="shared" ref="H67:H103" si="8">CONCATENATE(J67,K67,L67,M67,N67," -- ",B67)</f>
         <v xml:space="preserve"> [66] = {["ID"] = 1879513783; ["TIER"] = 1; }; -- Renewer of Idagâl</v>
       </c>
       <c r="I67">
@@ -8773,19 +8776,19 @@
         <v>66</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" ref="J67:J107" si="10">CONCATENATE(REPT(" ",3-LEN(I67)),"[",I67,"] = {")</f>
+        <f t="shared" ref="J67:J103" si="10">CONCATENATE(REPT(" ",3-LEN(I67)),"[",I67,"] = {")</f>
         <v xml:space="preserve"> [66] = {</v>
       </c>
       <c r="K67" t="str">
-        <f t="shared" ref="K67:K107" si="11">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
+        <f t="shared" ref="K67:K103" si="11">IF(LEN(A67)&gt;0,CONCATENATE("[""ID""] = ",A67,"; "),"")</f>
         <v xml:space="preserve">["ID"] = 1879513783; </v>
       </c>
       <c r="L67" t="str">
-        <f t="shared" ref="L67:L107" si="12">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
+        <f t="shared" ref="L67:L103" si="12">IF(LEN(D67)&gt;0,CONCATENATE("[""CAT_ID""] = ",D67,"; "),"")</f>
         <v/>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M128" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
+        <f t="shared" ref="M67:M103" si="13">IF(C67&gt;0,CONCATENATE("[""TIER""] = ",TEXT(C67,"0"),"; "),"")</f>
         <v xml:space="preserve">["TIER"] = 1; </v>
       </c>
       <c r="N67" t="str">
@@ -11130,10 +11133,19 @@
         <v>};</v>
       </c>
     </row>
-    <row r="129" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>1879523703</v>
+      </c>
+      <c r="B129" t="s">
+        <v>505</v>
+      </c>
+      <c r="C129">
+        <v>0</v>
+      </c>
       <c r="H129" t="str">
         <f t="shared" si="15"/>
-        <v xml:space="preserve">[128] = {}; -- </v>
+        <v>[128] = {["ID"] = 1879523703; }; -- Tales for the Storyteller</v>
       </c>
       <c r="I129">
         <f t="shared" si="9"/>
@@ -11145,7 +11157,7 @@
       </c>
       <c r="K129" t="str">
         <f t="shared" si="17"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879523703; </v>
       </c>
       <c r="L129" t="str">
         <f t="shared" si="18"/>

</xml_diff>